<commit_message>
Fix Login email default (Bugs.xlsx row 3), re-prioritised P2 -> P1
Sibling of the row-2 Login fix, on the same screen. Per team request,
bumped from P2 to P1 and fixed properly:
- Login email field now starts empty with a "you@company.com" placeholder
  instead of the sample sarah@acme.com default.

Sheet updated (row 3 priority P1 + Root Cause/Fix/Status, images preserved)
and the P1 review report amended.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -705,7 +705,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>The login page's email box was pre-filled with a sample address, sarah@acme.com, so a returning user had to clear it before typing their own email.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Made the email box start empty with an example hint ('you@company.com'), matching the signup form. Re-prioritised from P2 to P1 on team request so it ships with the sibling Login fix (row for 'Welcome back to Acme Corp.'). (Login.tsx line 19 and the email input.)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated the bug sheet with new P1 and other issues to fix
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Msi\projects\SDLC-App\AI-First-SDLC-App\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC72D5E-88D7-4CFC-94FB-0695301C0DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F27ECA-6C01-47A3-B7E3-88ECE724B660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="98">
   <si>
     <t>S.No</t>
   </si>
@@ -298,6 +298,92 @@
   </si>
   <si>
     <t>Clarifications</t>
+  </si>
+  <si>
+    <t>The shared Drawer and Modal building blocks were originally written as flat 'gallery' swatches for the design catalogue - their styling sat inside the page instead of floating above it, which is why opening the Create work item / Invite / Integrations form showed a grey block wedged into the page with the form squashed to the right, and the X and clicking outside did nothing.</t>
+  </si>
+  <si>
+    <t>Rebuilt Drawer and Modal as real overlays: a proper dimmed backdrop over the whole page with the form panel above it, and the X, a click on the dimmed area, and the Esc key all close it. Fixed once at the shared-component level so all three screens (Create work item, Invite user, Integrations connect forms) are corrected together. The Integrations connect screen, which is a full page rather than a pop-over, now shows a clean centred card instead of the grey right-floated block. frontend/src/components/ui/index.tsx (Drawer, Modal) + styles/components.css (.scrim-overlay). All 190 frontend tests pass.</t>
+  </si>
+  <si>
+    <t>The Create work item form marked Title as optional; the reporter wants it required. Separately, the Type field had no explanation of what Epic/Story/Task/Defect mean.</t>
+  </si>
+  <si>
+    <t>Title is now required: the field is marked with * and the Create button stays disabled until a title is entered. Added a tooltip/hint on the Type field explaining each type (Epic/Story = plan tier, Task = build tier, Defect = remediation) - this also closes the type-tooltip enhancement noted under the Work Item lifecycle row. frontend/src/features/lifecycle/WorkItemsBoard.tsx.</t>
+  </si>
+  <si>
+    <t>The invite form hard-coded only four roles and showed them as raw keys like 'product_owner' (with the underscore), and once you added a role row with 'grant another role' there was no way to remove it.</t>
+  </si>
+  <si>
+    <t>The role dropdown now lists the full set of ten roles from one shared source, every role shows a human-readable label (Product Owner, Security Engineer, ...) with no underscores, and each granted-role row has an X to remove it (shown whenever there's more than one). The same labels are used wherever a user's roles are listed. New shared list frontend/src/features/identity/roles.ts; UsersInvites.tsx; tests in roles.test.ts.</t>
+  </si>
+  <si>
+    <t>Several issues on the work-item lifecycle screen. (i) The rail listed brownfield/onboarding phases (context bridge, context extraction, on-boarding) that don't belong on a normal work item, and phase names showed with underscores/number prefixes. (ii) A Story (or any non-Epic) still showed 'Epic' because the screen hard-coded that word. (iv) The run console showed nothing because run events are stored with an 'action' + 'payload' but the console reads 'kind' and 'message', which weren't being sent - so every line rendered blank. (v) Re-running a failed phase sent the run's internal id (a UUID) where the system expects the short phase key, producing 'no AgentSpec registered for key &lt;uuid&gt;', and a failed run gave no reason.</t>
+  </si>
+  <si>
+    <t>(i) Phase names are now human-readable everywhere (Task Breakdown, Architecture, ...) and the brownfield/onboarding phases are hidden from a work item's rail - a display-only filter, no change to orchestration (as agreed with the team). (ii) The type badge and headings now show the work item's real type. (iv) Run events now carry a colour ('kind') and a readable 'message' from the action + payload, so the console shows progress - verified live on a real run, e.g. 'Phase dispatched - ideation' and 'Run failed - Command failed with exit code 1'. (v) Re-run now sends the phase key, not the UUID; verified live with the exact id from the report (d32f5ced-...): the UUID reproduces the error, the key '01_ideation' starts a run cleanly. A failed run now shows the actual reason. (iii, type tooltip, was an enhancement and is also done - see the 'Title is mandatory' row.) Files: frontend lifecycle/phases.ts, WorkItemEpic/Task/Defect.tsx, PhasesAndRuns.tsx, RunConsole.tsx, observability/OfflineTakeover.tsx, RunTranscriptScreen.tsx; backend api/serializers.py (RunSerializer agent_key/agent_phase, EventSerializer kind/message).</t>
+  </si>
+  <si>
+    <t>Artifacts generated by a phase are registered as internal drafts with the draft text stored inline in the artifact's external_ref.body field and an empty s3_key (the agent hadn't staged a snapshot to object storage). The Preview endpoint only knew how to fetch a body from s3_key, so for these drafts it found nothing and returned 'artifact has no body to preview' even though the text was sitting right there in external_ref.body.</t>
+  </si>
+  <si>
+    <t>Taught the preview read-through to also read an internal draft's body from external_ref.body when there is no s3_key yet, choosing the content type from the draft's 'format'. Nothing is copied or stored anywhere new - it's read where it already lives, so tenant isolation and 'platform owns state, not content' are untouched. Verified LIVE on the exact artifact from the report (08efb4c5-...-a232e): it previously 404'd and now returns its 5,834-character markdown body. On MinIO: the local object store container is up and healthy, and artifacts that DO have an s3_key still preview from S3 as before - both paths work. backend/integrations/preview.py (_read_internal); regression test test_preview_internal_artifact_reads_inline_external_ref_body.</t>
+  </si>
+  <si>
+    <t>When a clarification question offered an 'Other (please specify)' choice, picking it gave the user nowhere to type the specifics, and the literal option text would have been sent as the answer.</t>
+  </si>
+  <si>
+    <t>Selecting an 'Other / please specify' style option now reveals a text box, and what the user types is submitted as the answer (an empty box counts as unanswered so a required question still blocks). frontend/src/features/lifecycle/Clarifications.tsx.</t>
+  </si>
+  <si>
+    <t>When registering generated artifacts the agent raised a clarification asking the user for the project id, which the user can't know. The registration tool required project_id (and run_id) as inputs, so if the agent didn't have them it asked.</t>
+  </si>
+  <si>
+    <t>The platform now binds the project id and run id from the run the phase is executing under (the same way the tenant is already bound), so artifact registration fills them in automatically and never asks the user. Done on both the live companion path and the server-side path. runner/companion/state_mcp.py + runner.py (RUNNER_PROJECT_ID), mcp_platform_state/server.py + backend/orchestration/activities.py (PLATFORM_PROJECT_ID/RUN_ID).</t>
+  </si>
+  <si>
+    <t>Work Items
+1. In work items board all the trigger phases are not present in a perfect SDLC order - only 4 trigger phases are shown - Need to fix it
+2. In work item cards, when a phase is in waiting for gate approval, phase clarification - the card design is disturbed and not looking good appealing the user. Any unse of underscore names should also be humanised and readable.</t>
+  </si>
+  <si>
+    <t>Work item</t>
+  </si>
+  <si>
+    <t>Workspace Dashboard
+1. In the "Needs me" section all the info regarding - pending gates, clarifications and running work items etc should be human readable (currently underscores are been used) - need to fix. 
+Reference: Refer to the designs screen S31 in docs/designs
+2. Some values are hardcoded in the work space dashboard Navigation bar and side bar - namely: Notification icon showing 4 by default, clarifications showing 3 by default and gates showing one by default. Need to fix them.</t>
+  </si>
+  <si>
+    <t>Work Space Dashboard</t>
+  </si>
+  <si>
+    <t>Universal SDLC Application Flow Fixes needed - V1:
+1. In the SDLC app user flow: Wherever there is a usage of underscores for the names representation, thise should be human readable.
+2. In the application flow wherever you find a hardcoded value that should have been dynamic - you have to make them dynamic.</t>
+  </si>
+  <si>
+    <t>Universal</t>
+  </si>
+  <si>
+    <t>Work Space Admin</t>
+  </si>
+  <si>
+    <t>Workspace Admin Page
+1. Currently the users who are registered and invited are not been shown, but when clicked on the invite button it is showing in the background. Need to propely fix this
+2. The hardcoded "Acme Corp workspace" is shown but it should be dynamic as per registered work space.</t>
+  </si>
+  <si>
+    <t>After initial sign in, the get started page is shown for the user to set up his complete the 4 step process: During that process if the user clicks on "connect machine", "invite users" and "integrations" it takes the respective page and the user will see a button or link as "Back to get started" as option, once user does the 4 step process and then goes to any one of the above screens, it shows the same "back to get started" option even though the user has completed the on-borading process.</t>
+  </si>
+  <si>
+    <t>General issue</t>
+  </si>
+  <si>
+    <t>Artifacts &amp; Traceability
+1. The generated phase artifacts are Markdown files and the application is showing the preview as markdown text not a rendered markdwon file. In some cases when a architecure diagram present then it wont be human understandable Need to fix the rendering
+2. When artifacts are generated for a work item, if the same work item phase is run again: The artifacts are duplicated with same v1 as version instead of v2 and when clicked on preview it showing versions a v1 for both not v1 and v2 etc.</t>
   </si>
 </sst>
 </file>
@@ -674,6 +760,306 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3673039</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>1796213</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B2D494A-C781-F33D-1FB1-5E4C871A6036}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7470588" y="44138725"/>
+          <a:ext cx="3673039" cy="1796213"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>4026</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>1739347</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B6CCA93-20F1-AEC4-0D2F-70053E9D32B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7468153" y="47252283"/>
+          <a:ext cx="3689786" cy="1739347"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3672703</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>1762444</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4F375C2-42D0-71E6-F0E4-A815E3E01DE3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7482704" y="49581486"/>
+          <a:ext cx="3672702" cy="1762444"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3228411</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>1531714</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02467A17-CCE0-9D56-7860-DFFEF836ADFA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7483506" y="56253879"/>
+          <a:ext cx="3228410" cy="1531783"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1120588</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>1743138</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3623235</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>3505976</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{586E977A-EC3E-F17A-8EDB-DCE42404AFEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7445686" y="58021569"/>
+          <a:ext cx="3648137" cy="1762838"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1127125</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>1857375</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3654393</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>3635375</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B15BF7FE-AFEA-0C56-4784-5716E21958AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7461250" y="49101375"/>
+          <a:ext cx="3670268" cy="1778000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1413,20 +1799,14 @@
       <c r="G17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The shared Drawer and Modal building blocks were originally written as flat 'gallery' swatches for the design catalogue - their styling sat inside the page instead of floating above it, which is why opening the Create work item / Invite / Integrations form showed a grey block wedged into the page with the form squashed to the right, and the X and clicking outside did nothing.</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rebuilt Drawer and Modal as real overlays: a proper dimmed backdrop over the whole page with the form panel above it, and the X, a click on the dimmed area, and the Esc key all close it. Fixed once at the shared-component level so all three screens (Create work item, Invite user, Integrations connect forms) are corrected together. The Integrations connect screen, which is a full page rather than a pop-over, now shows a clean centred card instead of the grey right-floated block. frontend/src/components/ui/index.tsx (Drawer, Modal) + styles/components.css (.scrim-overlay). All 190 frontend tests pass.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
@@ -1446,20 +1826,14 @@
       <c r="G18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Create work item form marked Title as optional; the reporter wants it required. Separately, the Type field had no explanation of what Epic/Story/Task/Defect mean.</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Title is now required: the field is marked with * and the Create button stays disabled until a title is entered. Added a tooltip/hint on the Type field explaining each type (Epic/Story = plan tier, Task = build tier, Defect = remediation) - this also closes the type-tooltip enhancement noted under the Work Item lifecycle row. frontend/src/features/lifecycle/WorkItemsBoard.tsx.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="188.5" x14ac:dyDescent="0.35">
@@ -1519,20 +1893,14 @@
       <c r="G21" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The invite form hard-coded only four roles and showed them as raw keys like 'product_owner' (with the underscore), and once you added a role row with 'grant another role' there was no way to remove it.</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The role dropdown now lists the full set of ten roles from one shared source, every role shows a human-readable label (Product Owner, Security Engineer, ...) with no underscores, and each granted-role row has an X to remove it (shown whenever there's more than one). The same labels are used wherever a user's roles are listed. New shared list frontend/src/features/identity/roles.ts; UsersInvites.tsx; tests in roles.test.ts.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H21" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
@@ -1551,20 +1919,14 @@
       <c r="G22" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Several issues on the work-item lifecycle screen. (i) The rail listed brownfield/onboarding phases (context bridge, context extraction, on-boarding) that don't belong on a normal work item, and phase names showed with underscores/number prefixes. (ii) A Story (or any non-Epic) still showed 'Epic' because the screen hard-coded that word. (iv) The run console showed nothing because run events are stored with an 'action' + 'payload' but the console reads 'kind' and 'message', which weren't being sent - so every line rendered blank. (v) Re-running a failed phase sent the run's internal id (a UUID) where the system expects the short phase key, producing 'no AgentSpec registered for key &lt;uuid&gt;', and a failed run gave no reason.</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(i) Phase names are now human-readable everywhere (Task Breakdown, Architecture, ...) and the brownfield/onboarding phases are hidden from a work item's rail - a display-only filter, no change to orchestration (as agreed with the team). (ii) The type badge and headings now show the work item's real type. (iv) Run events now carry a colour ('kind') and a readable 'message' from the action + payload, so the console shows progress - verified live on a real run, e.g. 'Phase dispatched - ideation' and 'Run failed - Command failed with exit code 1'. (v) Re-run now sends the phase key, not the UUID; verified live with the exact id from the report (d32f5ced-...): the UUID reproduces the error, the key '01_ideation' starts a run cleanly. A failed run now shows the actual reason. (iii, type tooltip, was an enhancement and is also done - see the 'Title is mandatory' row.) Files: frontend lifecycle/phases.ts, WorkItemEpic/Task/Defect.tsx, PhasesAndRuns.tsx, RunConsole.tsx, observability/OfflineTakeover.tsx, RunTranscriptScreen.tsx; backend api/serializers.py (RunSerializer agent_key/agent_phase, EventSerializer kind/message).</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
@@ -1583,20 +1945,14 @@
       <c r="G23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Artifacts generated by a phase are registered as internal drafts with the draft text stored inline in the artifact's external_ref.body field and an empty s3_key (the agent hadn't staged a snapshot to object storage). The Preview endpoint only knew how to fetch a body from s3_key, so for these drafts it found nothing and returned 'artifact has no body to preview' even though the text was sitting right there in external_ref.body.</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Taught the preview read-through to also read an internal draft's body from external_ref.body when there is no s3_key yet, choosing the content type from the draft's 'format'. Nothing is copied or stored anywhere new - it's read where it already lives, so tenant isolation and 'platform owns state, not content' are untouched. Verified LIVE on the exact artifact from the report (08efb4c5-...-a232e): it previously 404'd and now returns its 5,834-character markdown body. On MinIO: the local object store container is up and healthy, and artifacts that DO have an s3_key still preview from S3 as before - both paths work. backend/integrations/preview.py (_read_internal); regression test test_preview_internal_artifact_reads_inline_external_ref_body.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H23" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -1635,23 +1991,17 @@
       <c r="G25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When a clarification question offered an 'Other (please specify)' choice, picking it gave the user nowhere to type the specifics, and the literal option text would have been sent as the answer.</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Selecting an 'Other / please specify' style option now reveals a text box, and what the user types is submitted as the answer (an empty box counts as unanswered so a required question still blocks). frontend/src/features/lifecycle/Clarifications.tsx.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="145" x14ac:dyDescent="0.35">
+      <c r="H25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1667,50 +2017,134 @@
       <c r="G26" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When registering generated artifacts the agent raised a clarification asking the user for the project id, which the user can't know. The registration tool required project_id (and run_id) as inputs, so if the agent didn't have them it asked.</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The platform now binds the project id and run id from the run the phase is executing under (the same way the tenant is already bound), so artifact registration fills them in automatically and never asks the user. Done on both the live companion path and the server-side path. runner/companion/state_mcp.py + runner.py (RUNNER_PROJECT_ID), mcp_platform_state/server.py + backend/orchestration/activities.py (PLATFORM_PROJECT_ID/RUN_ID).</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H26" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B27" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B28" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="319" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B29" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="203" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B30" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="325" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="261" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updated Work Item and Integrations Bugs
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Msi\projects\SDLC-App\AI-First-SDLC-App\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08916249-B9BA-4992-97A5-5949A1C6C751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{23CB08F4-CD86-4F8A-943F-B8813342C979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,11 +19,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$216</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="140">
   <si>
     <t>S.No</t>
   </si>
@@ -393,6 +394,137 @@
   </si>
   <si>
     <t>Phases &amp; Runs</t>
+  </si>
+  <si>
+    <t>Enhancement: the create-project page showed a long 'Greenfield starts from a blank profile. Brownfield opens onboarding…' sentence under the track selector; the request was to move it into a tooltip instead.</t>
+  </si>
+  <si>
+    <t>Removed the sentence and surfaced the same explanation as a hover tooltip on the Track selector (an info marker next to the label, plus tooltips on the Greenfield/Brownfield buttons). frontend features/setup/CreateProject.tsx + styles/components.css (.field__tip).</t>
+  </si>
+  <si>
+    <t>After creating a project the profile page showed '✓ Saved · v1' at the top and 'Saving will create v2' at the bottom, even though the profile had never been saved. Confirmed against the backend: a project with no profile yet returns a 404 (no version), and the page was defaulting that missing version to 1 - so it invented 'v1' as already saved, and the next-save hint then said v2.</t>
+  </si>
+  <si>
+    <t>A project with no saved profile is now treated as not-saved (version 0): the top badge shows 'Draft · not saved yet' until the first save, and the save hint correctly reads 'Saving will create v1'. Once saved it shows '✓ Saved · v1', then v2 on the next edit, as expected. frontend features/setup/ProjectProfileEditor.tsx.</t>
+  </si>
+  <si>
+    <t>Clarification: the API GET /api/runners/ is called on a repeating timer on every screen. This is the companion-liveness poll - the app checks whether your machine is still connected. It runs on every screen because the companion status pill lives in the app shell (which is always on screen); it became global as part of the P2 companion-pill fix. React Query de-duplicates all callers under one 'runners' key, so it's a single request per tick, not one per component.</t>
+  </si>
+  <si>
+    <t>Answered, and the background churn was reduced: the poll interval is now configurable, and the always-on app shell polls gently (every ~15s) while the Connect Machine and Phases &amp; Runs screens keep the fast ~4s cadence where live connection status actually matters - about a 4x reduction in background calls on ordinary screens. frontend features/identity/hooks.ts (useRunners interval) + components/AppShell.tsx.</t>
+  </si>
+  <si>
+    <t>On the Connect Machine page the Copy button next to the generated token did nothing when clicked, and on the token card it was barely visible. The button had no click handler at all, and its styling (white text on a translucent background, designed for the dark command block) was almost invisible on the light token card.</t>
+  </si>
+  <si>
+    <t>The Copy buttons on both the token and the command blocks now actually copy to the clipboard (with a fallback for older browsers) and briefly show '✓ Copied!' as confirmation; the button on the light token card was given proper contrast so it's clearly visible. frontend components/ui/index.tsx (new shared CopyButton, used by TokenReveal + CmdBlock) + styles/components.css.</t>
+  </si>
+  <si>
+    <t>On the Connect Machine page, after generating a token, two spinning loaders appeared next to 'Waiting for first check-in…'. The waiting status component already draws its own spinner, and the page was also passing a second spinner into it.</t>
+  </si>
+  <si>
+    <t>Removed the extra spinner; the waiting status now shows a single loader. frontend features/identity/ConnectMachine.tsx.</t>
+  </si>
+  <si>
+    <t>Navigation bar and sidebar showed hardcoded values: the notification bell always showed 4, the companion pill was always green 'Ready' even when not connected, and the sidebar Gates/Clarifications tabs showed fixed default counts.</t>
+  </si>
+  <si>
+    <t>Already resolved as part of the earlier P1/P2 fixes and re-verified here: the sidebar Gates and Clarifications counts and the notification bell are now driven by the real needs-me totals and hide when there's nothing pending; the companion pill (both sidebar and top bar) now shows Ready/Offline from the actual companion status. frontend components/AppShell.tsx.</t>
+  </si>
+  <si>
+    <t>On the Users &amp; Invitations (Workspace Admin) page the subtitle hardcoded 'Acme Corp' as the workspace name instead of the real registered workspace.</t>
+  </si>
+  <si>
+    <t>The subtitle now shows the actual workspace name from the signed-in session (e.g. 'Everyone in the Edven workspace…'). Same fix also covers the Workspace Admin row's hardcoded-name point. frontend features/identity/UsersInvites.tsx.</t>
+  </si>
+  <si>
+    <t>On the Artifacts &amp; Traceability page the search box and the Phase/Type/Status filters did nothing, and the filter dropdowns had no options to pick from.</t>
+  </si>
+  <si>
+    <t>The search box and all three filters now work: search matches on artifact type/phase, and the Phase/Type/Status dropdowns are populated from the artifacts actually present (labels humanised). Filtering is combinable, and a 'No artifacts match these filters' message shows when a combination excludes everything. frontend features/observability/ArtifactsRegistry.tsx.</t>
+  </si>
+  <si>
+    <t>Two problems on the Work Items board. (1) The board only ever showed four phase columns (Ideation, Requirements, Architecture, UX Design) and in the wrong order - PRD was missing - because the columns were a hardcoded list of four rather than the real lifecycle. (2) When a card was waiting for a gate or a clarification, a long status label overflowed and broke the card layout, and gate labels showed a raw phase name with underscores (e.g. '04_architecture gate').</t>
+  </si>
+  <si>
+    <t>(1) The board now builds its columns from the real phase catalog, so every lifecycle phase from Ideation through Deployment shows in correct SDLC order; the board already scrolls sideways so the extra columns just work, and each column title is human-readable. (2) The card header now wraps so a long 'needs' label no longer breaks the layout, and gate labels are humanised (e.g. 'Architecture gate' instead of '04_architecture gate'). Verified: the frontend compiles clean and all 204 UI tests pass, including new tests for the phase-column list and the label humaniser. Files: frontend WorkItemsBoard.tsx, lifecycle/phases.ts (lifecyclePhaseColumns / humanizeLabel), styles/components.css.</t>
+  </si>
+  <si>
+    <t>(1) Generated artifacts are Markdown, but the preview showed the raw Markdown source in a plain text box, and any embedded diagram was unreadable - the preview only knew how to render HTML. (2) Re-running the same work-item phase created a second artifact still labelled v1 instead of v2, and the preview's version history showed v1 for both, because artifact registration always stamped version 1 and never looked at the previous versions.</t>
+  </si>
+  <si>
+    <t>(1) The preview now renders Markdown properly (headings, lists, tables, code) with a real Markdown renderer, and ```mermaid diagram blocks are drawn as actual diagrams instead of shown as text. (2) A newly registered artifact now takes the next version number after the highest existing one for the same project+phase+type, so re-running a phase yields v2, v3, ... Only the version number changes - artifacts stay pointers, not content, and tenant isolation is untouched. Verified LIVE against the running backend: registering the same phase twice returned v1 then v2, the preview reported content type 'text/markdown' with a mermaid diagram in the body, and the version history listed [2, 1]; the single-instance API-contract artifact is unaffected (its tests still pass). Files: frontend components/ui/Markdown.tsx + observability/ArtifactPreviewScreen.tsx; backend mcp_platform_state/tools.py (register_artifact). New dependencies: react-markdown, remark-gfm, mermaid.</t>
+  </si>
+  <si>
+    <t>(1) In the 'Needs me' section of the Workspace Dashboard, phase and role names were shown raw with underscores (e.g. '04_architecture', 'product_owner'). (2) The sidebar and top bar showed hardcoded counts that never changed - Gates always '3', Clarifications always '1', and the notification bell always '4' - regardless of what actually needed the user.</t>
+  </si>
+  <si>
+    <t>(1) The Needs-me tiles and list now show human-readable phase and role names (e.g. 'Architecture', 'Product Owner') via the shared label helpers. (2) The sidebar Gates and Clarifications counts and the notification bell are now driven by the real needs-me totals (bell = gates + clarifications) and hide when nothing is pending, instead of the old fixed 3/1/4. Verified: frontend compiles clean and all 204 UI tests pass. Files: frontend observability/Dashboard.tsx, components/AppShell.tsx (live counts from the existing dashboard rollup).</t>
+  </si>
+  <si>
+    <t>Universal: (1) underscore-style names (phases, roles, statuses) should be human-readable everywhere; (2) values that were hardcoded but should be dynamic should be made dynamic.</t>
+  </si>
+  <si>
+    <t>Bounded sweep across the main in-app screens (brownfield/code-intel screens deferred to their own session, as agreed). (1) Humanised remaining raw phase/role renders on the Gate-role coverage list, Clarifications, Phases &amp; Runs gate tooltip, Work Item Epic/Task clarification rows, Traceability nodes, and the Run transcript title. (2) Made the sidebar/top-bar Companion status pill reflect the real runner status instead of a fixed 'Ready'; the workspace name, nav Gates/Clarifications counts and notification bell were made dynamic in the P1 work and the rows above. Much of this row overlaps the Work Items / Dashboard / Artifacts / Users rows and is cross-referenced there. frontend RolesMatrix.tsx, Clarifications.tsx, PhasesAndRuns.tsx, WorkItemEpic.tsx, WorkItemTask.tsx, TraceabilityView.tsx, RunTranscriptScreen.tsx, AppShell.tsx.</t>
+  </si>
+  <si>
+    <t>Workspace Admin page. (1) Registered and invited users weren't listed - the page showed an 'It's just you so far' empty state, and the users only appeared 'in the background' once the Invite drawer was opened. The empty state was being shown whenever there was at most one user and no still-pending invite, which hid the admin's own row (and any revoked/older invites). (2) The workspace name was hardcoded 'Acme Corp'.</t>
+  </si>
+  <si>
+    <t>(1) The table now shows whenever there's anyone to list (the signed-in admin always is a row); the empty state only appears when the list is genuinely empty. Verified against the live data (workspace 'Edven': the admin user plus a revoked invite) - the admin now shows in the table instead of being hidden. (2) The workspace name is now dynamic (same fix as the Users &amp; Invitations row). frontend features/identity/UsersInvites.tsx.</t>
+  </si>
+  <si>
+    <t>The '← Back to Get started' link kept showing on the Connect Machine / Invite / Integrations screens even after the user had finished setting up. It only hid once the user had a project, a connected machine, AND a second teammate who had accepted an invite - so a solo developer (who never needs to invite anyone) saw the link forever.</t>
+  </si>
+  <si>
+    <t>Per team decision, the link now hides once the user has a project and a connected machine (inviting a team stays optional), so it no longer nags after setup. frontend features/identity/SetupReturnLink.tsx.</t>
+  </si>
+  <si>
+    <t>On Phases &amp; Runs, when the companion isn't connected the screen didn't match the wireframe: the Runs panel still showed hardcoded sample/demo runs instead of an empty state, and the disabled phase list didn't match. (Phase names also needed to be human-readable.)</t>
+  </si>
+  <si>
+    <t>When the companion is offline (or there are simply no runs yet) the Runs panel now shows the 'No runs yet' empty state instead of demo rows, matching the S-18 wireframe, and the disabled phase buttons were aligned to the wireframe (Architecture, UX Design, Task Breakdown). Phase names on this screen go through the shared humaniser. Verified live against the running stack. frontend features/lifecycle/PhasesAndRuns.tsx.</t>
+  </si>
+  <si>
+    <t>In project profile page, the placeholders should be shown for all the fields to be filled, currently only tech stack is available.</t>
+  </si>
+  <si>
+    <t>In the Navigation bar, the companion text not visible clearly and light in color when the companion is offline</t>
+  </si>
+  <si>
+    <t>Navigation Bar</t>
+  </si>
+  <si>
+    <t>While connecting to the Claude Code in the users local system/machine (Companion): Currently the user has to connect to claude code by giving a command containing a token by giving to the claude in local CLI, the user has to be in the backend repository in the CLI to perform this. This is not a user friendly approach
+Enhancement: The approach has to be changed, while fixing this issues discuss with team the best possible way of dealing it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When clicked on create work item, the below text appears below the type dropdown. This needs to be updated
+Epic — a large body of work that runs the full plan tier (ideation → architecture). Story — a user-facing slice of an epic, also plan tier. Task — a concrete build-tier unit of work (implementation → review). Defect — a fix that runs the remediation tier.
+</t>
+  </si>
+  <si>
+    <t>bug</t>
+  </si>
+  <si>
+    <t>In the integration page: The Icons on each card are not visible until the connection is made by the user, but by default the icons should be visible to the user for better understanding.</t>
+  </si>
+  <si>
+    <t>Integrations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Integrations - under connect a capability page: 
+1. When provided the creds for Document store and after testing connect and when clicked on save - after successful connection no message is shown to the user - instead it silently performs the save operation which is confusing to the user.
+2. Initially when connection is tested it did not throw any error message and I was able to click on save. Then user clicked on re-test it showed the below response: http://localhost:8000/api/integrations/c362fb06-5c9e-4075-a1a5-6483f8896a98/test-connection/, Response: {
+    "ok": false,
+    "detail": "No connector registered for docstore:Confluence.",
+    "fix_hint": "Choose a supported vendor for this capability."
+}
+</t>
+  </si>
+  <si>
+    <t>In the integration page: For all the capability connectors the same form filling is shown but it should not be the case, because each one of them will have different fileds for creds. And for each connector the respective vendor drop down shown. For example: For doc store: confluence, share point or built-in docs etc. For task traker: JIRA, Trello etc. 
+Also validate: test connection, save functionality and Re-test issues mentioned in Bug/Issue 39 while doing the current issues.</t>
   </si>
 </sst>
 </file>
@@ -1119,6 +1251,106 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3553489</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>1705429</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BF13599-4F4F-D730-57D1-E1EF7912AAA5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7493000" y="78123144"/>
+          <a:ext cx="3553489" cy="1705428"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>3681931</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>1770673</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BA29DAE-443B-3E0E-5133-72C0A91D4735}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7485673" y="83246058"/>
+          <a:ext cx="3681931" cy="1770673"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1539,21 +1771,6 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement: several form fields had no placeholder text to hint the expected input.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Added placeholders to the remaining form fields (Login password, Accept-Invite name/password, the Invite teammate name field); the signup, create-project and create-work-item forms already had them. frontend features/identity/Login.tsx, AcceptInvite.tsx, UsersInvites.tsx.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
     </row>
     <row r="5" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
@@ -1632,21 +1849,6 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">After first login, the get-started panel on the Workspace Dashboard showed a green tick on 'Create your first project' even though no project had been created. Confirmed against the backend: signup creates the workspace and the admin user but no project, so the tick was simply hardcoded as done in that panel.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The 'Create your first project' step is now shown as the active, not-yet-done step (numbered 1) with a 'Create a project' action, and 'Connect your machine' follows as the next step. frontend features/observability/Dashboard.tsx. (The separate Setup checklist screen was already correct - it computes each step from real data.)</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
     </row>
     <row r="8" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
@@ -1692,20 +1894,14 @@
       <c r="G9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement: the create-project page showed a long 'Greenfield starts from a blank profile. Brownfield opens onboarding…' sentence under the track selector; the request was to move it into a tooltip instead.</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Removed the sentence and surfaced the same explanation as a hover tooltip on the Track selector (an info marker next to the label, plus tooltips on the Greenfield/Brownfield buttons). frontend features/setup/CreateProject.tsx + styles/components.css (.field__tip).</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H9" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="101.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1725,20 +1921,14 @@
       <c r="G10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">After creating a project the profile page showed '✓ Saved · v1' at the top and 'Saving will create v2' at the bottom, even though the profile had never been saved. Confirmed against the backend: a project with no profile yet returns a 404 (no version), and the page was defaulting that missing version to 1 - so it invented 'v1' as already saved, and the next-save hint then said v2.</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A project with no saved profile is now treated as not-saved (version 0): the top badge shows 'Draft · not saved yet' until the first save, and the save hint correctly reads 'Saving will create v1'. Once saved it shows '✓ Saved · v1', then v2 on the next edit, as expected. frontend features/setup/ProjectProfileEditor.tsx.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="362.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1812,20 +2002,14 @@
       <c r="G13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clarification: the API GET /api/runners/ is called on a repeating timer on every screen. This is the companion-liveness poll - the app checks whether your machine is still connected. It runs on every screen because the companion status pill lives in the app shell (which is always on screen); it became global as part of the P2 companion-pill fix. React Query de-duplicates all callers under one 'runners' key, so it's a single request per tick, not one per component.</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Answered, and the background churn was reduced: the poll interval is now configurable, and the always-on app shell polls gently (every ~15s) while the Connect Machine and Phases &amp; Runs screens keep the fast ~4s cadence where live connection status actually matters - about a 4x reduction in background calls on ordinary screens. frontend features/identity/hooks.ts (useRunners interval) + components/AppShell.tsx.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H13" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1845,20 +2029,14 @@
       <c r="G14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On the Connect Machine page the Copy button next to the generated token did nothing when clicked, and on the token card it was barely visible. The button had no click handler at all, and its styling (white text on a translucent background, designed for the dark command block) was almost invisible on the light token card.</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Copy buttons on both the token and the command blocks now actually copy to the clipboard (with a fallback for older browsers) and briefly show '✓ Copied!' as confirmation; the button on the light token card was given proper contrast so it's clearly visible. frontend components/ui/index.tsx (new shared CopyButton, used by TokenReveal + CmdBlock) + styles/components.css.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="58" customHeight="1" x14ac:dyDescent="0.35">
@@ -1905,20 +2083,14 @@
       <c r="G16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On the Connect Machine page, after generating a token, two spinning loaders appeared next to 'Waiting for first check-in…'. The waiting status component already draws its own spinner, and the page was also passing a second spinner into it.</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Removed the extra spinner; the waiting status now shows a single loader. frontend features/identity/ConnectMachine.tsx.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H16" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="116" customHeight="1" x14ac:dyDescent="0.35">
@@ -1992,23 +2164,17 @@
       <c r="G19" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Navigation bar and sidebar showed hardcoded values: the notification bell always showed 4, the companion pill was always green 'Ready' even when not connected, and the sidebar Gates/Clarifications tabs showed fixed default counts.</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Already resolved as part of the earlier P1/P2 fixes and re-verified here: the sidebar Gates and Clarifications counts and the notification bell are now driven by the real needs-me totals and hide when there's nothing pending; the companion pill (both sidebar and top bar) now shows Ready/Offline from the actual companion status. frontend components/AppShell.tsx.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="116" x14ac:dyDescent="0.35">
+      <c r="H19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="145" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -2024,20 +2190,14 @@
       <c r="G20" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On the Users &amp; Invitations (Workspace Admin) page the subtitle hardcoded 'Acme Corp' as the workspace name instead of the real registered workspace.</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The subtitle now shows the actual workspace name from the signed-in session (e.g. 'Everyone in the Edven workspace…'). Same fix also covers the Workspace Admin row's hardcoded-name point. frontend features/identity/UsersInvites.tsx.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H20" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="188.5" x14ac:dyDescent="0.35">
@@ -2134,20 +2294,14 @@
       <c r="G24" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On the Artifacts &amp; Traceability page the search box and the Phase/Type/Status filters did nothing, and the filter dropdowns had no options to pick from.</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The search box and all three filters now work: search matches on artifact type/phase, and the Phase/Type/Status dropdowns are populated from the artifacts actually present (labels humanised). Filtering is combinable, and a 'No artifacts match these filters' message shows when a combination excludes everything. frontend features/observability/ArtifactsRegistry.tsx.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="145" x14ac:dyDescent="0.35">
@@ -2218,20 +2372,14 @@
       <c r="G27" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two problems on the Work Items board. (1) The board only ever showed four phase columns (Ideation, Requirements, Architecture, UX Design) and in the wrong order - PRD was missing - because the columns were a hardcoded list of four rather than the real lifecycle. (2) When a card was waiting for a gate or a clarification, a long status label overflowed and broke the card layout, and gate labels showed a raw phase name with underscores (e.g. '04_architecture gate').</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) The board now builds its columns from the real phase catalog, so every lifecycle phase from Ideation through Deployment shows in correct SDLC order; the board already scrolls sideways so the extra columns just work, and each column title is human-readable. (2) The card header now wraps so a long 'needs' label no longer breaks the layout, and gate labels are humanised (e.g. 'Architecture gate' instead of '04_architecture gate'). Verified: the frontend compiles clean and all 204 UI tests pass, including new tests for the phase-column list and the label humaniser. Files: frontend WorkItemsBoard.tsx, lifecycle/phases.ts (lifecyclePhaseColumns / humanizeLabel), styles/components.css.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H27" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="333.5" x14ac:dyDescent="0.35">
@@ -2250,20 +2398,14 @@
       <c r="G28" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) Generated artifacts are Markdown, but the preview showed the raw Markdown source in a plain text box, and any embedded diagram was unreadable - the preview only knew how to render HTML. (2) Re-running the same work-item phase created a second artifact still labelled v1 instead of v2, and the preview's version history showed v1 for both, because artifact registration always stamped version 1 and never looked at the previous versions.</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) The preview now renders Markdown properly (headings, lists, tables, code) with a real Markdown renderer, and ```mermaid diagram blocks are drawn as actual diagrams instead of shown as text. (2) A newly registered artifact now takes the next version number after the highest existing one for the same project+phase+type, so re-running a phase yields v2, v3, ... Only the version number changes - artifacts stay pointers, not content, and tenant isolation is untouched. Verified LIVE against the running backend: registering the same phase twice returned v1 then v2, the preview reported content type 'text/markdown' with a mermaid diagram in the body, and the version history listed [2, 1]; the single-instance API-contract artifact is unaffected (its tests still pass). Files: frontend components/ui/Markdown.tsx + observability/ArtifactPreviewScreen.tsx; backend mcp_platform_state/tools.py (register_artifact). New dependencies: react-markdown, remark-gfm, mermaid.</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H28" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="319" x14ac:dyDescent="0.35">
@@ -2282,20 +2424,14 @@
       <c r="G29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) In the 'Needs me' section of the Workspace Dashboard, phase and role names were shown raw with underscores (e.g. '04_architecture', 'product_owner'). (2) The sidebar and top bar showed hardcoded counts that never changed - Gates always '3', Clarifications always '1', and the notification bell always '4' - regardless of what actually needed the user.</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) The Needs-me tiles and list now show human-readable phase and role names (e.g. 'Architecture', 'Product Owner') via the shared label helpers. (2) The sidebar Gates and Clarifications counts and the notification bell are now driven by the real needs-me totals (bell = gates + clarifications) and hide when nothing is pending, instead of the old fixed 3/1/4. Verified: frontend compiles clean and all 204 UI tests pass. Files: frontend observability/Dashboard.tsx, components/AppShell.tsx (live counts from the existing dashboard rollup).</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H29" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="203" x14ac:dyDescent="0.35">
@@ -2314,20 +2450,14 @@
       <c r="G30" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Universal: (1) underscore-style names (phases, roles, statuses) should be human-readable everywhere; (2) values that were hardcoded but should be dynamic should be made dynamic.</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bounded sweep across the main in-app screens (brownfield/code-intel screens deferred to their own session, as agreed). (1) Humanised remaining raw phase/role renders on the Gate-role coverage list, Clarifications, Phases &amp; Runs gate tooltip, Work Item Epic/Task clarification rows, Traceability nodes, and the Run transcript title. (2) Made the sidebar/top-bar Companion status pill reflect the real runner status instead of a fixed 'Ready'; the workspace name, nav Gates/Clarifications counts and notification bell were made dynamic in the P1 work and the rows above. Much of this row overlaps the Work Items / Dashboard / Artifacts / Users rows and is cross-referenced there. frontend RolesMatrix.tsx, Clarifications.tsx, PhasesAndRuns.tsx, WorkItemEpic.tsx, WorkItemTask.tsx, TraceabilityView.tsx, RunTranscriptScreen.tsx, AppShell.tsx.</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H30" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="325" customHeight="1" x14ac:dyDescent="0.35">
@@ -2346,20 +2476,14 @@
       <c r="G31" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workspace Admin page. (1) Registered and invited users weren't listed - the page showed an 'It's just you so far' empty state, and the users only appeared 'in the background' once the Invite drawer was opened. The empty state was being shown whenever there was at most one user and no still-pending invite, which hid the admin's own row (and any revoked/older invites). (2) The workspace name was hardcoded 'Acme Corp'.</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) The table now shows whenever there's anyone to list (the signed-in admin always is a row); the empty state only appears when the list is genuinely empty. Verified against the live data (workspace 'Edven': the admin user plus a revoked invite) - the admin now shows in the table instead of being hidden. (2) The workspace name is now dynamic (same fix as the Users &amp; Invitations row). frontend features/identity/UsersInvites.tsx.</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H31" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="261" x14ac:dyDescent="0.35">
@@ -2378,23 +2502,17 @@
       <c r="G32" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The '← Back to Get started' link kept showing on the Connect Machine / Invite / Integrations screens even after the user had finished setting up. It only hid once the user had a project, a connected machine, AND a second teammate who had accepted an invite - so a solo developer (who never needs to invite anyone) saw the link forever.</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Per team decision, the link now hides once the user has a project and a connected machine (inviting a team stays optional), so it no longer nags after setup. frontend features/identity/SetupReturnLink.tsx.</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="H32" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="232" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2410,93 +2528,192 @@
       <c r="G33" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On Phases &amp; Runs, when the companion isn't connected the screen didn't match the wireframe: the Runs panel still showed hardcoded sample/demo runs instead of an empty state, and the disabled phase list didn't match. (Phase names also needed to be human-readable.)</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the companion is offline (or there are simply no runs yet) the Runs panel now shows the 'No runs yet' empty state instead of demo rows, matching the S-18 wireframe, and the disabled phase buttons were aligned to the wireframe (Architecture, UX Design, Task Breakdown). Phase names on this screen go through the shared humaniser. Verified live against the running stack. frontend features/lifecycle/PhasesAndRuns.tsx.</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H33" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B34" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B35" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="261" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B36" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="232" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B37" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B38" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B39" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B40" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
@ Fix P1 integrations connectors: per-vendor forms + slug save (Bugs #39, #40)
Add a backend connector catalog (capability -> registered vendors -> binding/secret
fields) exposed at GET /api/integrations/catalog/. The connect form now renders the
correct vendor list and per-vendor fields for every capability and saves the registry
slug, so test-connection no longer fails with "No connector registered". Save shows an
explicit success/error banner, the grid reflects configured state, and an already-
connected capability hydrates + edits via PATCH instead of a duplicate POST.

Verified live (Jira) and by a test covering all six connectors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -2690,9 +2690,19 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>The connect form saved the vendor's display name ('Confluence') as the connector, but the backend connector registry is keyed by lowercase slugs ('confluence'), so test-connection failed with "No connector registered for docstore:Confluence." Separately, Save gave no confirmation - it mutated silently.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>The form now sends the registered connector slug (from a backend catalog that only lists builder-wired vendors, so this mismatch can't happen), and Save shows an explicit success or error banner (e.g. 'Jira saved. Test the connection to verify it.' / 'already connected'). The grid now shows 'Connected' once a connection is configured. Also fixed a hydration bug so opening an already-connected capability pre-fills its saved vendor/binding and edits via PATCH instead of a duplicate POST. (backend apps/integrations/catalog.py + api/serializers.py + api/views.py catalog endpoint; frontend features/setup/ConnectCapability.tsx + hooks.ts + api.ts + types.ts.) Verified live: Save -&gt; 'Saved' -&gt; Test -&gt; 'Connection OK'.</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2721,9 +2731,19 @@
           <t>P1</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>The Connect-a-capability form was hardcoded to Confluence-only fields (Space key, Base URL) and a Confluence vendor dropdown for every capability, so all six connectors showed the same form.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Added a backend connector catalog (capability -&gt; its vendors -&gt; that vendor's binding + secret fields) exposed at GET /api/integrations/catalog/. The form now renders the correct vendor list and the correct per-vendor fields for each capability - e.g. Task tracker shows Jira with Project key / Base URL / API token; Design source shows Figma with File key / Access token; Test management shows Xray with Client ID / Client secret; Code intelligence shows the Built-in analyzer with no credentials. The #39 test/save/re-test flow was validated as part of this. (backend apps/integrations/catalog.py; frontend features/setup/ConnectCapability.tsx.)</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix open_build_pr for agent pre-PR code pointer; log Bugs 86-88
- build_activities: open_build_pr_core now reconciles an agent-registered
  pre-PR code pointer (branch/files, no PR) in place — opens the PR and
  updates the pointer instead of mistaking it for an opened PR (KeyError
  'repo'). run_code_review_core guards non-PR refs. (_is_pr_ref helper)
- test_build_activities: cover the pre-PR-pointer reconcile path.
- Bugs.xlsx: log S.No 86 (open_build_pr pre-PR pointer, Fixed),
  87 (agent self-transitions WorkItem to done, Open),
  88 (external GitHub merge orphans BuildWorkflow, Open).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -5051,19 +5051,154 @@
         </is>
       </c>
     </row>
-    <row r="87" spans="1:1">
+    <row r="87" spans="1:10" ht="409.6">
       <c r="A87" s="2">
         <v>86</v>
       </c>
-    </row>
-    <row r="88" spans="1:1">
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build fails after push: agent's pre-PR 'code' pointer makes open_build_pr skip opening the real PR, then code review crashes (KeyError 'repo')</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The 07_implementation agent registers a pre-PR 'code' pointer (branch/files_changed, no PR) which its body says 'the platform reconciles with the PR it opens'. But open_build_pr_core treated ANY existing code artifact with a truthy external_ref as 'PR already opened' and returned early, so it never opened the real PR; then run_code_review_core read code.external_ref['repo'] and raised KeyError('repo'). Observed live on WI-18: code committed and pushed to feature/WI-aa6020d0 on GitHub, but NO PR opened and the run failed — blocking PR to review to merge.</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implementation / Build pipeline</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/orchestration/build_activities.py open_build_pr_core + run_code_review_core; agents/07_implementation/agent.md (~line 264 register code pointer)</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">open_build_pr's idempotency check mistook the agent's pre-PR pointer for an opened PR; the documented 'platform reconciles the pointer with the PR' behaviour was never implemented.</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Added _is_pr_ref (a real PR ref carries repo+number). open_build_pr short-circuits only on a real opened PR; when the agent's pre-PR pointer exists it OPENS the PR and reconciles that artifact in place (update_artifact with the PR external_ref + STAGED) instead of skipping/duplicating. run_code_review guards on _is_pr_ref (clear error, not KeyError). New test test_open_pr_reconciles_agent_pre_pr_pointer + 10 existing build-activities tests pass. Worker reloaded; failed WI-18 run cleaned for a fresh re-trigger.</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="409.6">
       <c r="A88" s="2">
         <v>87</v>
       </c>
-    </row>
-    <row r="89" spans="1:1">
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implementation agent can transition the WorkItem to 'done' itself (mid-build), bypassing the platform merge gate that owns completion</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">During the WI-18 build, the WorkItem was set to state='done' at 12:25:51 — a full minute BEFORE the PR opened (12:26:51), with no merge-gate approval and no webhook. The only actor with the tool and that timing is the 07_implementation agent: transition_work_item is in the build-phase tool allowlist (BUILD_STATE_TOOLS), so the agent marked its own task 'done' as it finished. This violates control-plane ownership of completion (non-negotiable: gates live in the control plane) — the platform should set 'done' only after the merge gate is approved and the PR merged. Effect: WorkItem state becomes premature/unreliable and the merge gate is cosmetic for state purposes.</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implementation / Guardrails / Work Items</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">runner/companion/runner.py BUILD_STATE_TOOLS ('transition_work_item'); backend/api/runner_views.py allowlist; mcp_platform_state/tools.py transition_work_item; backend/orchestration/build_workflow.py owns the done transition (~line 150)</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">transition_work_item is exposed to the build agent (needed for remediation child items) but nothing stops it from transitioning the MAIN WorkItem into a gated/terminal state. The platform's post-merge completion transition and the agent's tool access overlap.</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open — team to address later. Options: remove transition_work_item from the build agent's allowlist (platform owns all WorkItem state); or scope it so the agent may only transition remediation child items it owns; or reject agent-initiated transitions to gated states ('accepted'/'done') server-side.</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="409.6">
       <c r="A89" s="2">
         <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merging the PR directly on GitHub bypasses the platform merge gate and orphans the BuildWorkflow (no reachable webhook to reconcile the external merge)</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The intended completion flow is: PR -&gt; platform code review -&gt; merge gate approved in the platform -&gt; platform merges via CodeHost -&gt; WorkItem done. On WI-18 the developer merged PR #1 directly on GitHub instead. Because the platform runs on localhost and no GitHub webhook is configured/reachable (GITHUB_WEBHOOK_SECRET empty; GitHub cannot reach localhost), the platform never learned of the merge. Result: the BuildWorkflow (build-run-dbf76d68) is left RUNNING, parked at the review/merge-gate step for a PR that is already merged, and will never complete on its own. The code did land on main (the developer's merge), but the platform workflow and gate are out of sync.</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build pipeline / CodeHost / Webhooks</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/integrations/webhooks.py (GitHub PR-merge -&gt; transition done, needs a reachable endpoint + GITHUB_WEBHOOK_SECRET); backend/orchestration/build_workflow.py (merge gate expects the platform to merge); settings.GITHUB_WEBHOOK_SECRET (empty)</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The platform-driven merge (via the merge gate) and an external GitHub merge are two paths; only the platform-driven one completes the workflow. The inbound webhook that would reconcile an external merge is not configured/reachable in local dev, so external merges strand the workflow.</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open — team to address later. Either drive merges through the platform merge gate (Gates page) so the platform merges + completes the workflow, OR expose the platform on a reachable URL (tunnel/deploy) + configure the GitHub webhook with GITHUB_WEBHOOK_SECRET so external merges reconcile (transition done + let the workflow finish). Interim: terminate the currently-orphaned build-run-dbf76d68 workflow.</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="90" spans="1:1">

</xml_diff>

<commit_message>
Fix companion-run reliability before multi-repo build test (Bugs 84 + 105)
S.No 84: _resolve_enrollment prefers the newest ONLINE enrollment
(last_seen within ONLINE_THRESHOLD), then newest ever-seen, then newest
overall - a never-connected newer enrollment can no longer capture a
dispatch while the live companion polls 204s.

S.No 105: the companion survives a backend/worker restart - the work
poll retries connection errors with capped exponential backoff instead
of dying, and a finished phase/build report is retried (~2 min) so
completed work is not lost to a restart at report time.

Bugs.xlsx rows 84/105 -> Fixed (image-safe zip/XML update).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="230">
   <si>
     <t>S.No</t>
   </si>
@@ -922,6 +922,12 @@
   </si>
   <si>
     <t>Connet Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIXED (2026-07-14). _resolve_enrollment in backend/orchestration/trigger.py no longer picks purely by recency. It now prefers, in order: (1) the newest ACTIVE enrollment that is ONLINE (last_seen within the 2-minute ONLINE_THRESHOLD from apps/runs/enrollment.py - i.e. a companion is heartbeating/polling with that token right now); (2) the newest that has EVER checked in; (3) the newest overall (nothing connected yet - e.g. the user triggers before starting the companion; the dispatch waits, same as before). Applies to BOTH trigger_phase and trigger_build (they share the helper). Result: a Connect-Machine visit that mints a newer-but-never-connected enrollment can no longer capture a dispatch while the live companion polls 204s. Tests: backend/tests/test_build_trigger_api.py::test_resolve_enrollment_prefers_newest_online_over_newer_dead_one and test_resolve_enrollment_falls_back_seen_then_newest. Revoking stale enrollments is still good hygiene but no longer required for a correct dispatch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIXED (2026-07-14). The companion now survives a backend/worker restart instead of silently dying (a docker restart surfaces as a connection error/OSError on the long-poll, not an HTTP status - previously that escaped the serve loop and killed the daemon). Changes in runner/companion/daemon.py: (1) serve() catches connection-level errors from the work-poll and retries forever with capped exponential backoff (poll interval doubling up to 60s), logging 'backend unreachable... reconnecting in Ns' and 'backend reconnected; resuming'; (2) _report() retries a finished phase/build report through a transient outage (~2 min of backoff) so completed work is not lost to a restart at report time; HTTP 4xx/5xx answers still fail immediately. The 30s heartbeat already swallowed its own failures and resumes by itself. Tests: backend/tests/test_companion_daemon.py::test_claim_survives_backend_outage_and_resumes, test_report_retries_through_transient_outage, test_report_gives_up_after_bounded_retries. Operational note: a plain backend/worker restart now needs NO manual companion action; reconnecting with the SAME token only matters if the companion process itself is killed.</t>
   </si>
 </sst>
 </file>
@@ -4990,15 +4996,11 @@
           <t xml:space="preserve">_resolve_enrollment orders enrollments by recency and does not prefer ones that have actually checked in (last_seen recent / within the online window). RC-4 collapses re-enrollments by project but the selection still ignores liveness.</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not yet fixed (deferred to avoid a backend restart mid-build). Fix: _resolve_enrollment should prefer the newest enrollment with a recent last_seen (online) and ignore never-checked-in / stale ones; optionally fail-fast or re-point a dispatch whose target enrollment is offline. Interim mitigation: keep a single fresh enrollment (wipe stale ones before triggering).</t>
-        </is>
-      </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
+      <c r="I85" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="409.6">
@@ -6040,15 +6042,11 @@
           <t xml:space="preserve">The companion's heartbeat/work-poll loop doesn't robustly survive the backend going away and returning (transient connection loss on restart) - it stops rather than retrying until reconnected.</t>
         </is>
       </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open - P2, later. Make the companion resilient to a transient backend outage: retry/reconnect the heartbeat + work-poll with backoff instead of stopping; show a clear reconnecting state. Interim workaround: after any backend/worker restart, manually reconnect the companion with the SAME token (a new token would orphan an already-dispatched run - row 84).</t>
-        </is>
-      </c>
-      <c r="J106" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
+      <c r="I106" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="J106" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="107" spans="1:10" ht="409.6">

</xml_diff>

<commit_message>
Log enhancement S.No 140: no human action to resolve a failed/redundant WorkItem
Surfaced testing S.No 136/139 — an empty/redundant build (TASK-002) correctly FAILS with a
clear reason, but the WorkItem then sits at in_progress with no product path for a human to
mark it done, close it as redundant, or skip it. state is read-only on the API/UI (mutated
only by the orchestrator happy path); the only offered action is Retry, which re-fails for a
redundant task. Proposed: a gated "mark done / close as redundant / skip" action + endpoint
(reuse done or add a distinct terminal state). Related S.No 76. Logged Open, P2.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -7763,9 +7763,54 @@
         </is>
       </c>
     </row>
-    <row r="141" spans="1:1">
+    <row r="141" spans="1:10">
       <c r="A141" s="2">
         <v>140</v>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No human action to resolve a non-mergeable / redundant / failed WorkItem: a task can only reach 'done' via a successful automated build+merge. A build that fails (empty/redundant build, or a merge conflict needing manual resolution) leaves the WorkItem stuck at in_progress with no product path for a human to mark it done, skip it, or close it as redundant.</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surfaced 2026-07-16 while testing S.No 136/139: TASK-002 (redundant with TASK-001) produced an empty build that correctly FAILED with 'Empty build: no changes to commit'. The WorkItem then sits at in_progress with the branch/draft PR left in place, and the only offered action is Retry - which re-fails for a genuinely redundant task. A human can freely trigger the NEXT task (tasks are independent unless depends_on) but cannot close/resolve the failed one. Today the only ways to reach done are the happy-path orchestrator flow or an admin DB state change.</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work Items / Build recovery UX</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/apps/workitems/models.py (State: proposed/accepted/in_progress/in_review/blocked/done, no transition validation); backend/api/serializers.py WorkItemPatchSerializer (state NOT writable) + read_only state; backend/api/views.py WorkItemViewSet (trigger/build/take-over/lifecycle - no transition/mark-done action); mcp_platform_state/tools.py transition_work_item (any-&gt;any, internal only); frontend RunConsole.tsx (Retry only) / WorkItemTask.tsx (done is display-only) / OfflineTakeover.tsx</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WorkItem.state is read-only on the API (excluded from WorkItemPatchSerializer; read_only on the read serializer) and mutated ONLY internally by the orchestrator (successful build+merge / gate / reject / takeover). No human-facing transition/mark-done/close/skip action or endpoint exists; the frontend offers only Retry / Trigger phase / manual takeover (sets takeover_flag, not state). transition_work_item allows any-&gt;any but is unexposed to users.</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPEN - proposed: add a GATED human action + API endpoint to move a WorkItem to a terminal state outside the happy path (e.g. 'Mark done', 'Close as redundant / won't-do', or 'Skip'), surfaced on the Work Items board + task page, with an audit Event. Decide whether to reuse 'done' or add a distinct terminal state (e.g. 'closed'/'cancelled') to distinguish completed-by-build from human-closed; guard with role/permission. Related S.No 76 (no task-edit UI; state not editable).</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="142" spans="1:1">

</xml_diff>

<commit_message>
Log enhancement S.No 141: merge-conflict recovery (both options in one row)
Two related enhancements for recovering from a merge conflict without redoing the whole build:
ENH-2 (implement now) = re-openable merge gate / merge-only retry so a resolved conflict
completes through the platform without a full rebuild (soft-reconcile, like S.No 89); ENH-1
(future/if-needed) = reconcile the Run status on an external GitHub merge (part of S.No 88,
largely unnecessary once ENH-2 exists). Logged Open, P2.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -7813,9 +7813,54 @@
         </is>
       </c>
     </row>
-    <row r="142" spans="1:1">
+    <row r="142" spans="1:10">
       <c r="A142" s="2">
         <v>141</v>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merge gate can't recover from a conflict without redoing the whole build. TWO related enhancements (logged together): (ENH-2, IMPLEMENT NOW) Merge-only retry / re-openable merge gate - when a merge hits a conflict, PAUSE at the merge step and let the user retry the merge after fixing the conflict, WITHOUT re-running the whole build. (ENH-1, FUTURE / only if needed) Reconcile the Run status on an EXTERNAL merge - when a user merges the PR by hand in GitHub, also flip the Run from failed to done (today the webhook updates the WorkItem + artifact but leaves the Run 'failed').</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Today a merge conflict marks the ENTIRE build failed and ends the workflow, so finishing means re-running everything (AI re-writes the code, re-reviews, re-opens the PR) just to retry one merge. ENH-2 fixes this: keep the build paused at the merge gate; after the user resolves the conflict in GitHub they press Merge/Approve again and the platform completes the merge through its OWN flow (run + gate + work-item all stay correct automatically, no rebuild). ENH-1 covers a DIFFERENT path - the user merges by hand in GitHub instead of letting the platform do it; then the platform only learns via webhook (S.No 88) and today leaves the Run status stale. TEAM PLAN (2026-07-16): implement ENH-2 now; keep ENH-1 for future - it overlaps S.No 88 and is only needed if users merge OUTSIDE the platform. If ENH-2 is used, ENH-1 is largely unnecessary. Same 'soft, reconcilable' idea as the S.No 89 fix, applied to merge conflicts.</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build pipeline / Merge gate recovery</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/orchestration/build_workflow.py (merge gate + ActivityError-&gt;mark_build_failed is TERMINAL on a conflict); backend/orchestration/build_activities.py merge_build_pr_core (S.No 136 dirty-&gt;fail); backend/integrations/webhooks.py _reconcile_pull_request (updates WorkItem+artifact on an external merge, NOT the Run); frontend Gates.tsx (merge gate) + RunConsole.tsx. Related: S.No 88 (external merge / missing webhook), S.No 89 (soft-reconcilable pattern), S.No 136 (conflict detection).</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On a merge conflict the BuildWorkflow catches the ActivityError and calls mark_build_failed, which is TERMINAL - the workflow ends, so there is no live workflow to retry the merge and the merge-gate Approval is already spent. The only ways forward today are a full re-trigger (rebuilds from 07) or an external GitHub merge (needs the S.No 88 webhook, which also does not reconcile the Run status).</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPEN. PLAN: implement ENH-2 now = make a merge conflict NON-terminal - pause the build at the merge gate (re-openable) and add a merge-only retry so the user, after resolving the conflict, can complete the merge THROUGH the platform without a rebuild (mirror the S.No 89 soft-reconcile approach: keep the workflow alive / re-openable instead of dead). ENH-1 (reconcile Run status on an external merge) kept for FUTURE / if-needed - it is part of the S.No 88 external-merge story and largely unnecessary once ENH-2 exists.</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="143" spans="1:1">

</xml_diff>

<commit_message>
Surface merge conflict on the re-opened merge gate (ENH-2 / S.No 141)
ENH-2 re-opened the merge gate on a conflict but the gate panel gave the
user no reason for the retry (only the run console did). Expose the conflict
on the pending merge gate and explain the retry.

- ApprovalSerializer.merge_conflict: the run's recorded conflict reason,
  emitted ONLY while the gate is pending — a normal gate returns null, so the
  banner never shows on other approve gates.
- Gates.tsx: a warning banner on the pending merge gate — "resolve in GitHub,
  approve again to retry the merge, no rebuild needed."

ENH-2 validated live on TASK-003 (run 1d1dd943): injected an add/add conflict,
approve -> gate re-opened (once per remaining conflict) -> resolved -> approve
-> platform merged PR #1, WorkItem done, run completed, no rebuild. Bugs.xlsx
S.No 141 -> Fixed (image-safe, 33 media parts byte-identical).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -7881,12 +7881,12 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPEN. PLAN: implement ENH-2 now = make a merge conflict NON-terminal - pause the build at the merge gate (re-openable) and add a merge-only retry so the user, after resolving the conflict, can complete the merge THROUGH the platform without a rebuild (mirror the S.No 89 soft-reconcile approach: keep the workflow alive / re-openable instead of dead). ENH-1 (reconcile Run status on an external merge) kept for FUTURE / if-needed - it is part of the S.No 88 external-merge story and largely unnecessary once ENH-2 exists.</t>
+          <t xml:space="preserve">ENH-2 IMPLEMENTED &amp; VALIDATED LIVE (@ 66b70c8, + gate banner). A merge conflict is now NON-terminal: merge_build_pr detects a dirty PR and raises a typed MergeConflict; the BuildWorkflow catches it, RE-OPENS the merge gate (resets the approval to pending, records outputs.merge_conflict + a build.merge_conflict event) and waits — instead of failing the build. The user resolves the conflict in GitHub and approves again; the platform retries ONLY the merge (no rebuild, no re-review). Proven live on TASK-003 (run 1d1dd943): injected an add/add conflict on .env.example -&gt; approve -&gt; gate re-opened (once per remaining conflict) -&gt; resolved -&gt; approve -&gt; platform merged PR#1 (merge commit c1d7552a) -&gt; WorkItem done -&gt; run completed, with NO rebuild across retries. The merge gate now shows a warning banner explaining the conflict + retry (ApprovalSerializer.merge_conflict; shown ONLY on a re-opened merge gate, never other gates). ENH-1 (reconcile Run status on an EXTERNAL GitHub merge) remains FUTURE / optional — it overlaps S.No 88 and is only needed if users merge outside the platform, which ENH-2 makes largely unnecessary.</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated the Bugs sheet with Integrations, phase run erros etc.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="102" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C231EF7A-42E9-490A-B4B0-64F9F645D887}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{285B08F5-3480-48DB-957D-3CBD7D1D2C50}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="13">
+  <futureMetadata name="XLRICHVALUE" count="16">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -130,8 +130,29 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="13"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="14"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="15"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="13">
+  <valueMetadata count="16">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -171,12 +192,21 @@
     <bk>
       <rc t="1" v="12"/>
     </bk>
+    <bk>
+      <rc t="1" v="13"/>
+    </bk>
+    <bk>
+      <rc t="1" v="14"/>
+    </bk>
+    <bk>
+      <rc t="1" v="15"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="729">
   <si>
     <t>S.No</t>
   </si>
@@ -955,6 +985,9 @@
 3. The presentation format is also not good and confusing to the team whether they are directly rendered as output or any manipulations being done while presenting the clarifications by our engine?</t>
   </si>
   <si>
+    <t>Fixed on two fronts. (1) UI: the 'Other' free-text box no longer fails to appear when the agent labels an option with a letter prefix (e.g. 'd) Other') — the reveal now strips a leading enumerator before matching. Verified LIVE against the running app (served bundle). (2) Authoring: the ask_human tool contract now tells every phase agent to write ONE short plain-language question and put choices ONLY in the structured options, never inline them in the question text — stopping the duplicated-options / uppercase wall-of-text. Frontend + agent-contract change; regression test added.</t>
+  </si>
+  <si>
     <t>In the Connect Machine page: 
 When the user has connected his local companion and created a work item and executed/run a phase for example: Ideation, after sometime the engine is showing companion disconnect and saying to connect again wih error message. Sharing you the reference images, clearly go through and findout the root cause first and report it to the team working on this issue and take their approval before fixing.
 Due to this issue, even when the team is running the next phase i.e requirements, the UI showing that phase is running but never got any artifacts as ouptut or any gate for that run. This is very serious issue and need to be analysed accurately.
@@ -1218,7 +1251,7 @@
     <t>The token_ref indirection is a documented Phase-5 seam; Phase 1 hardcoded from_settings() and decrypt_secrets was never wired into the connector builders.</t>
   </si>
   <si>
-    <t>Deferred (Phase-5 seam). Fix = wire decrypt_secrets(conn) into the connector builders so per-tenant creds are used and retire the .env fallback; make test-connection a real reachability probe. For the current greenfield test, Jira is connected exactly like Confluence: the Integrations connection supplies scopes.project_key and the shared Atlassian creds live in .env.</t>
+    <t>Per-tenant credentials are now actually used at runtime. Figma, Xray and Atlassian (Confluence/Jira) resolve credentials from the tenant's own IntegrationConnection (decrypt_secrets) instead of the shared server .env — closing the multi-tenant credential-leak class already fixed for GitHub (S.No 112). Per-field .env fallback kept so CI/tests are unchanged. Done together with S.No 113. Config tests added.</t>
   </si>
   <si>
     <t>No dedicated Task Breakdown review screen; dependencies and estimates are not surfaced before the gate</t>
@@ -1269,7 +1302,7 @@
     <t>No idempotency/natural key on work-item creation, unlike register_artifact which versions siblings.</t>
   </si>
   <si>
-    <t>Deferred. Add an idempotency key (e.g. project+phase+title, or an agent-supplied external key) so a re-run upserts rather than duplicates. For today's run, delete any partial batch before re-triggering.</t>
+    <t>Three-part fix. (A) create_work_item is now idempotent: re-running Task Breakdown REPLACES matching proposed work items (natural key project+type+title+parent) instead of duplicating the whole backlog; already-accepted/in-progress/done items are never touched. (B) A concurrent-run guard blocks a second trigger while a run is live (HTTP 409), for both phase and build triggers. (C) A confirm dialog on both trigger surfaces (Phases &amp; Runs and the Task page): Case 1 (completed) warns 're-running restarts and replaces THIS phase's artifacts, no duplicates'; Case 2 (in progress) blocks with a clear message. Idempotency + guard tests added.</t>
   </si>
   <si>
     <t>Jira integration is one-way (create-only): no inbound webhook, no status sync, dropped fields</t>
@@ -1482,7 +1515,7 @@
     <t>FAILED is treated as terminal and a late successful phase.reported does not reconcile it; report_timeout (7200s wall-clock from dispatch) trips on an asleep companion that later completes fine. Once run() returns on takeover the workflow is gone, so both phase_report and decide_gate have no live workflow to signal.</t>
   </si>
   <si>
-    <t>Open - co-dev (tarun's team) to fix. Proposed: (1) a late phase.reported ok reconciles the run to awaiting_gate + opens the gate; (2) treat takeover as a reclaimable 'parked' state, not terminal, while the companion still heartbeats; (3) decide_gate tolerates an absent/closed workflow and drives publish_artifacts + transition_work_item directly; (4) fix the misleading UI copy. Run 8738d4ba manually reconciled to awaiting_gate 2026-07-13.</t>
+    <t>Fixed (session 2026-07-15). Report-timeout takeover is now NON-terminal and reconcilable. (1) New Run.Status.STALLED (runs migration 0006) replaces terminal FAILED on timeout: mark_phase_takeover_core parks the run as STALLED + sets the WorkItem takeover_flag. (2) AgentRunWorkflow no longer returns on timeout: it marks the soft takeover then KEEPS waiting for the report, so a companion that only slept returns and flows through register -&gt; verify_writes -&gt; open_gate -&gt; approve -&gt; publish. This fixes BOTH faces: the run no longer sticks in terminal FAILED (no false 'no artifact registered'), and the gate Approve works because the workflow is still alive. (3) register_phase_result_core clears takeover_flag on a successful late report (un-parks). (4) New abandon_run workflow signal + orchestration.takeover.abandon_stalled_run, wired into the run-level /runs/{id}/take-over/ endpoint, so an explicit human takeover ('Take over manually' / 'Reconnect &amp; re-run') ends the still-waiting run terminally (no lingering workflow). (5) UI: 'stalled' renders as 'Parked for takeover' (RunConsole) and OfflineTakeover recognizes it + explains auto-reconcile. Tests (test_phase_dispatch): STALLED park, late-report reconcile clears the flag, abandon-only-when-parked, offline-then-abandoned + recovers-after-takeover (both against real Temporal). Files: backend/apps/runs/models.py, backend/apps/runs/migrations/0006_run_stalled_status.py, backend/orchestration/{workflows,activities,takeover}.py, backend/api/views.py, frontend/src/features/lifecycle/RunConsole.tsx, frontend/src/features/observability/OfflineTakeover.tsx.</t>
   </si>
   <si>
     <t>EPIC: Multi-repo work-item assignment (Hybrid Option C) - agent proposes a repo per work item, human confirms/overrides at the Task Breakdown gate, then implementation routes each task to its repo</t>
@@ -1503,10 +1536,7 @@
     <t>Multi-repo infra (WorkItem.repo FK, repo-scoped context, repo_topology, per-repo manifest, build routing on work_item.repo) exists, but nothing lets Task Breakdown assign a repo, nor a user set/override it - so multi-repo routing was impossible end-to-end.</t>
   </si>
   <si>
-    <t>Open - build in order A1-&gt;A4, B1-&gt;B3, C1, E1, then D1 verify. Backward-compatible: repo_id optional, single-repo unchanged.</t>
-  </si>
-  <si>
-    <t>In Progress</t>
+    <t>Fixed / validated end-to-end (2026-07-15/16). Multi-repo Hybrid Option C proven live: TASK-001 built on SpendLogTest-1-backend, 08 review + 07&lt;-&gt;08 remediation loop ran, merge gate approved, squash-merged to main, WorkItem -&gt; done; multi-repo routing, per-repo PRs and single-repo backward-compat all confirmed. All decomposed sub-tasks A1-E1 complete.</t>
   </si>
   <si>
     <t>A1: get_context does not return the project's repository list for project-level/planning runs - only repo_topology + the single scoped repo. Task Breakdown can't see the repos to assign them</t>
@@ -1683,7 +1713,7 @@
     <t>Role is optional on the model; UI may not surface it.</t>
   </si>
   <si>
-    <t>Open - verify in the running app; add the role field if absent.</t>
+    <t>Verified working — no code change needed. The live 'Add repository' form captures each repo's Role (backend/frontend/infra) via a real selector, sends it to the backend, and persists it on Repository.role (shown back as a chip). Auto-assign keys off this role correctly. Closed as verified.</t>
   </si>
   <si>
     <t>C1: wire 'Approve assignment &amp; continue' as the Task Breakdown gate decision - approving locks the repo assignments</t>
@@ -1758,7 +1788,7 @@
     <t>The code-host connect form predates multi-repo. The 'Repository' field is the connection's default/fallback repo, but is not labeled as such, so on a multi-repo project it looks like you must pick one repo.</t>
   </si>
   <si>
-    <t>Open - P2, team to address later. Relabel to 'Default repository (optional)'; add a hint that ONE token must reach ALL of the project's repos (a classic PAT with repo scope, or a fine-grained token listing each repo); optionally list the project's repos + connected status inline so it's clear all are covered.</t>
+    <t>The code-host connect form's single 'Repository' field (which read as single-repo on multi-repo projects) is now labelled 'Default repository', made OPTIONAL, and carries a hint: 'Each build targets its own repo; this is only a fallback default. The token must have access to ALL repos in this project.' The connection is tenant-wide and each build already targets its work-item repo, so Save no longer gates on this field. Backend catalog + frontend render change.</t>
   </si>
   <si>
     <t>Project topology auto-derives from repo count (2=split, 3+=multi) and overrides the user's explicit 'Multi-repo' choice; the create form offers only Single/Multi (2 options) while the model has 3 (single/split/multi)</t>
@@ -1950,7 +1980,7 @@
     <t>Same root cause as S.No 112 (connectors authenticate from the server .env, not per-tenant DB creds). Phase A did only the codehost because it was the build-workflow blocker. The Atlassian connectors also need email + site_url, which are NOT in the connect form's catalog yet, so this is a larger change (catalog + form fields + config wiring) - hence deferred.</t>
   </si>
   <si>
-    <t>Open - follow-up to Phase A. Plan: (1) add email/site_url (or equivalent) fields to the Atlassian vendors in catalog.py + the connect form; (2) change _atlassian_config to take the conn and decrypt api_token + read email/site_url from scopes; (3) same decrypt-and-use for Figma access_token and Xray client_id/client_secret; (4) keep the settings fallback for back-compat; (5) tests per connector + a two-tenant isolation test. Not blocking now - SpendLog-1 is sor=internal with no non-codehost connections configured.</t>
+    <t>Phase B done (extends S.No 74/112). The remaining connectors — Atlassian Confluence/Jira, Figma, Xray — now authenticate with the tenant's own stored credentials on ANY worker, not the server .env. Atlassian needed a new 'Atlassian account email' field on the Confluence/Jira connect form (basic auth = email + token); the site URL is normalised to the bare site. Per-field .env fallback retained. Config tests added.</t>
   </si>
   <si>
     <t>Blocking code review silently 'passes' (fail-OPEN): the 07&lt;-&gt;08 remediation loop reads blocking findings ONLY from the json verdict block in the 08 agent's FINAL message. When the agent's final message is prose (its machine-readable json block missing / not last / delivered via a separate event) the platform parses 0 findings, counts 0 blocking, SKIPS remediation and opens the merge gate on an unreviewed downgrade.</t>
@@ -2020,6 +2050,9 @@
 </t>
   </si>
   <si>
+    <t>FIXED (2026-07-15). agents/06_task_breakdown/agent.md: added a 'Writing standard' requiring every Epic/Story/Task Description + Acceptance Criterion to be plain-language-with-technical-nuance, detailed and self-contained enough that a developer can implement by reading it ALONE (behaviour, inputs/outputs, states, edge cases), with concrete hand-verifiable acceptance criteria and no bare placeholders; modelled the standard in all three template placeholders. Improvement flows to the Work Items board + artifact previews automatically. Test: test_agents_migration.test_task_breakdown_descriptions_and_ac_are_humanized. Per team decision the blast radius today was 06 only; the SAME defect in 02/09/00c/04/03/10 is logged as S.No 121-126 (register-condition per audience: technical-humanized for testing/security, plain+nuance for the rest) and NOT fixed this session.</t>
+  </si>
+  <si>
     <t>In the work items board when clicked on either epic or user story it shows children(3 or 4), instead when clicked on the childern it should show those tasks</t>
   </si>
   <si>
@@ -2028,7 +2061,475 @@
 Note: The same issues applies to the internal artifact content when the user clicked on the preview. You must read all the phase agents to identify what are all the artifacts it generates and how they are represented as names or disply or written.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixed (session 2026-07-15). Report-timeout takeover is now NON-terminal and reconcilable. (1) New Run.Status.STALLED (runs migration 0006) replaces terminal FAILED on timeout: mark_phase_takeover_core parks the run as STALLED + sets the WorkItem takeover_flag. (2) AgentRunWorkflow no longer returns on timeout: it marks the soft takeover then KEEPS waiting for the report, so a companion that only slept returns and flows through register -&gt; verify_writes -&gt; open_gate -&gt; approve -&gt; publish. This fixes BOTH faces: the run no longer sticks in terminal FAILED (no false 'no artifact registered'), and the gate Approve works because the workflow is still alive. (3) register_phase_result_core clears takeover_flag on a successful late report (un-parks). (4) New abandon_run workflow signal + orchestration.takeover.abandon_stalled_run, wired into the run-level /runs/{id}/take-over/ endpoint, so an explicit human takeover ('Take over manually' / 'Reconnect &amp; re-run') ends the still-waiting run terminally (no lingering workflow). (5) UI: 'stalled' renders as 'Parked for takeover' (RunConsole) and OfflineTakeover recognizes it + explains auto-reconcile. Tests (test_phase_dispatch): STALLED park, late-report reconcile clears the flag, abandon-only-when-parked, offline-then-abandoned + recovers-after-takeover (both against real Temporal). Files: backend/apps/runs/models.py, backend/apps/runs/migrations/0006_run_stalled_status.py, backend/orchestration/{workflows,activities,takeover}.py, backend/api/views.py, frontend/src/features/lifecycle/RunConsole.tsx, frontend/src/features/observability/OfflineTakeover.tsx.</t>
+    <t>FIXED (2026-07-15) - FULL blast radius + Part C (team-approved re-scope). (1) Artifact.title field + migration 0003_artifact_title (nullable, backward-safe). (2) register_artifact/update_artifact gain a title param, plus MCP server + companion wrappers, tool docstrings say 'ALWAYS pass a title'. (3) Part C-1 versioning-collision FIXED: version scoped by (project,phase,type,title) when titled, so per-item siblings (adr/test_case/security_finding/code/code_review/test_report) each start v1 instead of falsely superseding; untitled/singletons keep old behaviour. (4) Platform code/code_review get titles (WI key). (5) Serializers/consumers: DRF ArtifactSerializer + MCP _artifact/_lean_ref + preview payload + traceability node + dashboard + publish title expose/prefer title. (6) Frontend: new artifactLabel(title,type) helper (falls back to humanized type) in Artifacts registry list+search, preview H1/row, Traceability node (was raw type), Export/Publish. (7) 7 agents 04/05/07/08/09/09b/10 author human titles (Wireframe - Login Page, ADR-003 - Event Sourcing, TC-014 - ...). (8) Part C-2 ContractsDrift FIXED: no JSON.stringify dump (humanized scalar summary); DriftRecordSerializer enriches impacted with node_title+repo_name (batched) so no raw UUIDs. Wireframe STATES stay a separate label axis by design. Tests: test_mcp_platform_state (title + per-item independent versions), test_agents_migration (06 + per-item titles), test_review_dispatch/test_api_contract green; frontend tsc clean; ruff clean. Migration NOT yet applied to shared cloud DB - held for a coordinated make migrate (nullable=back-compat).</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>Requirements agent (02) authors user stories, functional requirements, acceptance criteria and NFRs too technically/formally for its reviewer. Same defect class as S.No 118 (06 task breakdown): the content is engineer/QA-precision only with no human-readability bar, yet the Product Owner reviews it. HUMANIZATION REGISTER for the fix = PLAIN LANGUAGE retaining the technical nuance (broader audience: PO + developer).</t>
+  </si>
+  <si>
+    <t>Investigation (session 2026-07-15) edge-case sweep of all 16 phase agents for the S.No 118 pattern. 02 is the closest structural analog to 06.</t>
+  </si>
+  <si>
+    <t>Agents / 02 Requirements / content humanization</t>
+  </si>
+  <si>
+    <t>Quality bar is 'a QA engineer can execute without a follow-up question' (agents/02_requirements/agent.md:10); FR format is formal SHALL boilerplate (:115); acceptance criteria are bare BDD stubs (:85-97); user-story descriptions have no plain-language directive; reviewer is the Product Owner (:357). Related S.No 118, 120.</t>
+  </si>
+  <si>
+    <t>OPEN - NOT fixed this session. Team scoped today's fix to S.No 118 (06 task breakdown) only. Planned: add a plain-language-with-technical-nuance authoring bar to user-story descriptions, FR statements and acceptance criteria - mirror 06's assignment_rationale directive (:280) and the good patterns in 05_ux_design/12_deployment/08_code_review.</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>Testing agent (09) authors UAT scenarios FOR the Product Owner, plus defect reports and test-case descriptions, with an engineer-precision bar only. Same defect class as S.No 118. HUMANIZATION REGISTER for the fix = HUMANIZED-TECHNICAL (keep the technical register but make it clear and well-structured) - NOT plain language, because QA/UAT personnel must interpret the technical detail correctly; plain language would cause misinterpretation.</t>
+  </si>
+  <si>
+    <t>Investigation edge-case sweep. UAT is a business-verification event handed to a non-engineer, yet authored with two-engineer precision.</t>
+  </si>
+  <si>
+    <t>Agents / 09 Testing / content humanization</t>
+  </si>
+  <si>
+    <t>UAT scenarios authored for the PO (agents/09_testing/agent.md:483-494) and defect descriptions (:433-459) use a two-engineer precision bar (:212) with no readability directive for the PO-facing UAT. Test-case Expected Result/Description carry the same risk. Related S.No 118, 120.</t>
+  </si>
+  <si>
+    <t>OPEN - NOT fixed this session (team scope = 06 only). Planned: add a HUMANIZED-TECHNICAL clarity bar (structured, understandable, technical register retained) to UAT scenarios, defect reports and test-case descriptions - not plain language.</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>Intelligent Context Extractor agent (00c) authors the codebase_intelligence Executive Summary, health dashboard and module-documentation prose read by humans onboarding to a project, with no plain-language directive - jargon-prone. Same defect class as S.No 118. HUMANIZATION REGISTER = PLAIN LANGUAGE retaining technical nuance.</t>
+  </si>
+  <si>
+    <t>Investigation edge-case sweep.</t>
+  </si>
+  <si>
+    <t>Agents / 00c Context Extractor / content humanization</t>
+  </si>
+  <si>
+    <t>Agent 'writes the prose' (agents/00c_intelligent_context_extractor/agent.md:44; artifact spec :93-106) with no directive to keep it plain for onboarding readers. Related S.No 118, 120.</t>
+  </si>
+  <si>
+    <t>OPEN - NOT fixed this session (team scope = 06 only). Planned: add a plain-language-with-technical-nuance bar to the exec summary and module-doc prose.</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>Architecture agent (04) authors ADR Rationale/Context/Consequences prose and the architecture Executive Summary as human-read decision records, but only the Level-1 context diagram carries a 'readable by a non-technical stakeholder' bar - the ADR narrative and exec summary do not. Same defect class as S.No 118. HUMANIZATION REGISTER = PLAIN LANGUAGE retaining technical nuance.</t>
+  </si>
+  <si>
+    <t>Agents / 04 Architecture / content humanization</t>
+  </si>
+  <si>
+    <t>Context diagram must be 'readable by a non-technical stakeholder' (agents/04_architecture/agent.md:119) but ADR rationale (:373) and exec summary (:291) have no plain-language bar. Related S.No 118, 120.</t>
+  </si>
+  <si>
+    <t>OPEN - NOT fixed this session (team scope = 06 only). Planned: extend the existing non-technical-readability bar to ADR narrative fields and the exec summary.</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>PRD agent (03) is mostly well-humanized, but the per-feature ACCEPTANCE CRITERIA remain terse placeholders - the same artifact type flagged in S.No 118. HUMANIZATION REGISTER = PLAIN LANGUAGE retaining technical nuance.</t>
+  </si>
+  <si>
+    <t>Investigation edge-case sweep. Partially self-mitigated (strong readability directives elsewhere).</t>
+  </si>
+  <si>
+    <t>Agents / 03 PRD / content humanization</t>
+  </si>
+  <si>
+    <t>Strong readability directives overall (agents/03_prd/agent.md:15,76,354) but per-feature acceptance criteria are terse placeholders (:224-227). Related S.No 118, 120.</t>
+  </si>
+  <si>
+    <t>OPEN - NOT fixed this session (team scope = 06 only). Planned: apply the same detailed, plain-language-with-nuance bar to per-feature acceptance criteria.</t>
+  </si>
+  <si>
+    <t>126</t>
+  </si>
+  <si>
+    <t>Security agent (10) authors the Executive Summary and finding Impact statements that reach stakeholders with no plain-language bar. Same defect class as S.No 118. HUMANIZATION REGISTER = HUMANIZED-TECHNICAL for findings (security engineers must read the technical detail correctly); the stakeholder exec summary may be plain-language-with-nuance.</t>
+  </si>
+  <si>
+    <t>Investigation edge-case sweep. Primary audience is technical; remediation guidance is already appropriately specific.</t>
+  </si>
+  <si>
+    <t>Agents / 10 Security / content humanization</t>
+  </si>
+  <si>
+    <t>Exec summary and finding Impact (agents/10_security/agent.md:339-340,395-398) reach stakeholders without a readability bar. Related S.No 118, 120.</t>
+  </si>
+  <si>
+    <t>OPEN - NOT fixed this session (team scope = 06 only). Planned: humanized-technical clarity bar on findings; plain-language-with-nuance on the stakeholder exec summary.</t>
+  </si>
+  <si>
+    <t>Merging an approved build fails with HTTP 405 because the pull request is still a draft (the final blocker)</t>
+  </si>
+  <si>
+    <t>After a human approves the merge gate, the platform tries to merge the build's PR but GitHub rejects it, so the work item never reaches 'done'.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Merge gate</t>
+  </si>
+  <si>
+    <t>1258d85</t>
+  </si>
+  <si>
+    <t>During the automated 07&lt;-&gt;08 review-and-fix loop the platform opens the build's pull request as a GitHub 'draft' PR (a draft blocks a premature human merge while review is still running). GitHub does not allow a draft PR to be merged - its merge API returns HTTP 405 (Method Not Allowed). So the moment a human approved the merge gate, the final merge step always failed. The work item got stuck at the very last step, never transitioned to done, and nothing downstream could complete. This was the single blocker stopping any build from finishing.</t>
+  </si>
+  <si>
+    <t>FIXED (commit 1258d85). Added a mark_ready_for_review step that takes the PR out of draft immediately before merging, which is the one legitimate moment to un-draft (gate already approved). merge_build_pr_core now does: get the PR; if it is not already merged and is still a draft, call codehost.mark_ready_for_review(pr_ref) which runs GitHub's markPullRequestReadyForReview GraphQL mutation and re-checks (short retries) that it un-drafted, then merge. Supporting additions: a graphql() helper (integrations/github/rest.py), a graphql_url property (config.py), and the CodeHost.mark_ready_for_review capability (capabilities.py + github/codehost.py). Regression test added in test_build_activities.py (draft PR is un-drafted before merge).</t>
+  </si>
+  <si>
+    <t>Reviewer gets 'no opened PR to review' during the fix-and-re-review loop (wrong code pointer picked)</t>
+  </si>
+  <si>
+    <t>During remediation the platform sometimes points the reviewer at an empty pre-PR placeholder instead of the real pull request.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Review loop</t>
+  </si>
+  <si>
+    <t>The helper that looks up a build's code artifact (_code_artifact) fetched 'the first matching artifact' with no defined ordering. A single work item can have more than one code-artifact row: an early placeholder the agent registers before the PR exists, and the real one that carries the pull-request reference (repo/number/url). With no ORDER BY, the database returned rows in an arbitrary order, so the code sometimes picked the early placeholder that has no PR link. The reviewer then had nothing to look at and reported 'no opened PR to review', which broke the remediation cycle.</t>
+  </si>
+  <si>
+    <t>FIXED (commit 1258d85). _code_artifact now orders artifacts by created_at and explicitly prefers the one whose external_ref is a real PR reference: it returns the first PR-ref-bearing artifact and only falls back to the earliest row if none carries a PR ref. Regression test added in test_build_activities.py (duplicate-code-artifact prefers the PR-ref pointer).</t>
+  </si>
+  <si>
+    <t>A genuinely 'Approved' code review is wrongly blocked by the fail-closed review guard (false positive on a resolved finding ID)</t>
+  </si>
+  <si>
+    <t>The safety guard that blocks bad code mis-reads an approved review and rejects it, stalling the pipeline for no real reason.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Review guard (S.No 114 guard)</t>
+  </si>
+  <si>
+    <t>a2deeae</t>
+  </si>
+  <si>
+    <t>The review guard is deliberately 'fail-closed': if a review's prose looks like it demands changes but the structured verdict does not clearly say so, it blocks - to stop bad code slipping through. The old prose matcher (_looks_blocking) scanned the entire review text for blocking-sounding words. An APPROVED review referenced an already-RESOLVED finding by its ID (for example 'REM-W1'), and the matcher saw that mention and concluded the review was demanding changes. Result: a legitimately approved review was blocked and the build could not proceed - a false positive that halted good work.</t>
+  </si>
+  <si>
+    <t>FIXED (commit a2deeae). Rewrote parse_and_guard to trust a present, structured APPROVED verdict. Added _verdict_demands_changes(): a verdict is treated as demanding changes only when a verdict is actually present AND its status matches a negative pattern (change/reject/denied/blocked/fail, via _NEGATIVE_STATUS regex). The loose prose scan is now only a fallback used when there is NO structured verdict at all. Net effect: an approved verdict is honoured even if its prose happens to mention resolved finding IDs, while a review that truly downgrades still fails closed. Regression tests added in test_review_dispatch.py (trusts approved verdict with resolved REM ids; in-JSON downgrade still fails closed).</t>
+  </si>
+  <si>
+    <t>When the secret scanner blocks a push, the failure is invisible - only a bare count is shown, not what/where</t>
+  </si>
+  <si>
+    <t>A blocked hardcoded secret produces a silent 'build failed' with just a number; nobody can tell which secret, file or line.</t>
+  </si>
+  <si>
+    <t>Companion / Pre-push secret scan</t>
+  </si>
+  <si>
+    <t>52533c4</t>
+  </si>
+  <si>
+    <t>Before pushing code the companion (the worker on the developer machine) scans the changed files for hardcoded secrets (passwords, API keys, tokens, private keys). When it finds one it correctly blocks the push and reports the build as failed - but it only reported a bare count ('N finding(s)'). It did not surface which secret type, which file, or which line, and it then tore down the temporary work folder, so the evidence was gone. Operators saw 'build failed' with no way to know why or how to fix it, making the block undiagnosable.</t>
+  </si>
+  <si>
+    <t>FIXED (commit 52533c4). The companion now prints a redacted summary to its own terminal ('[companion] SECRET SCAN BLOCKED push (N finding(s)) - branch NOT pushed') listing each finding as '[kind] path:line - preview', and the same redacted detail travels in the build.failed reason so it also appears in the platform run console. Only the already-redacted preview is shown - never the raw secret value - and the list is capped at 8 findings with a '(+N more)' tail so the message stays bounded. Added the _format_secret_findings helper (runner/companion/runner.py) and regression tests in test_companion_runner.py (redacted findings surface; cap at 8).</t>
+  </si>
+  <si>
+    <t>The code-review result (code_review artifact) cannot be opened or read from the web UI</t>
+  </si>
+  <si>
+    <t>The 08 review report is produced and registered but there is no view/link in the product to read it.</t>
+  </si>
+  <si>
+    <t>UI / Review experience</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>The 08 review agent produces a code_review artifact holding the review findings and verdict, and the platform registers it as an artifact (pointer + provenance). However the web interface offers no view or link that opens the artifact body, so a human reviewer or manager cannot actually read the review inside the product - they would have to query the database or dig through logs. This undermines the human review gate: the gate exists but the evidence behind it is not surfaced to the person approving.</t>
+  </si>
+  <si>
+    <t>Verified already fixed — no code change needed. Cross-checked against a live run: the code_review artifact IS registered with a rendered report body (the companion uploads the .md to S3 — confirmed a ~22 KB report object exists for the latest run), and the generic artifact preview reads it, so the report opens and reads in the UI. The earlier 'no body' analysis looked only at the platform-side fallback registration and missed the companion upload. Closed as verified.</t>
+  </si>
+  <si>
+    <t>The 'sdlc/build' commit status is set to 'pending' when the PR opens and is never updated - it stays pending forever (latent)</t>
+  </si>
+  <si>
+    <t>A dormant flaw: the build commit status posted to GitHub is never moved off 'pending', which will block merges if branch protection ever requires it.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Commit status reporting</t>
+  </si>
+  <si>
+    <t>build_activities.py:140</t>
+  </si>
+  <si>
+    <t>When the build PR is opened, the platform posts a GitHub commit status with context 'sdlc/build' and state 'pending' against the head commit (build_activities.py line 140, best-effort - exceptions are swallowed). Nothing anywhere later updates that status to 'success' or 'failure'. So every build's commit shows the 'sdlc/build' check stuck on pending indefinitely. It is dormant today only because no branch-protection rule on the repo currently requires the 'sdlc/build' context to be green before merging. The day someone enables such a required check, merges will be blocked forever because the status can never reach success - a latent time-bomb, and misleading status UI in the meantime.</t>
+  </si>
+  <si>
+    <t>OPEN - not fixed this session. Recommended fix: complete the status lifecycle. Set 'sdlc/build' to 'success' once the build+review pass (or at merge), and to 'failure' on the mark_build_failed / secret-block / merge-failed paths, using the same head SHA. Keep it best-effort (do not fail the saga on a status-post error), but ensure a terminal state is always posted so the check does not dangle. Acceptance: after a run reaches a terminal outcome, the commit's 'sdlc/build' status reflects success or failure, never a permanent pending.</t>
+  </si>
+  <si>
+    <t>The companion crashes hard (fatal, exit 1) when the build agent errors, instead of failing gracefully and reporting back</t>
+  </si>
+  <si>
+    <t>If the AI build agent fails, the whole companion worker dies and needs a manual restart, stalling the build.</t>
+  </si>
+  <si>
+    <t>Companion / Build execution resilience</t>
+  </si>
+  <si>
+    <t>When the build agent (the Claude Agent SDK run inside the companion) exits with an error, the exception propagates all the way up and the companion process terminates fatally (Command failed / exit code 1). Because the companion runs one build at a time and is a long-lived poller, a single agent error takes the whole worker down: it stops polling, the current run is left dangling (claimed but not reported), and a human has to notice and restart the companion before any further work can proceed. Observed repeatedly this session (e.g. when a mid-build backend restart broke the agent's MCP calls, and when an environment/dependency mismatch made the agent exit).</t>
+  </si>
+  <si>
+    <t>Fixed (2026-07-16). runner/companion/daemon.py _run_build now catches a generic build-agent error, posts a failed BuildReport (status=failed + message) to /api/runner/builds/&lt;run&gt;/report/, and keeps polling (mirrors the plan/review path _run_engine_phase) instead of the exception propagating out of serve and killing the long-lived companion. EngineAuthError still fail-closes (explicit re-raise) so a subscription/auth halt is never downgraded to a per-build failure. Tests: test_companion_daemon (agent-error reported + no crash; auth-error still halts).</t>
+  </si>
+  <si>
+    <t>A worker can deadlock a job by self-renewing its own claim while making no progress (stuck job never released)</t>
+  </si>
+  <si>
+    <t>A worker keeps renewing its hold (heartbeat) on a job it isn't actually advancing, so the job sits claimed forever and nothing else can take it.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Claim + heartbeat (S.No 111)</t>
+  </si>
+  <si>
+    <t>Jobs are handed to a worker via a claim, and a heartbeat (S.No 111) periodically renews that claim so the platform knows the worker is alive. The problem: the heartbeat renews the claim based on the worker still running, not on the work actually progressing. If the worker gets wedged (e.g. the agent hangs, or a step is stuck) but the heartbeat thread keeps ticking, the claim is renewed indefinitely. The job stays 'claimed', the report-timeout takeover cannot fire (the claim looks fresh), and no other worker can pick it up - a silent deadlock that only a human notices. Seen this session as the 'companion claimed but never built' deadlock.</t>
+  </si>
+  <si>
+    <t>Fixed (2026-07-16). Cross-verified first: _renew_claims_for renewed the claim on process liveness alone (no progress signal, no cap), so a wedged-but-heartbeating worker held its claim until only the 2h workflow report-timeout (S.No 89) freed it. Fix: backend/api/runner_views.py stamps first_claimed_at at each claim (reset per claim, never touched by heartbeat) and MAX_CLAIM_AGE=60min caps renewal - past it the heartbeat stops renewing so the lease ages out and the run is recoverable well before the 2h backstop. Cap set above the longest legit build (&lt;60min, team-confirmed) so a healthy long build is never capped (no S.No 111 regression). Note: a companion progress-signal is the fundamentally optimal fix (distinguishes wedged-vs-working at any duration) - logged as the future upgrade if builds ever exceed ~1h. Tests: test_phase_dispatch (cap stops renewal; young claim still renews).</t>
+  </si>
+  <si>
+    <t>Dependency version skew: pinned claude-agent-sdk / anyio in the repo are behind what the runtime actually needs</t>
+  </si>
+  <si>
+    <t>The project's pinned library versions lag what the running machine requires; fixed by hand on the machine but not locked in the repo, so it will break for the next person.</t>
+  </si>
+  <si>
+    <t>Companion / Dependency management</t>
+  </si>
+  <si>
+    <t>The companion depends on claude-agent-sdk, which in turn requires a newer anyio (the anyio.open_process 'user' keyword arrives in anyio 4.5.0; claude-agent-sdk 0.1.72 needs it). The repo's pins were stale (an old claude-agent-sdk pin and no floor on anyio), so a fresh environment installed anyio 4.4.0 and the agent crashed with "anyio.open_process() got an unexpected keyword argument 'user'". This session it was worked around by manually upgrading anyio on the host (pip install -U 'anyio&gt;=4.5' -&gt; 4.14.2), but that fix lives only on this machine - the repo still pins the broken combination, so the next developer or a rebuilt container will hit the same crash.</t>
+  </si>
+  <si>
+    <t>OPEN - not fixed this session (env-patched only). Recommended fix: pin the correct, mutually compatible versions in the repo lockfile/requirements - bump claude-agent-sdk to the version actually in use and add an explicit anyio&gt;=4.5 floor - then rebuild the companion/worker images from the lockfile so a clean install reproduces the working environment. Acceptance: a from-scratch install (no manual pip upgrades) runs a build without the open_process 'user' error.</t>
+  </si>
+  <si>
+    <t>Build branches are merged without first being updated against their base, causing merge conflicts at the gate</t>
+  </si>
+  <si>
+    <t>The platform merges a feature branch without rebasing/updating it against the current base, so it hits conflicts (mergeable_state=dirty) and the merge fails.</t>
+  </si>
+  <si>
+    <t>When the merge gate is approved, the platform merges the feature branch as-is. It never updates the branch against the latest base first. If the base has moved on since the branch was cut - which is normal in a multi-developer repo - the PR can be in a conflicted state (GitHub mergeable_state = 'dirty'), and the merge API then returns HTTP 405 just like the draft case. This session WI-29 hit exactly this: an add/add conflict on frontend/.env.example left the PR dirty and the merge failed; it had to be resolved by hand. The pipeline has no step to bring a branch up to date with its base before attempting the merge.</t>
+  </si>
+  <si>
+    <t>Fixed (2026-07-16). The merge gate merged the feature branch as-is, so a base that moved since the branch was cut left the PR mergeable_state=dirty and the GitHub merge API returned a raw 405. Fix: integrations/types.py PullRequest gains mergeable/mergeable_state; github/codehost.py adds update_branch (GitHub Update-branch; swallow 422 already-up-to-date) + ensure_mergeable (bounded re-read for GitHub's async mergeability); build_activities.py merge_build_pr_core now, before merging: if 'behind' -&gt; update branch against base then re-check; if 'dirty'/not mergeable -&gt; fail fast (non-retryable ApplicationError) with a clear 'merge conflict - needs manual resolution' reason instead of a cryptic 405; merges only when mergeable. Idempotent behind the existing 'if not pr.merged' guard. Tests: test_build_activities (behind-&gt;update-&gt;merge; dirty-&gt;clean fail, never merged). Reason surfacing verified in live test: the classified reason reaches the user via the S.No 139 ActivityError-cause unwrap (build_workflow uses build_types.failure_reason), since str(ActivityError) is the opaque "Activity task failed".</t>
+  </si>
+  <si>
+    <t>Planning overlap: two separate work items are both told to create the same file (frontend/.env.example), guaranteeing a conflict</t>
+  </si>
+  <si>
+    <t>TASK-003 and TASK-005 each create frontend/.env.example, so when both build they collide - a work-breakdown/planning defect.</t>
+  </si>
+  <si>
+    <t>Planning / Work-item decomposition</t>
+  </si>
+  <si>
+    <t>Two independently-dispatched work items (TASK-003 and TASK-005) were each planned to create the same file, frontend/.env.example. When both branches are built and then merged, they produce an add/add conflict on that file - there is no shared ownership or de-duplication in the planning step. This is the upstream cause of the WI-29 merge conflict (S.No 136): the pipeline had no branch-update step to catch it, but the conflict should not have been planned in the first place. It points to a gap in how the planner assigns file ownership across parallel work items.</t>
+  </si>
+  <si>
+    <t>Not reproducible / not a bug — verified against stored work-item data. TASK-003 creates the FRONTEND .env.example (frontend repo); TASK-005 is a backend SQLAlchemy/Alembic task (backend repo) — different files, different repos, no collision. The likely confusion: TASK-002 (backend .env.example) and TASK-003 (frontend .env.example) are two correctly-separate files that merely share a name. Closed.</t>
+  </si>
+  <si>
+    <t>Two developers share a single enrollment record, risking incorrect work attribution and tenant isolation</t>
+  </si>
+  <si>
+    <t>Two devs point at the same enrollment identity (32db7f5f), so runs/work may be attributed or isolated to the wrong person.</t>
+  </si>
+  <si>
+    <t>Tenancy / Enrollment identity</t>
+  </si>
+  <si>
+    <t>enrollment 32db7f5f</t>
+  </si>
+  <si>
+    <t>During testing it was found that two different developers are operating under the same enrollment record (enrollment id 32db7f5f, under tenant 212395b8). Enrollment is meant to identify a single developer's participation in a project; sharing one record between two people means their runs, claims and attribution can be conflated, and any per-developer isolation or accounting keyed on enrollment is wrong. It also muddies debugging (whose companion claimed what) and could let one developer's actions appear under the other's identity.</t>
+  </si>
+  <si>
+    <t>OPEN - not fixed this session (flagged during testing). Recommended fix: give each developer their own enrollment record under the tenant/project, and ensure the companion is launched with the correct per-developer enrollment/credentials so claims and events attribute to the right person. Audit existing runs that used the shared enrollment. Acceptance: each developer has a distinct enrollment and their runs attribute correctly.</t>
+  </si>
+  <si>
+    <t>Build failures don't explain why - most failures show a generic 'build failed' or a raw, cryptic error instead of a clear reason</t>
+  </si>
+  <si>
+    <t>When a build fails for reasons other than a blocked secret (token/permission error, merge conflict, agent error, empty build), the platform shows 'build failed' or a raw exception string, not a plain classified reason.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Failure observability</t>
+  </si>
+  <si>
+    <t>The build.failed reason is populated inconsistently across the different failure paths (build_workflow.py). A companion report failure falls back to the generic literal 'build reported failed' when no message is set. Remediation-exhausted is the hardcoded 'remediation cycles exhausted'. The PR/gate-setup and merge paths embed a raw Python/Temporal exception string ('pr/gate setup failed: {exc}', 'merge failed: {exc}') - so a token-permission (403) error or a merge conflict (405) is technically present but buried in a cryptic stack string, not classified as 'token permission issue' or 'merge conflict'. Only the secret-scan case (S.No 130) was made human-readable. Net effect: for most failure kinds an operator sees 'build failed' with no actionable reason and must dig through logs to triage.</t>
+  </si>
+  <si>
+    <t>Fixed (2026-07-16). build.failed reasons were inconsistent (bare 'build reported failed', hardcoded 'remediation cycles exhausted', raw exception strings 'merge failed: {exc}') AND - a hidden gap - the EventSerializer never surfaced the 'reason' payload key, so the run console showed only 'Build failed'. Fix: build_activities.py classify_build_failure maps every failure path to a plain-language classified reason (merge conflict / permission-403 / remediation exhausted / empty build / agent error; the good S.No 130 secret-scan message passes through); mark_build_failed_core writes it to run.outputs.error (where the run console reads the failure line) and the build.failed event; api/serializers.py adds 'reason' to the event message keys. Composes with S.No 136 (single canonical 'merge conflict' reason). Tests: test_build_activities (classifier mappings; reason on run.outputs.error). CORRECTION (same session, caught by live test): the workflow now UNWRAPS the ActivityError .cause via build_types.failure_reason so the classifier sees the real message (Temporal str(ActivityError)="Activity task failed" otherwise hides the 405/422/conflict); AND open_build_pr_core fails an EMPTY build fast (non-retryable ApplicationError "empty build: no changes") instead of a cryptic 422 after 3 retries - an empty build still FAILS (clear reason), it does not auto-succeed. Tests: failure_reason unwrap + empty-build fast-fail + classifier mappings.</t>
+  </si>
+  <si>
+    <t>No human action to resolve a non-mergeable / redundant / failed WorkItem: a task can only reach 'done' via a successful automated build+merge. A build that fails (empty/redundant build, or a merge conflict needing manual resolution) leaves the WorkItem stuck at in_progress with no product path for a human to mark it done, skip it, or close it as redundant.</t>
+  </si>
+  <si>
+    <t>Surfaced 2026-07-16 while testing S.No 136/139: TASK-002 (redundant with TASK-001) produced an empty build that correctly FAILED with 'Empty build: no changes to commit'. The WorkItem then sits at in_progress with the branch/draft PR left in place, and the only offered action is Retry - which re-fails for a genuinely redundant task. A human can freely trigger the NEXT task (tasks are independent unless depends_on) but cannot close/resolve the failed one. Today the only ways to reach done are the happy-path orchestrator flow or an admin DB state change.</t>
+  </si>
+  <si>
+    <t>Work Items / Build recovery UX</t>
+  </si>
+  <si>
+    <t>backend/apps/workitems/models.py (State: proposed/accepted/in_progress/in_review/blocked/done, no transition validation); backend/api/serializers.py WorkItemPatchSerializer (state NOT writable) + read_only state; backend/api/views.py WorkItemViewSet (trigger/build/take-over/lifecycle - no transition/mark-done action); mcp_platform_state/tools.py transition_work_item (any-&gt;any, internal only); frontend RunConsole.tsx (Retry only) / WorkItemTask.tsx (done is display-only) / OfflineTakeover.tsx</t>
+  </si>
+  <si>
+    <t>WorkItem.state is read-only on the API (excluded from WorkItemPatchSerializer; read_only on the read serializer) and mutated ONLY internally by the orchestrator (successful build+merge / gate / reject / takeover). No human-facing transition/mark-done/close/skip action or endpoint exists; the frontend offers only Retry / Trigger phase / manual takeover (sets takeover_flag, not state). transition_work_item allows any-&gt;any but is unexposed to users.</t>
+  </si>
+  <si>
+    <t>OPEN - proposed: add a GATED human action + API endpoint to move a WorkItem to a terminal state outside the happy path (e.g. 'Mark done', 'Close as redundant / won't-do', or 'Skip'), surfaced on the Work Items board + task page, with an audit Event. Decide whether to reuse 'done' or add a distinct terminal state (e.g. 'closed'/'cancelled') to distinguish completed-by-build from human-closed; guard with role/permission. Related S.No 76 (no task-edit UI; state not editable).</t>
+  </si>
+  <si>
+    <t>Merge gate can't recover from a conflict without redoing the whole build. TWO related enhancements (logged together): (ENH-2, IMPLEMENT NOW) Merge-only retry / re-openable merge gate - when a merge hits a conflict, PAUSE at the merge step and let the user retry the merge after fixing the conflict, WITHOUT re-running the whole build. (ENH-1, FUTURE / only if needed) Reconcile the Run status on an EXTERNAL merge - when a user merges the PR by hand in GitHub, also flip the Run from failed to done (today the webhook updates the WorkItem + artifact but leaves the Run 'failed').</t>
+  </si>
+  <si>
+    <t>Today a merge conflict marks the ENTIRE build failed and ends the workflow, so finishing means re-running everything (AI re-writes the code, re-reviews, re-opens the PR) just to retry one merge. ENH-2 fixes this: keep the build paused at the merge gate; after the user resolves the conflict in GitHub they press Merge/Approve again and the platform completes the merge through its OWN flow (run + gate + work-item all stay correct automatically, no rebuild). ENH-1 covers a DIFFERENT path - the user merges by hand in GitHub instead of letting the platform do it; then the platform only learns via webhook (S.No 88) and today leaves the Run status stale. TEAM PLAN (2026-07-16): implement ENH-2 now; keep ENH-1 for future - it overlaps S.No 88 and is only needed if users merge OUTSIDE the platform. If ENH-2 is used, ENH-1 is largely unnecessary. Same 'soft, reconcilable' idea as the S.No 89 fix, applied to merge conflicts.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Merge gate recovery</t>
+  </si>
+  <si>
+    <t>backend/orchestration/build_workflow.py (merge gate + ActivityError-&gt;mark_build_failed is TERMINAL on a conflict); backend/orchestration/build_activities.py merge_build_pr_core (S.No 136 dirty-&gt;fail); backend/integrations/webhooks.py _reconcile_pull_request (updates WorkItem+artifact on an external merge, NOT the Run); frontend Gates.tsx (merge gate) + RunConsole.tsx. Related: S.No 88 (external merge / missing webhook), S.No 89 (soft-reconcilable pattern), S.No 136 (conflict detection).</t>
+  </si>
+  <si>
+    <t>On a merge conflict the BuildWorkflow catches the ActivityError and calls mark_build_failed, which is TERMINAL - the workflow ends, so there is no live workflow to retry the merge and the merge-gate Approval is already spent. The only ways forward today are a full re-trigger (rebuilds from 07) or an external GitHub merge (needs the S.No 88 webhook, which also does not reconcile the Run status).</t>
+  </si>
+  <si>
+    <t>ENH-2 IMPLEMENTED &amp; VALIDATED LIVE (@ 66b70c8, + gate banner). A merge conflict is now NON-terminal: merge_build_pr detects a dirty PR and raises a typed MergeConflict; the BuildWorkflow catches it, RE-OPENS the merge gate (resets the approval to pending, records outputs.merge_conflict + a build.merge_conflict event) and waits — instead of failing the build. The user resolves the conflict in GitHub and approves again; the platform retries ONLY the merge (no rebuild, no re-review). Proven live on TASK-003 (run 1d1dd943): injected an add/add conflict on .env.example -&gt; approve -&gt; gate re-opened (once per remaining conflict) -&gt; resolved -&gt; approve -&gt; platform merged PR#1 (merge commit c1d7552a) -&gt; WorkItem done -&gt; run completed, with NO rebuild across retries. The merge gate now shows a warning banner explaining the conflict + retry (ApprovalSerializer.merge_conflict; shown ONLY on a re-opened merge gate, never other gates). ENH-1 (reconcile Run status on an EXTERNAL GitHub merge) remains FUTURE / optional — it overlaps S.No 88 and is only needed if users merge outside the platform, which ENH-2 makes largely unnecessary.</t>
+  </si>
+  <si>
+    <t>Backlog push to Jira: tasks never reach Jira — each Task is created with its Story as parent, which Jira rejects</t>
+  </si>
+  <si>
+    <t>During a live Jira push of the SpendLog-1 backlog, all 5 epics + 15 stories were created but 0 of 29 tasks landed. reconcile creates each task with parent = its story's Jira key; Jira rejects a standard Task parented to a Story (400 'Please select valid parent issue') — only Sub-tasks can live under a Story (Jira hierarchy: Epic &gt; Story/Task, and Epic &gt; Story &gt; Sub-task).</t>
+  </si>
+  <si>
+    <t>reconcile.reconcile_work_item mapped WorkItem.type 'task' -&gt; Jira 'Task' and set parent={key: story}. Jira does not allow a standard Task under a Story. Stories succeeded because Story-under-Epic via the parent field IS valid; tasks-under-stories are not.</t>
+  </si>
+  <si>
+    <t>TWO layered causes, both fixed. (1) REAL ROOT CAUSE: reconcile's idempotency guard 'if wi.external_ref' wrongly treated a repo-assigned task as already-reconciled. Multi-repo tasks carry external_ref.repo_assignment (the planner's repo pick, Option C) with NO SoR id, so on the live push every task was SKIPPED before reaching Jira (export showed created:0, reconciled:29, no error — not a Jira rejection at all). Fixed: the guard now checks for a real SoR key (external_ref.id), and the SoR ref is MERGED into external_ref so the repo_assignment is preserved. (2) HIERARCHY (latent, also fixed): once tasks reach Jira, a standard Task can't be a child of a Story, so a task with a reconciled story parent is created as a SUB-TASK under it (the project's real sub-task issue-type name, resolved via AtlassianTaskTracker.subtask_type_name() + cached), and a parentless task as a top-level Task. Validated live (Sub-task-under-Story create succeeds; Task-under-Story returns 400). Tests in test_reconcile: repo-assigned task not-skipped + repo_assignment preserved, subtask mapping, parentless task, per-item failure capture. NOTE: my first commit fixed only the hierarchy; the guard/repo_assignment fix (the true blocker) landed in the follow-up commit after the re-push showed created:0.</t>
+  </si>
+  <si>
+    <t>Backlog publish reports a green 'Published' while items silently fail to reach the system of record</t>
+  </si>
+  <si>
+    <t>The same Jira push showed 'Published — 49 work items reconciled (20 created)' even though 29 tasks failed. reconcile_backlog ran each item with no per-item error handling and the publish response/dialog surfaced only reconciled/created — so partial failures were invisible and the reconciled count over-reported what actually landed.</t>
+  </si>
+  <si>
+    <t>Integrations / Publish</t>
+  </si>
+  <si>
+    <t>reconcile_backlog processed items in a list comprehension with no try/except, and _publish_tasktracker + the ExportPublish dialog reported only reconciled/created counts — never failures. A partial push read as a full success.</t>
+  </si>
+  <si>
+    <t>reconcile_backlog now isolates each item in try/except: a single item's SoR rejection is recorded (logged as a workitem.reconcile_failed event + returned in a 'failed' list) and the run continues, instead of aborting or being swallowed. The publish API returns status 'partial' plus the failed items; the artifact stores a failed count; the ExportPublish dialog now shows 'Published with some failures — N created, M failed' + the first error, instead of an all-green success. Test added in test_reconcile (per-item failure captured; epic/story still land).</t>
+  </si>
+  <si>
+    <t>Secret scanner false-positives on hyphenated placeholders (e.g. change-me-...) in .env.example, blocking legitimate builds</t>
+  </si>
+  <si>
+    <t>The pre-push secret scan flagged an obvious placeholder value as a real secret, so the push was blocked and the build failed.</t>
+  </si>
+  <si>
+    <t>3c33554</t>
+  </si>
+  <si>
+    <t>The companion's pre-push secret scanner (runner/companion/guardrails.py) blocks a push when it finds anything that looks like a hardcoded secret. Its placeholder allow-list recognised the literal token 'changeme' but NOT the far more common hyphenated/underscored form 'change-me'. So a legitimate .env.example placeholder - JWT_SECRET=change-me-minimum-32-characters-long (36 chars, Shannon entropy 3.875) - was not recognised as a placeholder, tripped the generic high-entropy heuristic, and was flagged as a 'high_entropy_secret'. The push was blocked and the build failed. This is a FALSE POSITIVE: the value is an obvious placeholder, not a real secret. It blocked WI-32 and would block any task whose example env file uses the very common change-me convention. The build agent did nothing wrong - the scanner was too aggressive.</t>
+  </si>
+  <si>
+    <t>FIXED (commit 3c33554). Two changes in runner/companion/guardrails.py: (1) broadened the placeholder allow-list to cover change[-_ ]?me / replace[-_ ]?me / to-be-(changed|set|replaced|filled|generated) / secret-(here|goes) / dummy / sample / redacted, so hyphenated placeholders are recognised. (2) Committed template files (.env.example, *.sample, *.template, *.dist, *.tpl) now skip the generic entropy heuristic - placeholders are expected there - while STILL running the high-precision key-format patterns (AWS AKIA..., GitHub ghp_..., PEM private keys, JWT), so a real key shape pasted into an example file is still blocked. Regression tests in backend/tests/test_guardrails.py: the exact WI-32 value + change_me/replace-me variants pass clean; a real random token in real source still blocks; AWS/GitHub key shapes inside .env.example still block; non-template source keeps the full entropy scan. 12/12 scanner tests pass.</t>
+  </si>
+  <si>
+    <t>AI-engine build failures (usage/rate limit, agent CLI exit 1) show a raw, unreadable message instead of a clear reason</t>
+  </si>
+  <si>
+    <t>When the agent CLI fails (e.g. the Anthropic usage limit is reached) the run console shows 'Command failed with exit code 1 ... Check stderr output for details' - opaque and non-actionable.</t>
+  </si>
+  <si>
+    <t>Build pipeline / Failure observability + Companion</t>
+  </si>
+  <si>
+    <t>daemon.py:271</t>
+  </si>
+  <si>
+    <t>When the AI build agent fails to run - most commonly because the Anthropic usage/rate limit is reached, but also on any agent CLI non-zero exit - the companion's error handler (runner/companion/daemon.py ~line 271) captures only the engine driver's generic wrapper string and reports it verbatim: 'Command failed with exit code 1 (exit code: 1) / Error output: Check stderr output for details'. The platform's classify_build_failure (backend/orchestration/build_activities.py) does not recognise this signature, so the raw string passes straight through to the build.failed reason and the run console. The user sees an opaque error with no indication that the real cause was a usage limit and no guidance on what to do. This bit WI-32: the usage limit was hit during the cycle-2 remediation build and the console showed only 'Command failed with exit code 1'. Same defect class as S.No 139 (classified reasons) but for the engine/usage-limit failure path, which was not covered.</t>
+  </si>
+  <si>
+    <t>OPEN - Fix A planned this session (this row's owner). Two parts: (1) Companion (daemon.py): capture the agent process's stderr tail and put the actual cause in the report message instead of the placeholder 'Check stderr output for details'. (2) Platform (classify_build_failure): recognise engine / usage-limit / rate-limit signatures ('exit code 1', 'usage limit', 'rate limit', '429', 'overloaded', 'quota', 'Failed to start Claude Code') and map them to a plain-language reason, e.g. 'The AI engine hit its usage limit - the build stopped; retry when the limit resets.' NOTE: true resume-from-checkpoint on a transient failure (so a re-run continues from the last cycle instead of rebuilding) is tracked separately as S.No 147 and is owned by the other developer. Acceptance: a usage-limit failure shows a clear, non-technical reason naming the usage limit, not a raw exit-code string.</t>
+  </si>
+  <si>
+    <t>When the implementation of a Work Item is completed and give it away for the review agent - The review agent is doing its job and creating Remediation Work Items (if blocking or critical issues are present): The created Remediation Work Item Tasks are too technical and not humasined and high level</t>
+  </si>
+  <si>
+    <t>In Implementation Phase:
+1. The implementation agent should ask the user for any clarifications 
+2. The implementation agent should ask the user for edits: should the edits be manual edit or auto mode.
+Note: For this Enhancement of the agent, you must reason and discuss with the team and take their inputs and then proceed.</t>
+  </si>
+  <si>
+    <t>Build Phase</t>
+  </si>
+  <si>
+    <t>This is a recon and report back job:
+In the Bug fixing sesions of the SDLC APP the team conducted so far (Git History and This Bugs sheet is the core evidence): You Must recon each and every single fix that has been done so far which are directly or indirectly related to the Core - Agents - agent.md for all phases and report back based on the evidence - Do any of the agents need optimization?</t>
+  </si>
+  <si>
+    <t>SDLC Phases</t>
+  </si>
+  <si>
+    <t>Optimization/Enhancement</t>
+  </si>
+  <si>
+    <t>In Phases &amp; Runs Page:
+Currently all created Work Items are shown in a drop down but if the created work items count reaches huge number it would be difficult for the user to find his work item. Instead we will give him a search option in the drop down itself - this way he can search for his work item and use the drop down also.</t>
+  </si>
+  <si>
+    <t>In the Artifacts &amp; Traceability page:
+1. The artifacts names for Code review, PR - should have task title/name to identify easily instead of only WI-ID
+Note: See the reference image for clarity</t>
+  </si>
+  <si>
+    <t>When the user approved the gate for implementation pahse - The artifacts: Assumptions, Implementation task/WI are still in draft state not published.
+Note: See the reference image for clarity</t>
+  </si>
+  <si>
+    <t>The user should be able to edit the generated phase artifacts - Task Breakdown phase, requirements phase, PRD phase etc. Right now the edit artifacts capability is missing.</t>
+  </si>
+  <si>
+    <t>The team have observed that each phase execution (mainly the Build phases) of the SDLC app is taking too long to run. The team wants to know the exact reason behind this before brain storming how to optimize it better 
+Note: You must co-ordinate with the team about this</t>
+  </si>
+  <si>
+    <t>In the Integration Mechanism of the SDLC APP: Integrations are per tenant but the team strongly wants the integrations should be per projects not tenant.</t>
+  </si>
+  <si>
+    <t>In the integration page: 
+1. For any integration of a capability - Currently the user cannot edit the saved token but that should be possible
+2. THe user should test the integration connection first and then save the creds not the other way around.</t>
+  </si>
+  <si>
+    <t>In the SDLC APP Phases and Runs: After any phase (mainly Build Phase but applies to all phases) trigger is interrupted due to any error/issue, the user should be able to continue from that point rather than starting from beginning of that phase. 
+Note: This is a very user important fix - should be applied accurately.</t>
+  </si>
+  <si>
+    <t>Phases and Runs</t>
   </si>
 </sst>
 </file>
@@ -2872,7 +3373,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="13">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="16">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -2925,6 +3426,18 @@
     <v>12</v>
     <v>5</v>
   </rv>
+  <rv s="0">
+    <v>13</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>14</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>15</v>
+    <v>5</v>
+  </rv>
 </rvData>
 </file>
 
@@ -2952,6 +3465,9 @@
   <rel r:id="rId11"/>
   <rel r:id="rId12"/>
   <rel r:id="rId13"/>
+  <rel r:id="rId14"/>
+  <rel r:id="rId15"/>
+  <rel r:id="rId16"/>
 </richValueRels>
 </file>
 
@@ -4922,15 +5438,11 @@
       <c r="G61" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed on two fronts. (1) UI: the 'Other' free-text box no longer fails to appear when the agent labels an option with a letter prefix (e.g. 'd) Other') — the reveal now strips a leading enumerator before matching. Verified LIVE against the running app (served bundle). (2) Authoring: the ask_human tool contract now tells every phase agent to write ONE short plain-language question and put choices ONLY in the structured options, never inline them in the question text — stopping the duplicated-options / uppercase wall-of-text. Frontend + agent-contract change; regression test added.</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="I61" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="409.6">
@@ -4938,10 +5450,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>12</v>
@@ -4953,10 +5465,10 @@
         <v>13</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J62" s="2" t="s">
         <v>16</v>
@@ -4967,28 +5479,28 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J63" s="2" t="s">
         <v>16</v>
@@ -4999,28 +5511,28 @@
         <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J64" s="2" t="s">
         <v>16</v>
@@ -5031,28 +5543,28 @@
         <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J65" s="2" t="s">
         <v>16</v>
@@ -5063,28 +5575,28 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J66" s="2" t="s">
         <v>16</v>
@@ -5095,28 +5607,28 @@
         <v>66</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>16</v>
@@ -5127,28 +5639,28 @@
         <v>67</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J68" s="2" t="s">
         <v>16</v>
@@ -5159,28 +5671,28 @@
         <v>68</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="J69" s="2" t="s">
         <v>16</v>
@@ -5191,28 +5703,28 @@
         <v>69</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>16</v>
@@ -5223,28 +5735,28 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J71" s="2" t="s">
         <v>16</v>
@@ -5255,28 +5767,28 @@
         <v>71</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J72" s="2" t="s">
         <v>16</v>
@@ -5287,28 +5799,28 @@
         <v>72</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>16</v>
@@ -5319,28 +5831,28 @@
         <v>73</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G74" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J74" s="2" t="s">
         <v>16</v>
@@ -5351,35 +5863,31 @@
         <v>74</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="G75" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Per-tenant credentials are now actually used at runtime. Figma, Xray and Atlassian (Confluence/Jira) resolve credentials from the tenant's own IntegrationConnection (decrypt_secrets) instead of the shared server .env — closing the multi-tenant credential-leak class already fixed for GitHub (S.No 112). Per-field .env fallback kept so CI/tests are unchanged. Done together with S.No 113. Config tests added.</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+        <v>307</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="409.6">
@@ -5387,28 +5895,28 @@
         <v>75</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I76" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J76" s="2" t="s">
         <v>141</v>
@@ -5419,28 +5927,28 @@
         <v>76</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G77" s="2" t="s">
         <v>23</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J77" s="2" t="s">
         <v>141</v>
@@ -5451,35 +5959,31 @@
         <v>77</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G78" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Three-part fix. (A) create_work_item is now idempotent: re-running Task Breakdown REPLACES matching proposed work items (natural key project+type+title+parent) instead of duplicating the whole backlog; already-accepted/in-progress/done items are never touched. (B) A concurrent-run guard blocks a second trigger while a run is live (HTTP 409), for both phase and build triggers. (C) A confirm dialog on both trigger surfaces (Phases &amp; Runs and the Task page): Case 1 (completed) warns 're-running restarts and replaces THIS phase's artifacts, no duplicates'; Case 2 (in progress) blocks with a clear message. Idempotency + guard tests added.</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+        <v>324</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="409.6">
@@ -5487,28 +5991,28 @@
         <v>78</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I79" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="J79" s="2" t="s">
         <v>141</v>
@@ -5519,28 +6023,28 @@
         <v>79</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G80" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I80" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="J80" s="2" t="s">
         <v>141</v>
@@ -5551,28 +6055,28 @@
         <v>80</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I81" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J81" s="2" t="s">
         <v>16</v>
@@ -5583,28 +6087,28 @@
         <v>81</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>23</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I82" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J82" s="2" t="s">
         <v>141</v>
@@ -5615,28 +6119,28 @@
         <v>82</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="I83" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="J83" s="2" t="s">
         <v>16</v>
@@ -5647,28 +6151,28 @@
         <v>83</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I84" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J84" s="2" t="s">
         <v>16</v>
@@ -5679,28 +6183,28 @@
         <v>84</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="I85" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J85" s="2" t="s">
         <v>16</v>
@@ -5711,28 +6215,28 @@
         <v>85</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>23</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="I86" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J86" s="2" t="s">
         <v>141</v>
@@ -5743,28 +6247,28 @@
         <v>86</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="I87" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J87" s="2" t="s">
         <v>16</v>
@@ -5775,28 +6279,28 @@
         <v>87</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I88" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J88" s="2" t="s">
         <v>141</v>
@@ -5807,28 +6311,28 @@
         <v>88</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I89" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J89" s="2" t="s">
         <v>141</v>
@@ -5839,28 +6343,28 @@
         <v>89</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="I90" s="2" t="s">
-        <v>575</v>
+        <v>396</v>
       </c>
       <c r="J90" s="2" t="s">
         <v>16</v>
@@ -5871,35 +6375,31 @@
         <v>90</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="I91" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed / validated end-to-end (2026-07-15/16). Multi-repo Hybrid Option C proven live: TASK-001 built on SpendLogTest-1-backend, 08 review + 07&lt;-&gt;08 remediation loop ran, merge gate approved, squash-merged to main, WorkItem -&gt; done; multi-repo routing, per-repo PRs and single-repo backward-compat all confirmed. All decomposed sub-tasks A1-E1 complete.</t>
-        </is>
-      </c>
-      <c r="J91" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+        <v>402</v>
+      </c>
+      <c r="I91" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="409.6">
@@ -6183,15 +6683,11 @@
       <c r="H100" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="I100" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Verified working — no code change needed. The live 'Add repository' form captures each repo's Role (backend/frontend/infra) via a real selector, sends it to the backend, and persists it on Repository.role (shown back as a chip). Auto-assign keys off this role correctly. Closed as verified.</t>
-        </is>
-      </c>
-      <c r="J100" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="I100" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="409.6">
@@ -6315,15 +6811,11 @@
       <c r="H104" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="I104" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The code-host connect form's single 'Repository' field (which read as single-repo on multi-repo projects) is now labelled 'Default repository', made OPTIONAL, and carries a hint: 'Each build targets its own repo; this is only a fallback default. The token must have access to ALL repos in this project.' The connection is tenant-wide and each build already targets its work-item repo, so Save no longer gates on this field. Backend catalog + frontend render change.</t>
-        </is>
-      </c>
-      <c r="J104" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="I104" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="J104" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="105" spans="1:10" ht="409.6">
@@ -6639,15 +7131,11 @@
       <c r="H114" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="I114" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phase B done (extends S.No 74/112). The remaining connectors — Atlassian Confluence/Jira, Figma, Xray — now authenticate with the tenant's own stored credentials on ANY worker, not the server .env. Atlassian needed a new 'Atlassian account email' field on the Confluence/Jira connect form (basic auth = email + token); the site URL is normalised to the bare site. Per-field .env fallback retained. Config tests added.</t>
-        </is>
-      </c>
-      <c r="J114" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="I114" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="380.1">
@@ -6788,15 +7276,11 @@
       <c r="G119" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I119" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (2026-07-15). agents/06_task_breakdown/agent.md: added a 'Writing standard' requiring every Epic/Story/Task Description + Acceptance Criterion to be plain-language-with-technical-nuance, detailed and self-contained enough that a developer can implement by reading it ALONE (behaviour, inputs/outputs, states, edge cases), with concrete hand-verifiable acceptance criteria and no bare placeholders; modelled the standard in all three template placeholders. Improvement flows to the Work Items board + artifact previews automatically. Test: test_agents_migration.test_task_breakdown_descriptions_and_ac_are_humanized. Per team decision the blast radius today was 06 only; the SAME defect in 02/09/00c/04/03/10 is logged as S.No 121-126 (register-condition per audience: technical-humanized for testing/security, plain+nuance for the rest) and NOT fixed this session.</t>
-        </is>
-      </c>
-      <c r="J119" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="I119" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="113.25">
@@ -6804,7 +7288,7 @@
         <v>119</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D120" s="2" t="s">
         <v>571</v>
@@ -6827,7 +7311,7 @@
         <v>120</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D121" s="2" t="s">
         <v>93</v>
@@ -6841,1321 +7325,1038 @@
       <c r="G121" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I121" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (2026-07-15) - FULL blast radius + Part C (team-approved re-scope). (1) Artifact.title field + migration 0003_artifact_title (nullable, backward-safe). (2) register_artifact/update_artifact gain a title param, plus MCP server + companion wrappers, tool docstrings say 'ALWAYS pass a title'. (3) Part C-1 versioning-collision FIXED: version scoped by (project,phase,type,title) when titled, so per-item siblings (adr/test_case/security_finding/code/code_review/test_report) each start v1 instead of falsely superseding; untitled/singletons keep old behaviour. (4) Platform code/code_review get titles (WI key). (5) Serializers/consumers: DRF ArtifactSerializer + MCP _artifact/_lean_ref + preview payload + traceability node + dashboard + publish title expose/prefer title. (6) Frontend: new artifactLabel(title,type) helper (falls back to humanized type) in Artifacts registry list+search, preview H1/row, Traceability node (was raw type), Export/Publish. (7) 7 agents 04/05/07/08/09/09b/10 author human titles (Wireframe - Login Page, ADR-003 - Event Sourcing, TC-014 - ...). (8) Part C-2 ContractsDrift FIXED: no JSON.stringify dump (humanized scalar summary); DriftRecordSerializer enriches impacted with node_title+repo_name (batched) so no raw UUIDs. Wireframe STATES stay a separate label axis by design. Tests: test_mcp_platform_state (title + per-item independent versions), test_agents_migration (06 + per-item titles), test_review_dispatch/test_api_contract green; frontend tsc clean; ruff clean. Migration NOT yet applied to shared cloud DB - held for a coordinated make migrate (nullable=back-compat).</t>
-        </is>
-      </c>
-      <c r="J121" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" spans="1:10" ht="380">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">121</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Requirements agent (02) authors user stories, functional requirements, acceptance criteria and NFRs too technically/formally for its reviewer. Same defect class as S.No 118 (06 task breakdown): the content is engineer/QA-precision only with no human-readability bar, yet the Product Owner reviews it. HUMANIZATION REGISTER for the fix = PLAIN LANGUAGE retaining the technical nuance (broader audience: PO + developer).</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investigation (session 2026-07-15) edge-case sweep of all 16 phase agents for the S.No 118 pattern. 02 is the closest structural analog to 06.</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agents / 02 Requirements / content humanization</t>
-        </is>
-      </c>
-      <c r="E122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F122" s="2"/>
-      <c r="G122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quality bar is 'a QA engineer can execute without a follow-up question' (agents/02_requirements/agent.md:10); FR format is formal SHALL boilerplate (:115); acceptance criteria are bare BDD stubs (:85-97); user-story descriptions have no plain-language directive; reviewer is the Product Owner (:357). Related S.No 118, 120.</t>
-        </is>
-      </c>
-      <c r="I122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - NOT fixed this session. Team scoped today's fix to S.No 118 (06 task breakdown) only. Planned: add a plain-language-with-technical-nuance authoring bar to user-story descriptions, FR statements and acceptance criteria - mirror 06's assignment_rationale directive (:280) and the good patterns in 05_ux_design/12_deployment/08_code_review.</t>
-        </is>
-      </c>
-      <c r="J122" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" spans="1:10" ht="380">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">122</t>
-        </is>
-      </c>
-      <c r="B123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Testing agent (09) authors UAT scenarios FOR the Product Owner, plus defect reports and test-case descriptions, with an engineer-precision bar only. Same defect class as S.No 118. HUMANIZATION REGISTER for the fix = HUMANIZED-TECHNICAL (keep the technical register but make it clear and well-structured) - NOT plain language, because QA/UAT personnel must interpret the technical detail correctly; plain language would cause misinterpretation.</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investigation edge-case sweep. UAT is a business-verification event handed to a non-engineer, yet authored with two-engineer precision.</t>
-        </is>
-      </c>
-      <c r="D123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agents / 09 Testing / content humanization</t>
-        </is>
-      </c>
-      <c r="E123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F123" s="2"/>
-      <c r="G123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UAT scenarios authored for the PO (agents/09_testing/agent.md:483-494) and defect descriptions (:433-459) use a two-engineer precision bar (:212) with no readability directive for the PO-facing UAT. Test-case Expected Result/Description carry the same risk. Related S.No 118, 120.</t>
-        </is>
-      </c>
-      <c r="I123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - NOT fixed this session (team scope = 06 only). Planned: add a HUMANIZED-TECHNICAL clarity bar (structured, understandable, technical register retained) to UAT scenarios, defect reports and test-case descriptions - not plain language.</t>
-        </is>
-      </c>
-      <c r="J123" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" spans="1:10" ht="380">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">123</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intelligent Context Extractor agent (00c) authors the codebase_intelligence Executive Summary, health dashboard and module-documentation prose read by humans onboarding to a project, with no plain-language directive - jargon-prone. Same defect class as S.No 118. HUMANIZATION REGISTER = PLAIN LANGUAGE retaining technical nuance.</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investigation edge-case sweep.</t>
-        </is>
-      </c>
-      <c r="D124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agents / 00c Context Extractor / content humanization</t>
-        </is>
-      </c>
-      <c r="E124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F124" s="2"/>
-      <c r="G124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agent 'writes the prose' (agents/00c_intelligent_context_extractor/agent.md:44; artifact spec :93-106) with no directive to keep it plain for onboarding readers. Related S.No 118, 120.</t>
-        </is>
-      </c>
-      <c r="I124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - NOT fixed this session (team scope = 06 only). Planned: add a plain-language-with-technical-nuance bar to the exec summary and module-doc prose.</t>
-        </is>
-      </c>
-      <c r="J124" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" spans="1:10" ht="380">
-      <c r="A125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">124</t>
-        </is>
-      </c>
-      <c r="B125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Architecture agent (04) authors ADR Rationale/Context/Consequences prose and the architecture Executive Summary as human-read decision records, but only the Level-1 context diagram carries a 'readable by a non-technical stakeholder' bar - the ADR narrative and exec summary do not. Same defect class as S.No 118. HUMANIZATION REGISTER = PLAIN LANGUAGE retaining technical nuance.</t>
-        </is>
-      </c>
-      <c r="C125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investigation edge-case sweep.</t>
-        </is>
-      </c>
-      <c r="D125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agents / 04 Architecture / content humanization</t>
-        </is>
-      </c>
-      <c r="E125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F125" s="2"/>
-      <c r="G125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Context diagram must be 'readable by a non-technical stakeholder' (agents/04_architecture/agent.md:119) but ADR rationale (:373) and exec summary (:291) have no plain-language bar. Related S.No 118, 120.</t>
-        </is>
-      </c>
-      <c r="I125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - NOT fixed this session (team scope = 06 only). Planned: extend the existing non-technical-readability bar to ADR narrative fields and the exec summary.</t>
-        </is>
-      </c>
-      <c r="J125" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" spans="1:10" ht="380">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">125</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PRD agent (03) is mostly well-humanized, but the per-feature ACCEPTANCE CRITERIA remain terse placeholders - the same artifact type flagged in S.No 118. HUMANIZATION REGISTER = PLAIN LANGUAGE retaining technical nuance.</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investigation edge-case sweep. Partially self-mitigated (strong readability directives elsewhere).</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agents / 03 PRD / content humanization</t>
-        </is>
-      </c>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F126" s="2"/>
-      <c r="G126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Strong readability directives overall (agents/03_prd/agent.md:15,76,354) but per-feature acceptance criteria are terse placeholders (:224-227). Related S.No 118, 120.</t>
-        </is>
-      </c>
-      <c r="I126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - NOT fixed this session (team scope = 06 only). Planned: apply the same detailed, plain-language-with-nuance bar to per-feature acceptance criteria.</t>
-        </is>
-      </c>
-      <c r="J126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" spans="1:10" ht="380">
-      <c r="A127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">126</t>
-        </is>
-      </c>
-      <c r="B127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Security agent (10) authors the Executive Summary and finding Impact statements that reach stakeholders with no plain-language bar. Same defect class as S.No 118. HUMANIZATION REGISTER = HUMANIZED-TECHNICAL for findings (security engineers must read the technical detail correctly); the stakeholder exec summary may be plain-language-with-nuance.</t>
-        </is>
-      </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investigation edge-case sweep. Primary audience is technical; remediation guidance is already appropriately specific.</t>
-        </is>
-      </c>
-      <c r="D127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agents / 10 Security / content humanization</t>
-        </is>
-      </c>
-      <c r="E127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F127" s="2"/>
-      <c r="G127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Exec summary and finding Impact (agents/10_security/agent.md:339-340,395-398) reach stakeholders without a readability bar. Related S.No 118, 120.</t>
-        </is>
-      </c>
-      <c r="I127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - NOT fixed this session (team scope = 06 only). Planned: humanized-technical clarity bar on findings; plain-language-with-nuance on the stakeholder exec summary.</t>
-        </is>
-      </c>
-      <c r="J127" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" spans="1:10" ht="460.0" customHeight="1">
+      <c r="I121" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="J121" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="380.1">
+      <c r="A122" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="I122" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="J122" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="380.1">
+      <c r="A123" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="I123" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="380.1">
+      <c r="A124" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="I124" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="J124" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="380.1">
+      <c r="A125" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H125" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="I125" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="J125" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="380.1">
+      <c r="A126" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="I126" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="J126" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="380.1">
+      <c r="A127" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="I127" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="J127" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="409.6" customHeight="1">
       <c r="A128" s="2">
         <v>127</v>
       </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Merging an approved build fails with HTTP 405 because the pull request is still a draft (the final blocker)</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">After a human approves the merge gate, the platform tries to merge the build's PR but GitHub rejects it, so the work item never reaches 'done'.</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Merge gate</t>
-        </is>
-      </c>
-      <c r="E128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1258d85</t>
-        </is>
-      </c>
-      <c r="G128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">During the automated 07&lt;-&gt;08 review-and-fix loop the platform opens the build's pull request as a GitHub 'draft' PR (a draft blocks a premature human merge while review is still running). GitHub does not allow a draft PR to be merged - its merge API returns HTTP 405 (Method Not Allowed). So the moment a human approved the merge gate, the final merge step always failed. The work item got stuck at the very last step, never transitioned to done, and nothing downstream could complete. This was the single blocker stopping any build from finishing.</t>
-        </is>
-      </c>
-      <c r="I128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (commit 1258d85). Added a mark_ready_for_review step that takes the PR out of draft immediately before merging, which is the one legitimate moment to un-draft (gate already approved). merge_build_pr_core now does: get the PR; if it is not already merged and is still a draft, call codehost.mark_ready_for_review(pr_ref) which runs GitHub's markPullRequestReadyForReview GraphQL mutation and re-checks (short retries) that it un-drafted, then merge. Supporting additions: a graphql() helper (integrations/github/rest.py), a graphql_url property (config.py), and the CodeHost.mark_ready_for_review capability (capabilities.py + github/codehost.py). Regression test added in test_build_activities.py (draft PR is un-drafted before merge).</t>
-        </is>
-      </c>
-      <c r="J128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B128" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H128" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="I128" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="J128" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="409.6" customHeight="1">
       <c r="A129" s="2">
         <v>128</v>
       </c>
-      <c r="B129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reviewer gets 'no opened PR to review' during the fix-and-re-review loop (wrong code pointer picked)</t>
-        </is>
-      </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">During remediation the platform sometimes points the reviewer at an empty pre-PR placeholder instead of the real pull request.</t>
-        </is>
-      </c>
-      <c r="D129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Review loop</t>
-        </is>
-      </c>
-      <c r="E129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1258d85</t>
-        </is>
-      </c>
-      <c r="G129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The helper that looks up a build's code artifact (_code_artifact) fetched 'the first matching artifact' with no defined ordering. A single work item can have more than one code-artifact row: an early placeholder the agent registers before the PR exists, and the real one that carries the pull-request reference (repo/number/url). With no ORDER BY, the database returned rows in an arbitrary order, so the code sometimes picked the early placeholder that has no PR link. The reviewer then had nothing to look at and reported 'no opened PR to review', which broke the remediation cycle.</t>
-        </is>
-      </c>
-      <c r="I129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (commit 1258d85). _code_artifact now orders artifacts by created_at and explicitly prefers the one whose external_ref is a real PR reference: it returns the first PR-ref-bearing artifact and only falls back to the earliest row if none carries a PR ref. Regression test added in test_build_activities.py (duplicate-code-artifact prefers the PR-ref pointer).</t>
-        </is>
-      </c>
-      <c r="J129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B129" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="I129" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="J129" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="409.6" customHeight="1">
       <c r="A130" s="2">
         <v>129</v>
       </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A genuinely 'Approved' code review is wrongly blocked by the fail-closed review guard (false positive on a resolved finding ID)</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The safety guard that blocks bad code mis-reads an approved review and rejects it, stalling the pipeline for no real reason.</t>
-        </is>
-      </c>
-      <c r="D130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Review guard (S.No 114 guard)</t>
-        </is>
-      </c>
-      <c r="E130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a2deeae</t>
-        </is>
-      </c>
-      <c r="G130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The review guard is deliberately 'fail-closed': if a review's prose looks like it demands changes but the structured verdict does not clearly say so, it blocks - to stop bad code slipping through. The old prose matcher (_looks_blocking) scanned the entire review text for blocking-sounding words. An APPROVED review referenced an already-RESOLVED finding by its ID (for example 'REM-W1'), and the matcher saw that mention and concluded the review was demanding changes. Result: a legitimately approved review was blocked and the build could not proceed - a false positive that halted good work.</t>
-        </is>
-      </c>
-      <c r="I130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (commit a2deeae). Rewrote parse_and_guard to trust a present, structured APPROVED verdict. Added _verdict_demands_changes(): a verdict is treated as demanding changes only when a verdict is actually present AND its status matches a negative pattern (change/reject/denied/blocked/fail, via _NEGATIVE_STATUS regex). The loose prose scan is now only a fallback used when there is NO structured verdict at all. Net effect: an approved verdict is honoured even if its prose happens to mention resolved finding IDs, while a review that truly downgrades still fails closed. Regression tests added in test_review_dispatch.py (trusts approved verdict with resolved REM ids; in-JSON downgrade still fails closed).</t>
-        </is>
-      </c>
-      <c r="J130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B130" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H130" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="I130" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="J130" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="409.6" customHeight="1">
       <c r="A131" s="2">
         <v>130</v>
       </c>
-      <c r="B131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the secret scanner blocks a push, the failure is invisible - only a bare count is shown, not what/where</t>
-        </is>
-      </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A blocked hardcoded secret produces a silent 'build failed' with just a number; nobody can tell which secret, file or line.</t>
-        </is>
-      </c>
-      <c r="D131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Companion / Pre-push secret scan</t>
-        </is>
-      </c>
-      <c r="E131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">52533c4</t>
-        </is>
-      </c>
-      <c r="G131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Before pushing code the companion (the worker on the developer machine) scans the changed files for hardcoded secrets (passwords, API keys, tokens, private keys). When it finds one it correctly blocks the push and reports the build as failed - but it only reported a bare count ('N finding(s)'). It did not surface which secret type, which file, or which line, and it then tore down the temporary work folder, so the evidence was gone. Operators saw 'build failed' with no way to know why or how to fix it, making the block undiagnosable.</t>
-        </is>
-      </c>
-      <c r="I131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (commit 52533c4). The companion now prints a redacted summary to its own terminal ('[companion] SECRET SCAN BLOCKED push (N finding(s)) - branch NOT pushed') listing each finding as '[kind] path:line - preview', and the same redacted detail travels in the build.failed reason so it also appears in the platform run console. Only the already-redacted preview is shown - never the raw secret value - and the list is capped at 8 findings with a '(+N more)' tail so the message stays bounded. Added the _format_secret_findings helper (runner/companion/runner.py) and regression tests in test_companion_runner.py (redacted findings surface; cap at 8).</t>
-        </is>
-      </c>
-      <c r="J131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B131" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H131" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="I131" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="J131" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="409.6" customHeight="1">
       <c r="A132" s="2">
         <v>131</v>
       </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The code-review result (code_review artifact) cannot be opened or read from the web UI</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The 08 review report is produced and registered but there is no view/link in the product to read it.</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UI / Review experience</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The 08 review agent produces a code_review artifact holding the review findings and verdict, and the platform registers it as an artifact (pointer + provenance). However the web interface offers no view or link that opens the artifact body, so a human reviewer or manager cannot actually read the review inside the product - they would have to query the database or dig through logs. This undermines the human review gate: the gate exists but the evidence behind it is not surfaced to the person approving.</t>
-        </is>
-      </c>
-      <c r="I132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Verified already fixed — no code change needed. Cross-checked against a live run: the code_review artifact IS registered with a rendered report body (the companion uploads the .md to S3 — confirmed a ~22 KB report object exists for the latest run), and the generic artifact preview reads it, so the report opens and reads in the UI. The earlier 'no body' analysis looked only at the platform-side fallback registration and missed the companion upload. Closed as verified.</t>
-        </is>
-      </c>
-      <c r="J132" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B132" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H132" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="I132" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="J132" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="409.6" customHeight="1">
       <c r="A133" s="2">
         <v>132</v>
       </c>
-      <c r="B133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The 'sdlc/build' commit status is set to 'pending' when the PR opens and is never updated - it stays pending forever (latent)</t>
-        </is>
-      </c>
-      <c r="C133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A dormant flaw: the build commit status posted to GitHub is never moved off 'pending', which will block merges if branch protection ever requires it.</t>
-        </is>
-      </c>
-      <c r="D133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Commit status reporting</t>
-        </is>
-      </c>
-      <c r="E133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">build_activities.py:140</t>
-        </is>
-      </c>
-      <c r="G133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="H133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the build PR is opened, the platform posts a GitHub commit status with context 'sdlc/build' and state 'pending' against the head commit (build_activities.py line 140, best-effort - exceptions are swallowed). Nothing anywhere later updates that status to 'success' or 'failure'. So every build's commit shows the 'sdlc/build' check stuck on pending indefinitely. It is dormant today only because no branch-protection rule on the repo currently requires the 'sdlc/build' context to be green before merging. The day someone enables such a required check, merges will be blocked forever because the status can never reach success - a latent time-bomb, and misleading status UI in the meantime.</t>
-        </is>
-      </c>
-      <c r="I133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - not fixed this session. Recommended fix: complete the status lifecycle. Set 'sdlc/build' to 'success' once the build+review pass (or at merge), and to 'failure' on the mark_build_failed / secret-block / merge-failed paths, using the same head SHA. Keep it best-effort (do not fail the saga on a status-post error), but ensure a terminal state is always posted so the check does not dangle. Acceptance: after a run reaches a terminal outcome, the commit's 'sdlc/build' status reflects success or failure, never a permanent pending.</t>
-        </is>
-      </c>
-      <c r="J133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B133" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H133" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="I133" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="J133" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="409.6" customHeight="1">
       <c r="A134" s="2">
         <v>133</v>
       </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The companion crashes hard (fatal, exit 1) when the build agent errors, instead of failing gracefully and reporting back</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">If the AI build agent fails, the whole companion worker dies and needs a manual restart, stalling the build.</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Companion / Build execution resilience</t>
-        </is>
-      </c>
-      <c r="E134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the build agent (the Claude Agent SDK run inside the companion) exits with an error, the exception propagates all the way up and the companion process terminates fatally (Command failed / exit code 1). Because the companion runs one build at a time and is a long-lived poller, a single agent error takes the whole worker down: it stops polling, the current run is left dangling (claimed but not reported), and a human has to notice and restart the companion before any further work can proceed. Observed repeatedly this session (e.g. when a mid-build backend restart broke the agent's MCP calls, and when an environment/dependency mismatch made the agent exit).</t>
-        </is>
-      </c>
-      <c r="I134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed (2026-07-16). runner/companion/daemon.py _run_build now catches a generic build-agent error, posts a failed BuildReport (status=failed + message) to /api/runner/builds/&lt;run&gt;/report/, and keeps polling (mirrors the plan/review path _run_engine_phase) instead of the exception propagating out of serve and killing the long-lived companion. EngineAuthError still fail-closes (explicit re-raise) so a subscription/auth halt is never downgraded to a per-build failure. Tests: test_companion_daemon (agent-error reported + no crash; auth-error still halts).</t>
-        </is>
-      </c>
-      <c r="J134" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B134" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H134" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="I134" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="J134" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" ht="409.6" customHeight="1">
       <c r="A135" s="2">
         <v>134</v>
       </c>
-      <c r="B135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A worker can deadlock a job by self-renewing its own claim while making no progress (stuck job never released)</t>
-        </is>
-      </c>
-      <c r="C135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A worker keeps renewing its hold (heartbeat) on a job it isn't actually advancing, so the job sits claimed forever and nothing else can take it.</t>
-        </is>
-      </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Claim + heartbeat (S.No 111)</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jobs are handed to a worker via a claim, and a heartbeat (S.No 111) periodically renews that claim so the platform knows the worker is alive. The problem: the heartbeat renews the claim based on the worker still running, not on the work actually progressing. If the worker gets wedged (e.g. the agent hangs, or a step is stuck) but the heartbeat thread keeps ticking, the claim is renewed indefinitely. The job stays 'claimed', the report-timeout takeover cannot fire (the claim looks fresh), and no other worker can pick it up - a silent deadlock that only a human notices. Seen this session as the 'companion claimed but never built' deadlock.</t>
-        </is>
-      </c>
-      <c r="I135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed (2026-07-16). Cross-verified first: _renew_claims_for renewed the claim on process liveness alone (no progress signal, no cap), so a wedged-but-heartbeating worker held its claim until only the 2h workflow report-timeout (S.No 89) freed it. Fix: backend/api/runner_views.py stamps first_claimed_at at each claim (reset per claim, never touched by heartbeat) and MAX_CLAIM_AGE=60min caps renewal - past it the heartbeat stops renewing so the lease ages out and the run is recoverable well before the 2h backstop. Cap set above the longest legit build (&lt;60min, team-confirmed) so a healthy long build is never capped (no S.No 111 regression). Note: a companion progress-signal is the fundamentally optimal fix (distinguishes wedged-vs-working at any duration) - logged as the future upgrade if builds ever exceed ~1h. Tests: test_phase_dispatch (cap stops renewal; young claim still renews).</t>
-        </is>
-      </c>
-      <c r="J135" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B135" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H135" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="I135" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="J135" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" ht="409.6" customHeight="1">
       <c r="A136" s="2">
         <v>135</v>
       </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dependency version skew: pinned claude-agent-sdk / anyio in the repo are behind what the runtime actually needs</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The project's pinned library versions lag what the running machine requires; fixed by hand on the machine but not locked in the repo, so it will break for the next person.</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Companion / Dependency management</t>
-        </is>
-      </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The companion depends on claude-agent-sdk, which in turn requires a newer anyio (the anyio.open_process 'user' keyword arrives in anyio 4.5.0; claude-agent-sdk 0.1.72 needs it). The repo's pins were stale (an old claude-agent-sdk pin and no floor on anyio), so a fresh environment installed anyio 4.4.0 and the agent crashed with "anyio.open_process() got an unexpected keyword argument 'user'". This session it was worked around by manually upgrading anyio on the host (pip install -U 'anyio&gt;=4.5' -&gt; 4.14.2), but that fix lives only on this machine - the repo still pins the broken combination, so the next developer or a rebuilt container will hit the same crash.</t>
-        </is>
-      </c>
-      <c r="I136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - not fixed this session (env-patched only). Recommended fix: pin the correct, mutually compatible versions in the repo lockfile/requirements - bump claude-agent-sdk to the version actually in use and add an explicit anyio&gt;=4.5 floor - then rebuild the companion/worker images from the lockfile so a clean install reproduces the working environment. Acceptance: a from-scratch install (no manual pip upgrades) runs a build without the open_process 'user' error.</t>
-        </is>
-      </c>
-      <c r="J136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B136" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H136" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="I136" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="J136" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" ht="409.6" customHeight="1">
       <c r="A137" s="2">
         <v>136</v>
       </c>
-      <c r="B137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build branches are merged without first being updated against their base, causing merge conflicts at the gate</t>
-        </is>
-      </c>
-      <c r="C137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The platform merges a feature branch without rebasing/updating it against the current base, so it hits conflicts (mergeable_state=dirty) and the merge fails.</t>
-        </is>
-      </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Merge gate</t>
-        </is>
-      </c>
-      <c r="E137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the merge gate is approved, the platform merges the feature branch as-is. It never updates the branch against the latest base first. If the base has moved on since the branch was cut - which is normal in a multi-developer repo - the PR can be in a conflicted state (GitHub mergeable_state = 'dirty'), and the merge API then returns HTTP 405 just like the draft case. This session WI-29 hit exactly this: an add/add conflict on frontend/.env.example left the PR dirty and the merge failed; it had to be resolved by hand. The pipeline has no step to bring a branch up to date with its base before attempting the merge.</t>
-        </is>
-      </c>
-      <c r="I137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed (2026-07-16). The merge gate merged the feature branch as-is, so a base that moved since the branch was cut left the PR mergeable_state=dirty and the GitHub merge API returned a raw 405. Fix: integrations/types.py PullRequest gains mergeable/mergeable_state; github/codehost.py adds update_branch (GitHub Update-branch; swallow 422 already-up-to-date) + ensure_mergeable (bounded re-read for GitHub's async mergeability); build_activities.py merge_build_pr_core now, before merging: if 'behind' -&gt; update branch against base then re-check; if 'dirty'/not mergeable -&gt; fail fast (non-retryable ApplicationError) with a clear 'merge conflict - needs manual resolution' reason instead of a cryptic 405; merges only when mergeable. Idempotent behind the existing 'if not pr.merged' guard. Tests: test_build_activities (behind-&gt;update-&gt;merge; dirty-&gt;clean fail, never merged). Reason surfacing verified in live test: the classified reason reaches the user via the S.No 139 ActivityError-cause unwrap (build_workflow uses build_types.failure_reason), since str(ActivityError) is the opaque "Activity task failed".</t>
-        </is>
-      </c>
-      <c r="J137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B137" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H137" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="I137" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="J137" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" ht="409.6" customHeight="1">
       <c r="A138" s="2">
         <v>137</v>
       </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Planning overlap: two separate work items are both told to create the same file (frontend/.env.example), guaranteeing a conflict</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TASK-003 and TASK-005 each create frontend/.env.example, so when both build they collide - a work-breakdown/planning defect.</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Planning / Work-item decomposition</t>
-        </is>
-      </c>
-      <c r="E138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two independently-dispatched work items (TASK-003 and TASK-005) were each planned to create the same file, frontend/.env.example. When both branches are built and then merged, they produce an add/add conflict on that file - there is no shared ownership or de-duplication in the planning step. This is the upstream cause of the WI-29 merge conflict (S.No 136): the pipeline had no branch-update step to catch it, but the conflict should not have been planned in the first place. It points to a gap in how the planner assigns file ownership across parallel work items.</t>
-        </is>
-      </c>
-      <c r="I138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not reproducible / not a bug — verified against stored work-item data. TASK-003 creates the FRONTEND .env.example (frontend repo); TASK-005 is a backend SQLAlchemy/Alembic task (backend repo) — different files, different repos, no collision. The likely confusion: TASK-002 (backend .env.example) and TASK-003 (frontend .env.example) are two correctly-separate files that merely share a name. Closed.</t>
-        </is>
-      </c>
-      <c r="J138" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B138" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H138" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="I138" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="J138" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="409.6" customHeight="1">
       <c r="A139" s="2">
         <v>138</v>
       </c>
-      <c r="B139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two developers share a single enrollment record, risking incorrect work attribution and tenant isolation</t>
-        </is>
-      </c>
-      <c r="C139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two devs point at the same enrollment identity (32db7f5f), so runs/work may be attributed or isolated to the wrong person.</t>
-        </is>
-      </c>
-      <c r="D139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tenancy / Enrollment identity</t>
-        </is>
-      </c>
-      <c r="E139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">enrollment 32db7f5f</t>
-        </is>
-      </c>
-      <c r="G139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">During testing it was found that two different developers are operating under the same enrollment record (enrollment id 32db7f5f, under tenant 212395b8). Enrollment is meant to identify a single developer's participation in a project; sharing one record between two people means their runs, claims and attribution can be conflated, and any per-developer isolation or accounting keyed on enrollment is wrong. It also muddies debugging (whose companion claimed what) and could let one developer's actions appear under the other's identity.</t>
-        </is>
-      </c>
-      <c r="I139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - not fixed this session (flagged during testing). Recommended fix: give each developer their own enrollment record under the tenant/project, and ensure the companion is launched with the correct per-developer enrollment/credentials so claims and events attribute to the right person. Audit existing runs that used the shared enrollment. Acceptance: each developer has a distinct enrollment and their runs attribute correctly.</t>
-        </is>
-      </c>
-      <c r="J139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B139" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H139" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="I139" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="J139" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="409.6" customHeight="1">
       <c r="A140" s="2">
         <v>139</v>
       </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build failures don't explain why - most failures show a generic 'build failed' or a raw, cryptic error instead of a clear reason</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When a build fails for reasons other than a blocked secret (token/permission error, merge conflict, agent error, empty build), the platform shows 'build failed' or a raw exception string, not a plain classified reason.</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Failure observability</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The build.failed reason is populated inconsistently across the different failure paths (build_workflow.py). A companion report failure falls back to the generic literal 'build reported failed' when no message is set. Remediation-exhausted is the hardcoded 'remediation cycles exhausted'. The PR/gate-setup and merge paths embed a raw Python/Temporal exception string ('pr/gate setup failed: {exc}', 'merge failed: {exc}') - so a token-permission (403) error or a merge conflict (405) is technically present but buried in a cryptic stack string, not classified as 'token permission issue' or 'merge conflict'. Only the secret-scan case (S.No 130) was made human-readable. Net effect: for most failure kinds an operator sees 'build failed' with no actionable reason and must dig through logs to triage.</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed (2026-07-16). build.failed reasons were inconsistent (bare 'build reported failed', hardcoded 'remediation cycles exhausted', raw exception strings 'merge failed: {exc}') AND - a hidden gap - the EventSerializer never surfaced the 'reason' payload key, so the run console showed only 'Build failed'. Fix: build_activities.py classify_build_failure maps every failure path to a plain-language classified reason (merge conflict / permission-403 / remediation exhausted / empty build / agent error; the good S.No 130 secret-scan message passes through); mark_build_failed_core writes it to run.outputs.error (where the run console reads the failure line) and the build.failed event; api/serializers.py adds 'reason' to the event message keys. Composes with S.No 136 (single canonical 'merge conflict' reason). Tests: test_build_activities (classifier mappings; reason on run.outputs.error). CORRECTION (same session, caught by live test): the workflow now UNWRAPS the ActivityError .cause via build_types.failure_reason so the classifier sees the real message (Temporal str(ActivityError)="Activity task failed" otherwise hides the 405/422/conflict); AND open_build_pr_core fails an EMPTY build fast (non-retryable ApplicationError "empty build: no changes") instead of a cryptic 422 after 3 retries - an empty build still FAILS (clear reason), it does not auto-succeed. Tests: failure_reason unwrap + empty-build fast-fail + classifier mappings.</t>
-        </is>
-      </c>
-      <c r="J140" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="B140" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H140" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="I140" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="J140" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="141" spans="1:10">
       <c r="A141" s="2">
         <v>140</v>
       </c>
-      <c r="B141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No human action to resolve a non-mergeable / redundant / failed WorkItem: a task can only reach 'done' via a successful automated build+merge. A build that fails (empty/redundant build, or a merge conflict needing manual resolution) leaves the WorkItem stuck at in_progress with no product path for a human to mark it done, skip it, or close it as redundant.</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Surfaced 2026-07-16 while testing S.No 136/139: TASK-002 (redundant with TASK-001) produced an empty build that correctly FAILED with 'Empty build: no changes to commit'. The WorkItem then sits at in_progress with the branch/draft PR left in place, and the only offered action is Retry - which re-fails for a genuinely redundant task. A human can freely trigger the NEXT task (tasks are independent unless depends_on) but cannot close/resolve the failed one. Today the only ways to reach done are the happy-path orchestrator flow or an admin DB state change.</t>
-        </is>
-      </c>
-      <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Work Items / Build recovery UX</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement</t>
-        </is>
-      </c>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">backend/apps/workitems/models.py (State: proposed/accepted/in_progress/in_review/blocked/done, no transition validation); backend/api/serializers.py WorkItemPatchSerializer (state NOT writable) + read_only state; backend/api/views.py WorkItemViewSet (trigger/build/take-over/lifecycle - no transition/mark-done action); mcp_platform_state/tools.py transition_work_item (any-&gt;any, internal only); frontend RunConsole.tsx (Retry only) / WorkItemTask.tsx (done is display-only) / OfflineTakeover.tsx</t>
-        </is>
-      </c>
-      <c r="G141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WorkItem.state is read-only on the API (excluded from WorkItemPatchSerializer; read_only on the read serializer) and mutated ONLY internally by the orchestrator (successful build+merge / gate / reject / takeover). No human-facing transition/mark-done/close/skip action or endpoint exists; the frontend offers only Retry / Trigger phase / manual takeover (sets takeover_flag, not state). transition_work_item allows any-&gt;any but is unexposed to users.</t>
-        </is>
-      </c>
-      <c r="I141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - proposed: add a GATED human action + API endpoint to move a WorkItem to a terminal state outside the happy path (e.g. 'Mark done', 'Close as redundant / won't-do', or 'Skip'), surfaced on the Work Items board + task page, with an audit Event. Decide whether to reuse 'done' or add a distinct terminal state (e.g. 'closed'/'cancelled') to distinguish completed-by-build from human-closed; guard with role/permission. Related S.No 76 (no task-edit UI; state not editable).</t>
-        </is>
-      </c>
-      <c r="J141" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
+      <c r="B141" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H141" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="I141" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="J141" s="2" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="142" spans="1:10">
       <c r="A142" s="2">
         <v>141</v>
       </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Merge gate can't recover from a conflict without redoing the whole build. TWO related enhancements (logged together): (ENH-2, IMPLEMENT NOW) Merge-only retry / re-openable merge gate - when a merge hits a conflict, PAUSE at the merge step and let the user retry the merge after fixing the conflict, WITHOUT re-running the whole build. (ENH-1, FUTURE / only if needed) Reconcile the Run status on an EXTERNAL merge - when a user merges the PR by hand in GitHub, also flip the Run from failed to done (today the webhook updates the WorkItem + artifact but leaves the Run 'failed').</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Today a merge conflict marks the ENTIRE build failed and ends the workflow, so finishing means re-running everything (AI re-writes the code, re-reviews, re-opens the PR) just to retry one merge. ENH-2 fixes this: keep the build paused at the merge gate; after the user resolves the conflict in GitHub they press Merge/Approve again and the platform completes the merge through its OWN flow (run + gate + work-item all stay correct automatically, no rebuild). ENH-1 covers a DIFFERENT path - the user merges by hand in GitHub instead of letting the platform do it; then the platform only learns via webhook (S.No 88) and today leaves the Run status stale. TEAM PLAN (2026-07-16): implement ENH-2 now; keep ENH-1 for future - it overlaps S.No 88 and is only needed if users merge OUTSIDE the platform. If ENH-2 is used, ENH-1 is largely unnecessary. Same 'soft, reconcilable' idea as the S.No 89 fix, applied to merge conflicts.</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Merge gate recovery</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement</t>
-        </is>
-      </c>
-      <c r="F142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">backend/orchestration/build_workflow.py (merge gate + ActivityError-&gt;mark_build_failed is TERMINAL on a conflict); backend/orchestration/build_activities.py merge_build_pr_core (S.No 136 dirty-&gt;fail); backend/integrations/webhooks.py _reconcile_pull_request (updates WorkItem+artifact on an external merge, NOT the Run); frontend Gates.tsx (merge gate) + RunConsole.tsx. Related: S.No 88 (external merge / missing webhook), S.No 89 (soft-reconcilable pattern), S.No 136 (conflict detection).</t>
-        </is>
-      </c>
-      <c r="G142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On a merge conflict the BuildWorkflow catches the ActivityError and calls mark_build_failed, which is TERMINAL - the workflow ends, so there is no live workflow to retry the merge and the merge-gate Approval is already spent. The only ways forward today are a full re-trigger (rebuilds from 07) or an external GitHub merge (needs the S.No 88 webhook, which also does not reconcile the Run status).</t>
-        </is>
-      </c>
-      <c r="I142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ENH-2 IMPLEMENTED &amp; VALIDATED LIVE (@ 66b70c8, + gate banner). A merge conflict is now NON-terminal: merge_build_pr detects a dirty PR and raises a typed MergeConflict; the BuildWorkflow catches it, RE-OPENS the merge gate (resets the approval to pending, records outputs.merge_conflict + a build.merge_conflict event) and waits — instead of failing the build. The user resolves the conflict in GitHub and approves again; the platform retries ONLY the merge (no rebuild, no re-review). Proven live on TASK-003 (run 1d1dd943): injected an add/add conflict on .env.example -&gt; approve -&gt; gate re-opened (once per remaining conflict) -&gt; resolved -&gt; approve -&gt; platform merged PR#1 (merge commit c1d7552a) -&gt; WorkItem done -&gt; run completed, with NO rebuild across retries. The merge gate now shows a warning banner explaining the conflict + retry (ApprovalSerializer.merge_conflict; shown ONLY on a re-opened merge gate, never other gates). ENH-1 (reconcile Run status on an EXTERNAL GitHub merge) remains FUTURE / optional — it overlaps S.No 88 and is only needed if users merge outside the platform, which ENH-2 makes largely unnecessary.</t>
-        </is>
-      </c>
-      <c r="J142" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" spans="1:1">
+      <c r="B142" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H142" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="I142" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="J142" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10">
       <c r="A143" s="2">
         <v>142</v>
       </c>
-      <c r="B143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Backlog push to Jira: tasks never reach Jira — each Task is created with its Story as parent, which Jira rejects</t>
-        </is>
-      </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">During a live Jira push of the SpendLog-1 backlog, all 5 epics + 15 stories were created but 0 of 29 tasks landed. reconcile creates each task with parent = its story's Jira key; Jira rejects a standard Task parented to a Story (400 'Please select valid parent issue') — only Sub-tasks can live under a Story (Jira hierarchy: Epic &gt; Story/Task, and Epic &gt; Story &gt; Sub-task).</t>
-        </is>
-      </c>
-      <c r="D143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Integrations / TaskTracker (Jira)</t>
-        </is>
-      </c>
-      <c r="E143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">reconcile.reconcile_work_item mapped WorkItem.type 'task' -&gt; Jira 'Task' and set parent={key: story}. Jira does not allow a standard Task under a Story. Stories succeeded because Story-under-Epic via the parent field IS valid; tasks-under-stories are not.</t>
-        </is>
-      </c>
-      <c r="I143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TWO layered causes, both fixed. (1) REAL ROOT CAUSE: reconcile's idempotency guard 'if wi.external_ref' wrongly treated a repo-assigned task as already-reconciled. Multi-repo tasks carry external_ref.repo_assignment (the planner's repo pick, Option C) with NO SoR id, so on the live push every task was SKIPPED before reaching Jira (export showed created:0, reconciled:29, no error — not a Jira rejection at all). Fixed: the guard now checks for a real SoR key (external_ref.id), and the SoR ref is MERGED into external_ref so the repo_assignment is preserved. (2) HIERARCHY (latent, also fixed): once tasks reach Jira, a standard Task can't be a child of a Story, so a task with a reconciled story parent is created as a SUB-TASK under it (the project's real sub-task issue-type name, resolved via AtlassianTaskTracker.subtask_type_name() + cached), and a parentless task as a top-level Task. Validated live (Sub-task-under-Story create succeeds; Task-under-Story returns 400). Tests in test_reconcile: repo-assigned task not-skipped + repo_assignment preserved, subtask mapping, parentless task, per-item failure capture. NOTE: my first commit fixed only the hierarchy; the guard/repo_assignment fix (the true blocker) landed in the follow-up commit after the re-push showed created:0.</t>
-        </is>
-      </c>
-      <c r="J143" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" spans="1:1">
+      <c r="B143" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G143" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H143" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="I143" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="J143" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10">
       <c r="A144" s="2">
         <v>143</v>
       </c>
-      <c r="B144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Backlog publish reports a green 'Published' while items silently fail to reach the system of record</t>
-        </is>
-      </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The same Jira push showed 'Published — 49 work items reconciled (20 created)' even though 29 tasks failed. reconcile_backlog ran each item with no per-item error handling and the publish response/dialog surfaced only reconciled/created — so partial failures were invisible and the reconciled count over-reported what actually landed.</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Integrations / Publish</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">reconcile_backlog processed items in a list comprehension with no try/except, and _publish_tasktracker + the ExportPublish dialog reported only reconciled/created counts — never failures. A partial push read as a full success.</t>
-        </is>
-      </c>
-      <c r="I144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">reconcile_backlog now isolates each item in try/except: a single item's SoR rejection is recorded (logged as a workitem.reconcile_failed event + returned in a 'failed' list) and the run continues, instead of aborting or being swallowed. The publish API returns status 'partial' plus the failed items; the artifact stores a failed count; the ExportPublish dialog now shows 'Published with some failures — N created, M failed' + the first error, instead of an all-green success. Test added in test_reconcile (per-item failure captured; epic/story still land).</t>
-        </is>
-      </c>
-      <c r="J144" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="145" spans="1:10" ht="460.0" customHeight="1">
+      <c r="B144" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F144" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G144" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H144" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="I144" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="J144" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="409.6" customHeight="1">
       <c r="A145" s="2">
         <v>144</v>
       </c>
-      <c r="B145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Secret scanner false-positives on hyphenated placeholders (e.g. change-me-...) in .env.example, blocking legitimate builds</t>
-        </is>
-      </c>
-      <c r="C145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The pre-push secret scan flagged an obvious placeholder value as a real secret, so the push was blocked and the build failed.</t>
-        </is>
-      </c>
-      <c r="D145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Companion / Pre-push secret scan</t>
-        </is>
-      </c>
-      <c r="E145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3c33554</t>
-        </is>
-      </c>
-      <c r="G145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The companion's pre-push secret scanner (runner/companion/guardrails.py) blocks a push when it finds anything that looks like a hardcoded secret. Its placeholder allow-list recognised the literal token 'changeme' but NOT the far more common hyphenated/underscored form 'change-me'. So a legitimate .env.example placeholder - JWT_SECRET=change-me-minimum-32-characters-long (36 chars, Shannon entropy 3.875) - was not recognised as a placeholder, tripped the generic high-entropy heuristic, and was flagged as a 'high_entropy_secret'. The push was blocked and the build failed. This is a FALSE POSITIVE: the value is an obvious placeholder, not a real secret. It blocked WI-32 and would block any task whose example env file uses the very common change-me convention. The build agent did nothing wrong - the scanner was too aggressive.</t>
-        </is>
-      </c>
-      <c r="I145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED (commit 3c33554). Two changes in runner/companion/guardrails.py: (1) broadened the placeholder allow-list to cover change[-_ ]?me / replace[-_ ]?me / to-be-(changed|set|replaced|filled|generated) / secret-(here|goes) / dummy / sample / redacted, so hyphenated placeholders are recognised. (2) Committed template files (.env.example, *.sample, *.template, *.dist, *.tpl) now skip the generic entropy heuristic - placeholders are expected there - while STILL running the high-precision key-format patterns (AWS AKIA..., GitHub ghp_..., PEM private keys, JWT), so a real key shape pasted into an example file is still blocked. Regression tests in backend/tests/test_guardrails.py: the exact WI-32 value + change_me/replace-me variants pass clean; a real random token in real source still blocks; AWS/GitHub key shapes inside .env.example still block; non-template source keeps the full entropy scan. 12/12 scanner tests pass.</t>
-        </is>
-      </c>
-      <c r="J145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" spans="1:1">
+      <c r="B145" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F145" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="G145" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H145" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="I145" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="J145" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10">
       <c r="A146" s="2">
         <v>145</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="460.0" customHeight="1">
+    <row r="147" spans="1:10" ht="409.6" customHeight="1">
       <c r="A147" s="2">
         <v>146</v>
       </c>
-      <c r="B147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AI-engine build failures (usage/rate limit, agent CLI exit 1) show a raw, unreadable message instead of a clear reason</t>
-        </is>
-      </c>
-      <c r="C147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the agent CLI fails (e.g. the Anthropic usage limit is reached) the run console shows 'Command failed with exit code 1 ... Check stderr output for details' - opaque and non-actionable.</t>
-        </is>
-      </c>
-      <c r="D147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Build pipeline / Failure observability + Companion</t>
-        </is>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">daemon.py:271</t>
-        </is>
-      </c>
-      <c r="G147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When the AI build agent fails to run - most commonly because the Anthropic usage/rate limit is reached, but also on any agent CLI non-zero exit - the companion's error handler (runner/companion/daemon.py ~line 271) captures only the engine driver's generic wrapper string and reports it verbatim: 'Command failed with exit code 1 (exit code: 1) / Error output: Check stderr output for details'. The platform's classify_build_failure (backend/orchestration/build_activities.py) does not recognise this signature, so the raw string passes straight through to the build.failed reason and the run console. The user sees an opaque error with no indication that the real cause was a usage limit and no guidance on what to do. This bit WI-32: the usage limit was hit during the cycle-2 remediation build and the console showed only 'Command failed with exit code 1'. Same defect class as S.No 139 (classified reasons) but for the engine/usage-limit failure path, which was not covered.</t>
-        </is>
-      </c>
-      <c r="I147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - Fix A planned this session (this row's owner). Two parts: (1) Companion (daemon.py): capture the agent process's stderr tail and put the actual cause in the report message instead of the placeholder 'Check stderr output for details'. (2) Platform (classify_build_failure): recognise engine / usage-limit / rate-limit signatures ('exit code 1', 'usage limit', 'rate limit', '429', 'overloaded', 'quota', 'Failed to start Claude Code') and map them to a plain-language reason, e.g. 'The AI engine hit its usage limit - the build stopped; retry when the limit resets.' NOTE: true resume-from-checkpoint on a transient failure (so a re-run continues from the last cycle instead of rebuilding) is tracked separately as S.No 147 and is owned by the other developer. Acceptance: a usage-limit failure shows a clear, non-technical reason naming the usage limit, not a raw exit-code string.</t>
-        </is>
-      </c>
-      <c r="J147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" spans="1:1">
+      <c r="B147" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F147" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="G147" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H147" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="I147" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="J147" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" ht="210.75">
       <c r="A148" s="2">
         <v>147</v>
       </c>
-    </row>
-    <row r="149" spans="1:1">
+      <c r="B148" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G148" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J148" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" ht="259.5">
       <c r="A149" s="2">
         <v>148</v>
       </c>
-    </row>
-    <row r="150" spans="1:1">
+      <c r="B149" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J149" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" ht="275.25">
       <c r="A150" s="2">
         <v>149</v>
       </c>
-    </row>
-    <row r="151" spans="1:1">
+      <c r="B150" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>719</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J150" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" ht="226.5">
       <c r="A151" s="2">
         <v>150</v>
       </c>
-    </row>
-    <row r="152" spans="1:1">
+      <c r="B151" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F151" s="2" t="e" vm="14">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G151" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J151" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" ht="162">
       <c r="A152" s="2">
         <v>151</v>
       </c>
-    </row>
-    <row r="153" spans="1:1">
+      <c r="B152" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F152" s="2" t="e" vm="15">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G152" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J152" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" ht="162">
       <c r="A153" s="2">
         <v>152</v>
       </c>
-    </row>
-    <row r="154" spans="1:1">
+      <c r="B153" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F153" s="2" t="e" vm="15">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G153" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J153" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" ht="129">
       <c r="A154" s="2">
         <v>153</v>
       </c>
-    </row>
-    <row r="155" spans="1:1">
+      <c r="B154" s="2" t="s">
+        <v>723</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F154" s="2" t="e" vm="16">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G154" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J154" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" ht="210.75">
       <c r="A155" s="2">
         <v>154</v>
       </c>
-    </row>
-    <row r="156" spans="1:1">
+      <c r="B155" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>719</v>
+      </c>
+      <c r="G155" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J155" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="113.25">
       <c r="A156" s="2">
         <v>155</v>
       </c>
-    </row>
-    <row r="157" spans="1:1">
+      <c r="B156" s="2" t="s">
+        <v>725</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G156" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J156" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="162">
       <c r="A157" s="2">
         <v>156</v>
       </c>
-    </row>
-    <row r="158" spans="1:1">
+      <c r="B157" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J157" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="226.5">
       <c r="A158" s="2">
         <v>157</v>
       </c>
-    </row>
-    <row r="159" spans="1:1">
+      <c r="B158" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G158" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J158" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10">
       <c r="A159" s="2">
         <v>158</v>
       </c>
     </row>
-    <row r="160" spans="1:1">
+    <row r="160" spans="1:10">
       <c r="A160" s="2">
         <v>159</v>
       </c>

</xml_diff>

<commit_message>
Log the clarifications tier fix and a follow-up in the bug tracker
Adds two rows to docs/Bugs.xlsx (screenshots preserved):
- S.No 163 (Fixed): the clarification gate used to show only the must-ask
  (Tier 1) questions, so the agent's Tier 2 suggestions and Tier 3 guesses
  never reached the user. All three tiers are now surfaced in one gate.
- S.No 164 (Open, P3): a follow-up - the platform still trusts the agent's
  own tier labelling and does not yet double-check that a business-critical
  question wasn't mislabelled as a low-risk guess.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -8642,14 +8642,104 @@
         <v>162</v>
       </c>
     </row>
-    <row r="164" spans="1:1">
+    <row r="164" spans="1:10">
       <c r="A164" s="2">
         <v>163</v>
       </c>
-    </row>
-    <row r="165" spans="1:1">
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clarification gate surfaced only Tier-1 (must-ask) questions - Tier-2 suggestions and Tier-3 inferences never reached the user</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The SDLC app promises a human is always in the loop and the platform never silently assumes. But agents classified each context gap into three tiers and only surfaced Tier 1 through the clarifications gate. Tier 2 (the agent's own suggestions) was written inline inside the deliverable, and Tier 3 (industry-standard inferences) was logged silently as assumptions the user never saw. So the user could not confirm or override the agent's Tier-2/3 choices, and the 'no silent assumptions' assurance was only partly true.</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clarifications / Context Gap Scan</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed live across Ideation, Requirements and PRD runs on tenant Edvensoft-2: every phase logged Tier-3 items as assumptions and opened 0 clarifications, so the user never saw the agent's inferences. Verified in code: ask_human was the only human-question touchpoint and the shared rules told agents to front-load only Tier 1 and Tier 2. Retested after the fix on a live UX-design run - a single gate now shows Tier 1/2/3 sections.</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The behaviour lived in the shared agent rules (backend/manifest/rules/prompt_rules.py): agents were told to 'front-load ALL Tier-1 and Tier-2 questions' and to record every Tier-3 inference silently as an assumption. Only Tier 1 was required/blocking; nothing surfaced Tier 2 or Tier 3 through the clarifications gate. The tier definitions were also thin (one line each), so classification was inconsistent.</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reworked the shared rules so the agent front-loads ALL three tiers into ONE clarifications gate before starting work, each question tagged with its tier. Tier 1 stays required; Tier 2/3 are optional and carry the agent's proposed answer as a pre-filled 'suggestion' the user can accept, edit or override, with an 'Accept all' one-click. Any untouched Tier-2/3 item falls back to the suggestion, and the confirmed Tier-3 values are still recorded as assumptions for provenance. Also strengthened the tier definitions (a four-question test plus concrete examples per tier). The web gate groups questions under Tier 1/2/3 headers. No DB migration (questions are stored as JSON). Landed on develop in commit 0c19292; backend + frontend tests, type-checks and lint all pass; user-tested on a live UX-design run.</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" spans="1:10">
       <c r="A165" s="2">
         <v>164</v>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platform does not verify the agent's tier classification - a mislabelled Tier-1 gap can still slip through as a Tier-3 guess</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Even with all three tiers now surfaced in the gate, the platform trusts the agent's own Tier 1/2/3 labelling. If the agent wrongly files a business-critical gap (for example pricing, compliance or a third-party integration) as a Tier-3 inference, it is shown pre-filled and quietly accepted rather than hard-asked. So the 'never assume' assurance still depends on the agent classifying correctly and the human reviewer noticing at the gate.</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clarifications / Context Gap Scan</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design gap, not a live failure. ask_human and create_clarification carry no tier logic (runner/companion/state_mcp.py, backend/apps/clarifications/services.py); the tier reasoning lives only in the agent prompt (backend/manifest/rules/prompt_rules.py). No validator checks a question or assumption against the hard-coded Tier-1 'never infer' category list.</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">By design, tier classification is the agent's own reasoning; there is no control-plane check. The platform records and delivers whatever tiers the agent labels, and only a human reviewer reading the gate or the Assumptions Log can catch a misclassification.</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposed (future): a platform-side validator that scans each phase's questions and assumptions for the Tier-1 'never infer' categories and auto-promotes any match to a required Tier-1 question before the gate can close - turning tier classification from 'trust the agent' into 'the platform double-checks the high-risk categories'. Not yet implemented.</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="166" spans="1:1">

</xml_diff>

<commit_message>
Updated the Bugs sheet with Architecture Phase Artifact rendering issue(Container and Component Diagrams and Table)
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="166" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{285B08F5-3480-48DB-957D-3CBD7D1D2C50}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77C94B95-75A2-4B7D-95F4-DEC09B2B7B6F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="16">
+  <futureMetadata name="XLRICHVALUE" count="17">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -151,8 +151,15 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="16"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="16">
+  <valueMetadata count="17">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -201,12 +208,15 @@
     <bk>
       <rc t="1" v="15"/>
     </bk>
+    <bk>
+      <rc t="1" v="16"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1314" uniqueCount="775">
   <si>
     <t>S.No</t>
   </si>
@@ -2178,7 +2188,7 @@
     <t>Build pipeline / Merge gate</t>
   </si>
   <si>
-    <t>1258d85</t>
+    <t>Fix landed in commit 1258d85 on develop ("Un-draft build PRs before merge + prefer real PR ref in _code_artifact") · github.com/RAGUWING369/AI-First-SDLC-App/commit/1258d85. Walk it: backend/integrations/github/codehost.py → mark_ready_for_review(); backend/orchestration/build_activities.py → merge_build_pr_core() (un-drafts before merging, because GitHub refuses to merge a draft PR with a 405). Prove it: pytest backend/tests/test_build_activities.py -k draft</t>
   </si>
   <si>
     <t>During the automated 07&lt;-&gt;08 review-and-fix loop the platform opens the build's pull request as a GitHub 'draft' PR (a draft blocks a premature human merge while review is still running). GitHub does not allow a draft PR to be merged - its merge API returns HTTP 405 (Method Not Allowed). So the moment a human approved the merge gate, the final merge step always failed. The work item got stuck at the very last step, never transitioned to done, and nothing downstream could complete. This was the single blocker stopping any build from finishing.</t>
@@ -2196,6 +2206,9 @@
     <t>Build pipeline / Review loop</t>
   </si>
   <si>
+    <t>Same fix as S.No 127 — commit 1258d85 on develop ("Un-draft build PRs before merge + prefer real PR ref in _code_artifact") · github.com/RAGUWING369/AI-First-SDLC-App/commit/1258d85. Walk it: backend/orchestration/build_activities.py → _code_artifact() (prefers the real PR ref over the agent's pre-PR pointer).</t>
+  </si>
+  <si>
     <t>The helper that looks up a build's code artifact (_code_artifact) fetched 'the first matching artifact' with no defined ordering. A single work item can have more than one code-artifact row: an early placeholder the agent registers before the PR exists, and the real one that carries the pull-request reference (repo/number/url). With no ORDER BY, the database returned rows in an arbitrary order, so the code sometimes picked the early placeholder that has no PR link. The reviewer then had nothing to look at and reported 'no opened PR to review', which broke the remediation cycle.</t>
   </si>
   <si>
@@ -2211,7 +2224,7 @@
     <t>Build pipeline / Review guard (S.No 114 guard)</t>
   </si>
   <si>
-    <t>a2deeae</t>
+    <t>Fix landed in commit a2deeae on develop ("Trust a present APPROVED verdict in the review fail-closed guard (S.No 114)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/a2deeae. Walk it: backend/orchestration/review_provider.py → parse_and_guard(). Prove it: pytest backend/tests/test_review_dispatch.py</t>
   </si>
   <si>
     <t>The review guard is deliberately 'fail-closed': if a review's prose looks like it demands changes but the structured verdict does not clearly say so, it blocks - to stop bad code slipping through. The old prose matcher (_looks_blocking) scanned the entire review text for blocking-sounding words. An APPROVED review referenced an already-RESOLVED finding by its ID (for example 'REM-W1'), and the matcher saw that mention and concluded the review was demanding changes. Result: a legitimately approved review was blocked and the build could not proceed - a false positive that halted good work.</t>
@@ -2229,7 +2242,7 @@
     <t>Companion / Pre-push secret scan</t>
   </si>
   <si>
-    <t>52533c4</t>
+    <t>Fix landed in commit 52533c4 on develop ("Surface redacted secret-scan findings on companion + in build.failed reason") · github.com/RAGUWING369/AI-First-SDLC-App/commit/52533c4. Walk it: runner/companion/runner.py (the secret-scan block that reports the redacted finding). Prove it: pytest backend/tests/test_companion_runner.py -k secret</t>
   </si>
   <si>
     <t>Before pushing code the companion (the worker on the developer machine) scans the changed files for hardcoded secrets (passwords, API keys, tokens, private keys). When it finds one it correctly blocks the push and reports the build as failed - but it only reported a bare count ('N finding(s)'). It did not surface which secret type, which file, or which line, and it then tore down the temporary work folder, so the evidence was gone. Operators saw 'build failed' with no way to know why or how to fix it, making the block undiagnosable.</t>
@@ -2265,7 +2278,7 @@
     <t>Build pipeline / Commit status reporting</t>
   </si>
   <si>
-    <t>build_activities.py:140</t>
+    <t>Code location (the old reference said build_activities.py:140, which has since ROTTED — line 140 is now unrelated `except CapabilityError` code; naming the function instead so it cannot rot again): backend/orchestration/build_activities.py → open_build_pr_core() sets set_commit_status(context="sdlc/build", state="pending") and nothing ever sets it to success/failure afterwards. Grep to see it for yourself: grep -rn 'sdlc/build' backend/orchestration/build_activities.py</t>
   </si>
   <si>
     <t>When the build PR is opened, the platform posts a GitHub commit status with context 'sdlc/build' and state 'pending' against the head commit (build_activities.py line 140, best-effort - exceptions are swallowed). Nothing anywhere later updates that status to 'success' or 'failure'. So every build's commit shows the 'sdlc/build' check stuck on pending indefinitely. It is dormant today only because no branch-protection rule on the repo currently requires the 'sdlc/build' context to be green before merging. The day someone enables such a required check, merges will be blocked forever because the status can never reach success - a latent time-bomb, and misleading status UI in the meantime.</t>
@@ -2355,7 +2368,7 @@
     <t>Tenancy / Enrollment identity</t>
   </si>
   <si>
-    <t>enrollment 32db7f5f</t>
+    <t>Evidence: a single RunnerEnrollment row is shared by two developers, so a run started by either is attributed to the same enrollment. See it for yourself — GET /api/runners/ returns one enrollment for the project (the id seen when this was logged was 32db7f5f). Code: backend/apps/runs/models.py → RunnerEnrollment (project + developer), and backend/orchestration/trigger.py → _resolve_enrollment(), which picks the enrollment for the triggering user.</t>
   </si>
   <si>
     <t>During testing it was found that two different developers are operating under the same enrollment record (enrollment id 32db7f5f, under tenant 212395b8). Enrollment is meant to identify a single developer's participation in a project; sharing one record between two people means their runs, claims and attribution can be conflated, and any per-developer isolation or accounting keyed on enrollment is wrong. It also muddies debugging (whose companion claimed what) and could let one developer's actions appear under the other's identity.</t>
@@ -2448,7 +2461,7 @@
     <t>The pre-push secret scan flagged an obvious placeholder value as a real secret, so the push was blocked and the build failed.</t>
   </si>
   <si>
-    <t>3c33554</t>
+    <t>Fix landed in commit 3c33554 on develop ("Fix secret-scan false positive on hyphenated placeholders (Bugs S.No 143)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/3c33554 (the commit message says S.No 143; the sheet row is 144 — the sheet is correct). Walk it: runner/companion/guardrails.py (the placeholder allow-list). Prove it: pytest backend/tests/test_guardrails.py -k placeholder  (scoped on purpose — running the whole file also picks up test_run_build_clean_change_reports_ok, which fails for an unrelated, pre-existing reason: it needs real git workspace access. That failure is not this fix.)</t>
   </si>
   <si>
     <t>The companion's pre-push secret scanner (runner/companion/guardrails.py) blocks a push when it finds anything that looks like a hardcoded secret. Its placeholder allow-list recognised the literal token 'changeme' but NOT the far more common hyphenated/underscored form 'change-me'. So a legitimate .env.example placeholder - JWT_SECRET=change-me-minimum-32-characters-long (36 chars, Shannon entropy 3.875) - was not recognised as a placeholder, tripped the generic high-entropy heuristic, and was flagged as a 'high_entropy_secret'. The push was blocked and the build failed. This is a FALSE POSITIVE: the value is an obvious placeholder, not a real secret. It blocked WI-32 and would block any task whose example env file uses the very common change-me convention. The build agent did nothing wrong - the scanner was too aggressive.</t>
@@ -2466,7 +2479,7 @@
     <t>Build pipeline / Failure observability + Companion</t>
   </si>
   <si>
-    <t>daemon.py:271</t>
+    <t>Fix landed in commit 6f9671f on develop ("Make AI-engine / usage-limit build failures human-readable (Bugs S.No 146)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/6f9671f. NOTE the old reference said daemon.py:271, which has ROTTED (that line is now a bare `except`); the real code is: backend/drivers/claude_driver.py (captures the engine's stderr tail) and backend/orchestration/build_activities.py → classify_build_failure() (turns a raw usage/rate-limit error into a plain-language reason). Prove it: pytest backend/tests/test_build_activities.py -k classify. This row is still marked Open — the code fix has landed but is awaiting the team's live test.</t>
   </si>
   <si>
     <t>When the AI build agent fails to run - most commonly because the Anthropic usage/rate limit is reached, but also on any agent CLI non-zero exit - the companion's error handler (runner/companion/daemon.py ~line 271) captures only the engine driver's generic wrapper string and reports it verbatim: 'Command failed with exit code 1 (exit code: 1) / Error output: Check stderr output for details'. The platform's classify_build_failure (backend/orchestration/build_activities.py) does not recognise this signature, so the raw string passes straight through to the build.failed reason and the run console. The user sees an opaque error with no indication that the real cause was a usage limit and no guidance on what to do. This bit WI-32: the usage limit was hit during the cycle-2 remediation build and the console showed only 'Command failed with exit code 1'. Same defect class as S.No 139 (classified reasons) but for the engine/usage-limit failure path, which was not covered.</t>
@@ -2476,6 +2489,15 @@
   </si>
   <si>
     <t>When the implementation of a Work Item is completed and give it away for the review agent - The review agent is doing its job and creating Remediation Work Items (if blocking or critical issues are present): The created Remediation Work Item Tasks are too technical and not humasined and high level</t>
+  </si>
+  <si>
+    <t>Evidence — reproduce on any build with blocking findings: the remediation child work items on the Work Items board show a bare title and an EMPTY description. Root of the evidence trail, verifiable by reading the code: backend/orchestration/review_provider.py → parse_findings() read only rem/severity/title/file/line and silently dropped the agent's `problem`/`fix`/`category`, and build_activities.py → run_code_review_core() created the WorkItem with no description at all — so the reviewer's words could not reach the board. The agent's own contract already emits those fields: see the verdict JSON example in agents/08_code_review/agent.md.</t>
+  </si>
+  <si>
+    <t>BOTH sides, and the PLATFORM was the hard blocker. (1) Platform: the remediation child WorkItem was created with title=finding.title and NO description at all (build_activities). Worse, the Finding dataclass had no description field and parse_findings (review_provider) SILENTLY DROPPED the agent's problem/fix/category — so even a perfectly humanized review could never reach the board; the reviewer's words were discarded before they got there. Agent 07's remediation manifest had the same hole: it was asked to fix each finding from its one-line title. (2) Agent: 08_code_review/agent.md asked for 'a concise title' with no readability directive, and its JSON example — which is what the agent actually imitates — showed terse fragments ('unbounded result set').</t>
+  </si>
+  <si>
+    <t>Mirrors the proven S.No 118 pattern. PLATFORM: Finding now carries description/problem/fix/category and parse_findings maps them through; the WorkItem gets a real humanized brief composed by _remediation_description — a plain-language severity lead, 'What's wrong', 'What to do', and a 'Where' line keeping the technical nuance (file:line, review dimension, severity, REM id). A title-only finding says so honestly instead of implying a fuller brief. _render_remediation_section now folds the same detail into agent 07's manifest. AGENT: added a 'Writing standard' to 08_code_review/agent.md mirroring 06's proven one and scoped to the verdict findings fields (title = a board item's title, problem = what is wrong AND why it matters, fix = what to actually do, self-contained, no 'see above'); made the contract explicit that title/problem/fix are read by people on the Work Items board and are required on every blocking finding; REWROTE the JSON example into properly humanized findings. Audience is a developer, so the bar is 06's: plain language that keeps the technical nuance. Tests: parse_findings carries the fields + tolerates a detail-less finding; the composed description; the child WI end-to-end; the 07 brief. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/orchestration/review_provider.py → parse_findings() (now carries problem/fix/category); backend/orchestration/build_activities.py → Finding, _remediation_description() (builds the brief), _render_remediation_section() (gives agent 07 the same detail); agents/08_code_review/agent.md → 'Writing standard' + the rewritten verdict JSON example. Prove it: pytest backend/tests/test_build_activities.py -k remediation and pytest backend/tests/test_build_agents_migration.py -k parse_findings</t>
   </si>
   <si>
     <t>In Implementation Phase:
@@ -2501,13 +2523,31 @@
 Currently all created Work Items are shown in a drop down but if the created work items count reaches huge number it would be difficult for the user to find his work item. Instead we will give him a search option in the drop down itself - this way he can search for his work item and use the drop down also.</t>
   </si>
   <si>
+    <t>PhasesAndRuns rendered a plain native &lt;Select&gt; listing every work item in the project (~54), so finding one meant scrolling and eyeballing the list. The UI kit had only Input and Select — no Combobox/Autocomplete existed, so a searchable picker had to be built, not just wired up.</t>
+  </si>
+  <si>
+    <t>Built a small reusable Combobox in the UI kit (team's choice over a filter box or a native &lt;datalist&gt;): type to filter the list in the dropdown itself, arrow keys move, Enter picks, Esc closes/reverts, click-outside closes, and it uses the standard combobox ARIA roles so screen readers announce it. Reuses the .input frame + .select chevron so it looks identical to the other controls, and says 'No work items match' rather than showing an empty box. Swapped into the Phases &amp; Runs work-item picker; available for any other long list. Tests (Combobox.test.tsx): filters as you type + click to pick, keyboard operable, empty-state, and shows the current selection when closed. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: frontend/src/components/ui/index.tsx → Combobox (new reusable component); frontend/src/features/lifecycle/PhasesAndRuns.tsx (the picker now uses it); frontend/src/styles/components.css (.combobox*). Prove it: cd frontend &amp;&amp; npx vitest run src/components/ui/Combobox.test.tsx</t>
+  </si>
+  <si>
     <t>In the Artifacts &amp; Traceability page:
 1. The artifacts names for Code review, PR - should have task title/name to identify easily instead of only WI-ID
 Note: See the reference image for clarity</t>
   </si>
   <si>
+    <t>work_item_key is a BRANCH SLUG, not a display name (build_types: 'branch name + run prompt'). trigger.py builds it as caller-supplied -&gt; the Jira id (TASK-001) -&gt; a fallback of 'WI-&lt;first 8 chars of the uuid&gt;'. Three places used it as a title: the Code Review artifact, the Code artifact, and the GitHub PR title (so it leaked to the system of record too). Rows that looked fine were agent-authored: open_build_pr / run_code_review are register-don't-recreate and never overwrite the agent's title — so bad names were always the platform's own fallback. The frontend was NOT at fault (artifactLabel already prefers the title).</t>
+  </si>
+  <si>
+    <t>Added work_item_title to BuildInput, populated in trigger.py from work_item.title, and a display_name() helper that prefers the title and falls back to the key only when there is no title. The Code artifact, the Code Review artifact and the PR title now read the task title; work_item_key still names the branch, and the PR body carries it for traceability. Passed on the input rather than read from the DB inside the activity, so activities stay deterministic for Temporal replay. Tests: display_name prefers the title / falls back on blank+whitespace; artifacts + PR title carry the task title while the key stays in the body. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/orchestration/build_types.py → BuildInput.work_item_title + display_name(); backend/orchestration/trigger.py (populates it from work_item.title); backend/orchestration/build_activities.py → open_build_pr_core() (PR title + Code artifact) and run_code_review_core() (Code Review artifact). Prove it: pytest backend/tests/test_build_activities.py -k "display_name or task_title"</t>
+  </si>
+  <si>
     <t>When the user approved the gate for implementation pahse - The artifacts: Assumptions, Implementation task/WI are still in draft state not published.
 Note: See the reference image for clarity</t>
+  </si>
+  <si>
+    <t>The BUILD path had no publish step at all. The planning path has publish_artifacts_core, which publishes EVERY artifact of the run; the build path published exactly one — merge_build_pr_core grabbed only the single type='code' row. Grepping Status.PUBLISHED across orchestration returned only those two hits, so nothing else COULD publish them: the Assumptions and Code Review artifacts stayed Draft forever even though their gate was approved. Not intentional — 'internal' is those artifacts' SoR, not a lifecycle status, and the planning path deliberately publishes internal-SoR artifacts. A gap, not a decision.</t>
+  </si>
+  <si>
+    <t>Added publish_build_artifacts_core mirroring the planning path's publish_artifacts_core and called it from BuildWorkflow after merge_build_pr: it publishes every artifact of the run, skips already-published ones, and takes an immutable S3 audit snapshot of any body-bearing artifact. It changes ONLY `status` — each artifact already carries its correct SoR from registration (code -&gt; git, review -&gt; internal), so this is structurally incapable of clobbering the code pointer's sor=git. Run.status=COMPLETED and the artifacts.published event moved out of merge into publish, so a run can no longer report 'completed' while its artifacts are still draft; merge now performs only the gated SoR write. Idempotent for Temporal retries/replays. Tests: publishes all three artifact types (not just code), sor=git + the PR pointer survive, snapshot written, idempotent, and the merge/publish split; the phase-2 acceptance replay test was extended through the new step. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/orchestration/build_activities.py → publish_build_artifacts_core() (new; mirrors the planning path's publish_artifacts_core in backend/orchestration/activities.py — compare them side-by-side) and merge_build_pr_core() (now does only the gated write); backend/orchestration/build_workflow.py (calls publish_build_artifacts after the merge). Prove it: pytest backend/tests/test_build_activities.py -k publish_build</t>
   </si>
   <si>
     <t>The user should be able to edit the generated phase artifacts - Task Breakdown phase, requirements phase, PRD phase etc. Right now the edit artifacts capability is missing.</t>
@@ -2525,11 +2565,149 @@
 2. THe user should test the integration connection first and then save the creds not the other way around.</t>
   </si>
   <si>
+    <t>Evidence (1) rotation deadlock — Integrations → any configured capability → the secret field renders a disabled 'configured' box with no way to type a new value; the input was gated on secrets[field] being non-empty while the only control that could set it was that same input (frontend/src/features/setup/ConnectCapability.tsx). Evidence (2) DATA LOSS, reproduced by a test written BEFORE the fix — PATCH /api/integrations/{id}/ with {"binding": {...}, "secrets": {}} (exactly what the drawer sends when you edit a configured connection without retyping the token) returned 200 with configured=False and the stored token destroyed. Verbatim failure: `assert resp.data["configured"] is True` -&gt; `assert False is True`. Re-run it yourself: pytest backend/tests/test_integrations_admin.py -k empty_secrets_object. Evidence (3) not-a-live-probe — the old docstring on backend/apps/integrations/services.py → test_integration_connection() stated it proves the pair is 'constructible and a secret has been stored, not that the upstream API is currently reachable'.</t>
+  </si>
+  <si>
+    <t>TWO independent causes, plus a latent data-loss bug found while investigating. (1) ROTATION — a UI deadlock; the backend was always fine (update_integration happily re-encrypts a new secret). ConnectCapability rendered the editable secret input ONLY when secrets[field] was already non-empty — and the only control that could set it was that very input, so it could never appear. The help text 'Enter a new value only to rotate it' described something unreachable. (2) TEST-BEFORE-SAVE — test_integration_connection was NOT a live probe (its own docstring said it proves the capability+vendor pair is constructible and a secret is stored, not that the API is reachable), AND the endpoint was detail=True + get_object(), so it structurally REQUIRED a saved row: that is why saving first was forced. (3) DATA LOSS (latent, proven by a failing test before fixing): the drawer sends secrets:{} whenever an admin edits a configured connection without retyping the token (e.g. changing only the project key). {} is not None, so update_integration re-encrypted an empty dict and SILENTLY WIPED the stored credential — the test showed `configured` flipping to False.</t>
+  </si>
+  <si>
+    <t>(1) Rotation: an explicit `rotating` state + a Replace button next to the Configured badge (and Cancel to keep the stored value), which breaks the deadlock; secretsComplete now requires a value only once a rotation is actually opened, so Save is never blocked by a cancelled one. (2) Data loss fixed on BOTH ends: the frontend omits the `secrets` key entirely when nothing was typed, and the server treats an empty object as 'no change' rather than 'erase' (there is deliberately no way to blank a secret via PATCH — disconnect to remove). Regression test added. (3) Test-before-save: extracted a pure probe_connection() that writes nothing to the DB, and added POST /api/integrations/test-credentials/ (detail=False) which probes a throwaway in-memory connection that is NEVER saved; test-connection still probes a saved row and records health. The frontend dropped its !savedId guard and tests as-typed credentials. (4) REAL live probes via a capability-seam ping() on Jira (/rest/api/3/myself), GitHub (/user), Confluence (/rest/api/user/current) and Figma (/v1/me) — cheap, read-only 'who am I' calls that touch no project data; vendor errors are translated into actionable messages (401/403 -&gt; credentials rejected, 404 -&gt; check the site URL, 429 -&gt; rate-limited, 5xx -&gt; vendor down). Xray keeps the wiring-only check and SAYS SO ('no live check for this vendor') rather than implying reachability. NOTE — BEHAVIOR CHANGE: Test connection now makes a real authenticated call, so credentials that used to pass the constructible-only check will now fail if they are wrong; that is the point of the fix. Two pre-existing #39 tests saved dummy creds and asserted ok=True; their intent was 'the catalog slug resolves to a registered, constructible connector', never reachability, so they now assert the failure is not a registry-miss/build error. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/apps/integrations/services.py → probe_connection() (new pure core, no DB writes), test_credentials() (unsaved in-memory probe), update_integration() (empty secrets = no change); backend/api/views.py → IntegrationViewSet.test_credentials_action (POST /api/integrations/test-credentials/); the ping() methods on integrations/atlassian/tasktracker.py, atlassian/docstore.py, github/codehost.py, figma/designsource.py; frontend/src/features/setup/ConnectCapability.tsx (rotating state + Replace). Prove it: pytest backend/tests/test_integrations_admin.py</t>
+  </si>
+  <si>
     <t>In the SDLC APP Phases and Runs: After any phase (mainly Build Phase but applies to all phases) trigger is interrupted due to any error/issue, the user should be able to continue from that point rather than starting from beginning of that phase. 
 Note: This is a very user important fix - should be applied accurately.</t>
   </si>
   <si>
     <t>Phases and Runs</t>
+  </si>
+  <si>
+    <t>Evidence — reproduce: trigger a build, make the merge fail for a non-conflict reason (e.g. a branch-protection rule on the base), and the run goes terminally FAILED; the only way forward is re-triggering, which re-runs the WHOLE build from step 1. Why it was unavoidable, verifiable in code: backend/orchestration/build_workflow.py called mark_build_failed and RETURNED, which closes the Temporal workflow — and a closed workflow can never be signalled, so there was nothing left to resume. Check the Temporal history of any failed build: it ends at that activity. Note run.inputs (backend/apps/runs/models.py) is never written — there was no checkpoint anywhere.</t>
+  </si>
+  <si>
+    <t>On any error both workflows called mark_build_failed/fail_run and RETURNED — which CLOSES the Temporal history for good. A closed workflow can never be signalled, so there was nothing left to resume: the only way forward was trigger_build/trigger_phase creating a brand-new Run + workflow from step 1, re-doing the expensive build. No checkpoint existed anywhere (run.inputs is never written). Note Temporal ALREADY retries transient activity errors (3 attempts) — that was never the gap; the gap was the terminally-closed workflow.</t>
+  </si>
+  <si>
+    <t>The workflow now PARKS instead of dying — the same pattern already proven three times here (ENH-2's merge-gate loop S.No 141, the S.No 89 non-terminal STALLED park, and the abandon_run signal). New idempotent activities park_build/park_run (STALLED + a classified reason + the step to resume from) and resume_build/resume_run_state (back to RUNNING, markers cleared), plus a _park() helper in both workflows that waits (human-paced, no timeout) for `resume_run` or `abandon_run`. Wired to: BuildWorkflow's PR/review/gate-setup errors and NON-conflict merge errors, and AgentRunWorkflow's verify_writes. dispatch_build sits OUTSIDE the retry loop, so the build itself is NEVER redone; every retried step is idempotent (open_build_pr register-don't-recreate, open_merge_gate get_or_create). A merge error resumes under the SAME approval — clicking Resume IS the human action. ENH-2's conflict loop is preserved untouched, and abandon reuses today's exact terminal path, so the worst case is today's behavior. EmptyBuild stays terminal (is_empty_build): the agent produced no changes, so resuming would fail identically forever. New POST /api/runs/{id}/resume/ + resume_stalled_run (modelled on take-over/; fires only for a run parked at a resumable error, never an S.No 89 companion-offline park). RunConsole shows the reason + 'Resume from where it stopped' / 'Take over instead'. No workflow.patched needed: the changes are on exception paths, and a workflow that had taken one would already have completed. Tests: park/resume idempotency + marker clearing, is_empty_build, resume refusing a companion-offline park, and three live-Temporal saga tests (merge-error -&gt; park -&gt; resume -&gt; merge with no rebuild; abandon -&gt; terminal; empty-build -&gt; never parked). — REVIEW THE FIX: landed in commit d12d9c7 on develop ("Resume an interrupted phase instead of restarting it (Bugs S.No 157)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/d12d9c7. Walk it: backend/orchestration/build_workflow.py → BuildWorkflow._park() + the resume_run/abandon_run signals; backend/orchestration/build_activities.py → park_build_core()/resume_build_core(); backend/orchestration/workflows.py → AgentRunWorkflow._park(); backend/orchestration/activities.py → park_run_core()/resume_run_state_core(); backend/orchestration/takeover.py → resume_stalled_run(); backend/api/views.py → RunViewSet.resume (POST /api/runs/{id}/resume/); build_types.py → is_empty_build(); frontend/src/features/lifecycle/RunConsole.tsx (Resume button). Prove it: pytest backend/tests/test_build_activities.py -k "park or resume or empty_build" and pytest backend/tests/test_phase_dispatch.py -k "park or resume". Live saga tests (need Temporal on localhost:7233, run ONE at a time — the file OOMs if run whole): pytest backend/tests/test_build_workflow.py::test_build_workflow_merge_error_parks_then_resumes_without_rebuilding</t>
+  </si>
+  <si>
+    <t>A phase run can fail with no reason shown at all — the run console says it failed but the failure line is empty</t>
+  </si>
+  <si>
+    <t>Found while investigating S.No 157. When the write-completeness check (verify_writes) rejects a phase, the run shows as failed but the console shows NO reason — the user is told only that something went wrong, with nothing to act on. Every other failure path records a readable reason; this one recorded nothing.</t>
+  </si>
+  <si>
+    <t>Evidence — reproduce: run a phase whose expected artifact is not registered, so the write-completeness check rejects it. The run console shows the run FAILED with an empty failure line — no reason at all. Verifiable in code: backend/orchestration/workflows.py ran verify_writes with RetryPolicy(maximum_attempts=1) and nothing caught its error, so the workflow crashed before fail_run — and fail_run is the only thing that writes run.outputs.error, which is exactly the field frontend/src/features/lifecycle/RunConsole.tsx reads for that line. Not a display bug: the reason was never recorded. Found while investigating S.No 157.</t>
+  </si>
+  <si>
+    <t>verify_writes runs with RetryPolicy(maximum_attempts=1) and NOTHING caught its error, so the exception propagated and CRASHED AgentRunWorkflow before fail_run could run. fail_run is the only thing that writes run.outputs.error — and RunConsole reads exactly that field for its failure line — so the run was left FAILED with an empty reason. Not a display bug: the reason was never recorded anywhere.</t>
+  </si>
+  <si>
+    <t>Fixed by the same change as S.No 157: verify_writes is now wrapped, and its failure PARKS the run via park_run, which always records the classified reason on run.outputs.error. So the console now shows the real reason, and the user can Resume to re-check once the missing artifact is registered instead of re-running the whole phase. Test: park_run_core records the reason and stays non-terminal. — REVIEW THE FIX: landed in commit d12d9c7 on develop ("Resume an interrupted phase instead of restarting it (Bugs S.No 157)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/d12d9c7 (same change as S.No 157). Walk it: backend/orchestration/workflows.py (verify_writes is now wrapped in try/except and parks instead of crashing) → backend/orchestration/activities.py → park_run_core() (always records the classified reason on run.outputs.error). Prove it: pytest backend/tests/test_phase_dispatch.py -k park_run_core</t>
+  </si>
+  <si>
+    <t>Test connection reports OK without checking the repo address it was given - a mistyped repo still shows a green tick, and nothing validates it until the build phase fails</t>
+  </si>
+  <si>
+    <t>Found live on 2026-07-17 while setting up tenant SpendLog-2 (Edvensoft-2) for the fresh single-repo end-to-end retest. The Code Host repo was saved as 'RAGUWING369/ SpendLog-2-single-repo-refresh-test' - a stray SPACE after the slash. Test connection reported success and health was written 'healthy', because the probe only asks GitHub 'who am I' (GET /user) and, by its own docstring, 'touches no repository'. The repo address - the one field the whole build depends on - is never resolved. The typo is harmless through ideation / requirements / PRD / architecture / UX / task breakdown (none of them touch the repo), and would only surface at the build phase, AFTER a full planning run, when GitHubCodeHost._repo() passes the string straight into the request path (GET /repos/RAGUWING369/ SpendLog-2-single-repo-refresh-test/branches/main) with no strip/normalisation - a 404 on a malformed URL. Same class of defect as S.No 156, one level up: 156 upgraded the probe from 'is the connector constructible' to 'is the token real' precisely because the old check 'reported OK for a mistyped token, which is exactly what a connection test exists to catch'. A mistyped REPO now reports OK for the same reason. Not GitHub-specific: the same gap applies to any connector with a configured target (Jira project key, Confluence space, Figma file, Xray).</t>
+  </si>
+  <si>
+    <t>Integrations / Code Host / Connection test</t>
+  </si>
+  <si>
+    <t>Evidence - reproduce: in Integrations &gt; Code Host, save a repo with a typo (e.g. a space after the slash: 'OWNER/ repo-name'), then click Test connection.
+Observed: Test connection PASSES ('Signed in to GitHub as RAGUWING369.') and IntegrationConnection.health is written 'healthy', while scopes['repo'] still holds the invalid address. No warning anywhere. Live record on tenant 7828e953-987e-43b2-8d5f-c8a45bfa8c6a at 11:17-11:59 held scopes={'repo': 'RAGUWING369/ SpendLog-2-single-repo-refresh-test'} with health reported OK.
+Proof the probe cannot catch it - GitHubCodeHost.ping() in backend/integrations/github/codehost.py issues only GET /user and its docstring states it 'touches no repository'. probe_connection() in backend/apps/integrations/services.py calls exactly that ping() and returns {ok: True} on success.
+Proof the address is never normalised - GitHubCodeHost._repo() returns the configured string unchanged (no .strip()); callers such as get_branch() / open_pull_request() interpolate it directly into '/repos/{repo}/...'.
+Proof a real check is cheap and would have caught it - with the space removed, the same connector resolves the repo for real:
+  ch.ping()             -&gt; 'Signed in to GitHub as RAGUWING369.'
+  ch.get_branch(name='main') -&gt; BranchRef(sha=e252eaedb3, url=https://github.com/RAGUWING369/SpendLog-2-single-repo-refresh-test/tree/main)
+The identical call against the space version raises a 404. One extra read-only call is the whole difference.</t>
+  </si>
+  <si>
+    <t>probe_connection() validates CREDENTIALS only; it has no notion of the connection's configured TARGET. ping() is deliberately scoped to a cheap 'who am I' that touches no repository, and nothing else in the setup path resolves scopes['repo']. The first code that touches the repo address is the build phase, so a setup typo stays invisible until then. Compounding it, GitHubCodeHost._repo() does not strip or validate the string, so whitespace survives into the URL.</t>
+  </si>
+  <si>
+    <t>OPEN - not fixed, logged for completeness at the team's request (2026-07-17); typo corrected by hand on SpendLog-2 so the retest could proceed. Proposed: extend probe_connection() so that where a connection carries a configured target, the probe resolves THAT too, not just /user - for codehost, a read-only get_branch(default_base) or GET /repos/{repo}; the connector already exposes everything needed. Report it as its own line ('Signed in as X; repo Y found') so the admin sees both facts. Keep it capability-generic (Jira project key, Confluence space, Figma file), not a GitHub special case, and reuse _probe_failure_detail() - its existing 404 wording ('Authenticated, but that address isn't right - check for typos') is already almost exactly the message this needs. Cheap hardening worth doing at the same time: strip the repo string on save in create_integration()/update_integration() and in GitHubCodeHost._repo(), and reject an address that is not OWNER/NAME shaped. Related: S.No 156 (same principle, one level down).</t>
+  </si>
+  <si>
+    <t>The platform silently DISCARDS the agent's entire phase document and reports its cost as zero: every artifact the platform files itself is 0 bytes, and the gate opens on a blank page</t>
+  </si>
+  <si>
+    <t>Found live on 2026-07-17 on tenant SpendLog-2 (Edvensoft-2), run 2894a1e0 - the first ideation of the fresh single-repo retest. The companion ran the 01_ideation agent for ~6 minutes and reported a 34,474-character document costing $0.397562. The platform stored a 0-BYTE draft, content_hash = sha256 of the empty string, and run.cost_usd = 0.0. verify_writes then PASSED (it only checks that an artifact of the expected TYPE exists, never that it has content) and the gate opened on a blank document, asking a human to approve nothing. Temporal shows a clean history with no failure anywhere: the run looks perfect from every angle the platform reports on.
+SCOPE - this bites ONLY the platform's own fallback registration, which is why it hid for so long. When the agent registers its artifacts itself (register_artifact + stage_artifact_body over MCP), that path stages the body and the artifact is fine. Across the three live tenants: SpendLog-1 56 artifacts / 1 empty; Edvensoft 170 / 2 empty; SpendLog-2 1 / 1 empty. The empties are exactly the phase-typed artifacts the platform created itself - e.g. Edvensoft 'testing/testing' empty at 08:26 on 2026-07-17 while its sibling test_case / test_report artifacts, which the agent registered, have real bodies. On run 2894a1e0 the agent registered NOTHING, so the broken fallback carried the whole phase and the loss was total.
+AGGRAVATING - the phase.empty_result event blames the ENGINE for the platform's own bug: 'companion reported ok but the engine returned no final text', when the engine had in fact returned 34,474 characters. That message sent this investigation down the wrong path for a considerable time.</t>
+  </si>
+  <si>
+    <t>Orchestration / Phase result registration / Artifacts</t>
+  </si>
+  <si>
+    <t>Evidence - reproduce: run any planning phase on the companion in which the agent does not register the phase artifact itself. The staged draft is 0 bytes and the run's cost is 0.0, while the companion's report holds the real body and cost.
+Observed live (run 2894a1e0, tenant 7828e953-987e-43b2-8d5f-c8a45bfa8c6a):
+  run.outputs['report'] = {'status':'ok', 'body': &lt;34474 chars&gt;, 'cost_usd': 0.397562, 'message': ''}
+  run.outputs['cost_usd'] = 0.0                    &lt;- should be 0.397562
+  run.cost_usd            = 0.0000                 &lt;- should be 0.3976
+  artifact e619681e: content_hash = sha256:e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855
+                     (that is the sha256 of the EMPTY string), title = '', status = draft
+  S3 drafts/&lt;tenant&gt;/&lt;project&gt;/2894a1e0-.../ideation.md -&gt; get() returns b'', length 0
+The COST is the decisive proof: 0.397562 arrived and 0.0 was stored. Only a defaulted read explains both fields going wrong at once, from one line.
+Ledger events for the run, in order: run.triggered 12:09:24 / phase.dispatched 12:09:28 / phase.reported 12:15:32 {'status':'ok'} / run.executed 12:15:36 / phase.empty_result 12:15:36 'companion reported ok but the engine returned no final text; the staged phase draft is empty' (FALSE - see Description) / gate.opened 12:15:38.
+Temporal history (agent-run-2894a1e0-6b6f-4772-9b0a-cc7ad8d4376f on 13.203.56.29:7233): #5 compose_manifest, #11 dispatch_phase, #18 SIGNAL phase_reported, #23 register_phase_result, #29 verify_writes, #35 open_gate. No failures.
+Code location - register_phase_result_core() in backend/orchestration/activities.py read the report with getattr(report,'body',''), getattr(report,'cost_usd',0.0) and getattr(report,'message',''), while register_phase_result_activity(inp: AgentRunInput, report) left `report` UNANNOTATED. It was the ONLY unannotated activity parameter in backend/orchestration (whole package scanned).
+Why the tests never caught it - every existing test in backend/tests/test_phase_dispatch.py passes a real PhaseReport dataclass straight into the core, a shape production never sends; the dict only appears once the argument crosses Temporal. Proof the new regression test reproduces it: on the pre-fix code it fails with  assert b'' == b'# PRD\nreal body'.</t>
+  </si>
+  <si>
+    <t>Temporal's data converter converts an activity argument to the type its parameter is ANNOTATED with, and hands an UNANNOTATED parameter back as the raw decoded JSON - a plain dict. register_phase_result_activity annotated `inp: AgentRunInput` (which is exactly why inp always worked) but left `report` bare, so the PhaseReport arrived as a dict. register_phase_result_core then read it with getattr, which looks up an ATTRIBUTE - a dict has none - so getattr returned its DEFAULT for every field: body '' and cost_usd 0.0. Nothing raised. The defaults are indistinguishable from an engine that genuinely produced nothing, which is precisely what the phase.empty_result message then asserted.
+verify_writes could not save it either: verify_write_completeness_core asserts only that an artifact of the expected TYPE exists, never that its body is non-empty - so the platform's own 0-byte row satisfied the last check before the gate.</t>
+  </si>
+  <si>
+    <t>IN PROGRESS (2026-07-17) - fixed locally, NOT committed, pending team test. Three parts, all in backend/orchestration/activities.py:
+1. ROOT FIX - annotate the activity: register_phase_result_activity(inp: AgentRunInput, report: PhaseReport). Temporal now converts the payload to a PhaseReport, matching the `inp` parameter that always worked. A test asserts the annotation stays put, so it cannot be silently dropped again.
+2. DEFENCE - new _as_phase_report() coerces dict / PhaseReport / duck-typed object to a PhaseReport, and the core reads report.body / report.cost_usd / report.message directly - no getattr on a possible dict anywhere in the path. The cores are also called directly by tests and by the takeover path, so both shapes must keep working.
+3. HONESTY - the phase.empty_result message no longer reads the report via getattr, so it can no longer blame the engine for the platform's own defaulted read.
+Tests (backend/tests/test_phase_dispatch.py): test_register_phase_result_core_reads_a_dict_report sends the exact wire shape Temporal delivers and asserts the body is staged, the hash is not the empty-file hash, and the cost survives (run.cost_usd is a 4dp Decimal column, so the stored value is the rounded 0.3976). test_register_phase_result_activity_annotates_its_report_param guards the root fix. Both fail on the pre-fix code and pass after.
+Verified: test_phase_dispatch 26 passed / 3 skipped; test_orchestration_activities + test_acceptance_phase45 + test_acceptance_phase47 = 14 passed / 1 failed, that 1 being the PRE-EXISTING test_offline_companion_parks_for_takeover, which fails identically without this change (logged as S.No 161).
+NOT fixed here, deliberately: verify_writes still passes an empty artifact (it checks type presence, not content). Logged separately so the last line of defence is fixed on its own merits rather than as a side effect. Related: S.No 59 (the other half of this seam - pointer-only artifacts never staged), S.No 158 (verify_writes crash).</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Clarification gate surfaced only Tier-1 (must-ask) questions - Tier-2 suggestions and Tier-3 inferences never reached the user</t>
+  </si>
+  <si>
+    <t>The SDLC app promises a human is always in the loop and the platform never silently assumes. But agents classified each context gap into three tiers and only surfaced Tier 1 through the clarifications gate. Tier 2 (the agent's own suggestions) was written inline inside the deliverable, and Tier 3 (industry-standard inferences) was logged silently as assumptions the user never saw. So the user could not confirm or override the agent's Tier-2/3 choices, and the 'no silent assumptions' assurance was only partly true.</t>
+  </si>
+  <si>
+    <t>Clarifications / Context Gap Scan</t>
+  </si>
+  <si>
+    <t>Observed live across Ideation, Requirements and PRD runs on tenant Edvensoft-2: every phase logged Tier-3 items as assumptions and opened 0 clarifications, so the user never saw the agent's inferences. Verified in code: ask_human was the only human-question touchpoint and the shared rules told agents to front-load only Tier 1 and Tier 2. Retested after the fix on a live UX-design run - a single gate now shows Tier 1/2/3 sections.</t>
+  </si>
+  <si>
+    <t>The behaviour lived in the shared agent rules (backend/manifest/rules/prompt_rules.py): agents were told to 'front-load ALL Tier-1 and Tier-2 questions' and to record every Tier-3 inference silently as an assumption. Only Tier 1 was required/blocking; nothing surfaced Tier 2 or Tier 3 through the clarifications gate. The tier definitions were also thin (one line each), so classification was inconsistent.</t>
+  </si>
+  <si>
+    <t>Reworked the shared rules so the agent front-loads ALL three tiers into ONE clarifications gate before starting work, each question tagged with its tier. Tier 1 stays required; Tier 2/3 are optional and carry the agent's proposed answer as a pre-filled 'suggestion' the user can accept, edit or override, with an 'Accept all' one-click. Any untouched Tier-2/3 item falls back to the suggestion, and the confirmed Tier-3 values are still recorded as assumptions for provenance. Also strengthened the tier definitions (a four-question test plus concrete examples per tier). The web gate groups questions under Tier 1/2/3 headers. No DB migration (questions are stored as JSON). Landed on develop in commit 0c19292; backend + frontend tests, type-checks and lint all pass; user-tested on a live UX-design run.</t>
+  </si>
+  <si>
+    <t>Platform does not verify the agent's tier classification - a mislabelled Tier-1 gap can still slip through as a Tier-3 guess</t>
+  </si>
+  <si>
+    <t>Even with all three tiers now surfaced in the gate, the platform trusts the agent's own Tier 1/2/3 labelling. If the agent wrongly files a business-critical gap (for example pricing, compliance or a third-party integration) as a Tier-3 inference, it is shown pre-filled and quietly accepted rather than hard-asked. So the 'never assume' assurance still depends on the agent classifying correctly and the human reviewer noticing at the gate.</t>
+  </si>
+  <si>
+    <t>Design gap, not a live failure. ask_human and create_clarification carry no tier logic (runner/companion/state_mcp.py, backend/apps/clarifications/services.py); the tier reasoning lives only in the agent prompt (backend/manifest/rules/prompt_rules.py). No validator checks a question or assumption against the hard-coded Tier-1 'never infer' category list.</t>
+  </si>
+  <si>
+    <t>By design, tier classification is the agent's own reasoning; there is no control-plane check. The platform records and delivers whatever tiers the agent labels, and only a human reviewer reading the gate or the Assumptions Log can catch a misclassification.</t>
+  </si>
+  <si>
+    <t>Proposed (future): a platform-side validator that scans each phase's questions and assumptions for the Tier-1 'never infer' categories and auto-promotes any match to a required Tier-1 question before the gate can close - turning tier classification from 'trust the agent' into 'the platform double-checks the high-risk categories'. Not yet implemented.</t>
+  </si>
+  <si>
+    <t>The team has observed that in the Architecture phase of System Architecure artifact: The container and component diagrams are not rendered properly and also NFR-to-Architecture Traceability Matrix Table is over entended not fitted in the designated window. 
+Note: The above issue is observed for tenant - test2@edvensoft.com but the same issues are not present for the tenant - test@edvensoft.com. You must go through both the tenant Architecture Phase - System architecture artifact to confirm and come up with the best fix.
+Important Note: The same issues might be come up in later phases or will be observed (definitive chance) - so we need a surgical fix not temporary.</t>
   </si>
 </sst>
 </file>
@@ -3373,7 +3551,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="16">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="17">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -3438,6 +3616,10 @@
     <v>15</v>
     <v>5</v>
   </rv>
+  <rv s="0">
+    <v>16</v>
+    <v>5</v>
+  </rv>
 </rvData>
 </file>
 
@@ -3468,6 +3650,7 @@
   <rel r:id="rId14"/>
   <rel r:id="rId15"/>
   <rel r:id="rId16"/>
+  <rel r:id="rId17"/>
 </richValueRels>
 </file>
 
@@ -7522,10 +7705,8 @@
       <c r="E128" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fix landed in commit 1258d85 on develop ("Un-draft build PRs before merge + prefer real PR ref in _code_artifact") · github.com/RAGUWING369/AI-First-SDLC-App/commit/1258d85. Walk it: backend/integrations/github/codehost.py → mark_ready_for_review(); backend/orchestration/build_activities.py → merge_build_pr_core() (un-drafts before merging, because GitHub refuses to merge a draft PR with a 405). Prove it: pytest backend/tests/test_build_activities.py -k draft</t>
-        </is>
+      <c r="F128" s="2" t="s">
+        <v>615</v>
       </c>
       <c r="G128" s="2" t="s">
         <v>13</v>
@@ -7556,19 +7737,17 @@
       <c r="E129" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Same fix as S.No 127 — commit 1258d85 on develop ("Un-draft build PRs before merge + prefer real PR ref in _code_artifact") · github.com/RAGUWING369/AI-First-SDLC-App/commit/1258d85. Walk it: backend/orchestration/build_activities.py → _code_artifact() (prefers the real PR ref over the agent's pre-PR pointer).</t>
-        </is>
+      <c r="F129" s="2" t="s">
+        <v>621</v>
       </c>
       <c r="G129" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H129" s="2" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="I129" s="2" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="J129" s="2" t="s">
         <v>16</v>
@@ -7579,30 +7758,28 @@
         <v>129</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F130" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fix landed in commit a2deeae on develop ("Trust a present APPROVED verdict in the review fail-closed guard (S.No 114)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/a2deeae. Walk it: backend/orchestration/review_provider.py → parse_and_guard(). Prove it: pytest backend/tests/test_review_dispatch.py</t>
-        </is>
+      <c r="F130" s="2" t="s">
+        <v>627</v>
       </c>
       <c r="G130" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H130" s="2" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="I130" s="2" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="J130" s="2" t="s">
         <v>16</v>
@@ -7613,30 +7790,28 @@
         <v>130</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fix landed in commit 52533c4 on develop ("Surface redacted secret-scan findings on companion + in build.failed reason") · github.com/RAGUWING369/AI-First-SDLC-App/commit/52533c4. Walk it: runner/companion/runner.py (the secret-scan block that reports the redacted finding). Prove it: pytest backend/tests/test_companion_runner.py -k secret</t>
-        </is>
+      <c r="F131" s="2" t="s">
+        <v>633</v>
       </c>
       <c r="G131" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H131" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="I131" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="J131" s="2" t="s">
         <v>16</v>
@@ -7647,28 +7822,28 @@
         <v>131</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G132" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="2" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="I132" s="2" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="J132" s="2" t="s">
         <v>16</v>
@@ -7679,30 +7854,28 @@
         <v>132</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Code location (the old reference said build_activities.py:140, which has since ROTTED — line 140 is now unrelated `except CapabilityError` code; naming the function instead so it cannot rot again): backend/orchestration/build_activities.py → open_build_pr_core() sets set_commit_status(context="sdlc/build", state="pending") and nothing ever sets it to success/failure afterwards. Grep to see it for yourself: grep -rn 'sdlc/build' backend/orchestration/build_activities.py</t>
-        </is>
+      <c r="F133" s="2" t="s">
+        <v>645</v>
       </c>
       <c r="G133" s="2" t="s">
         <v>23</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="I133" s="2" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="J133" s="2" t="s">
         <v>141</v>
@@ -7713,28 +7886,28 @@
         <v>133</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G134" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H134" s="2" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="I134" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="J134" s="2" t="s">
         <v>16</v>
@@ -7745,28 +7918,28 @@
         <v>134</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G135" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H135" s="2" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="I135" s="2" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="J135" s="2" t="s">
         <v>16</v>
@@ -7777,28 +7950,28 @@
         <v>135</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F136" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G136" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H136" s="2" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="I136" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="J136" s="2" t="s">
         <v>141</v>
@@ -7809,10 +7982,10 @@
         <v>136</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D137" s="2" t="s">
         <v>614</v>
@@ -7821,16 +7994,16 @@
         <v>12</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G137" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="I137" s="2" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="J137" s="2" t="s">
         <v>16</v>
@@ -7841,28 +8014,28 @@
         <v>137</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G138" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="I138" s="2" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="J138" s="2" t="s">
         <v>16</v>
@@ -7873,30 +8046,28 @@
         <v>138</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F139" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence: a single RunnerEnrollment row is shared by two developers, so a run started by either is attributed to the same enrollment. See it for yourself — GET /api/runners/ returns one enrollment for the project (the id seen when this was logged was 32db7f5f). Code: backend/apps/runs/models.py → RunnerEnrollment (project + developer), and backend/orchestration/trigger.py → _resolve_enrollment(), which picks the enrollment for the triggering user.</t>
-        </is>
+      <c r="F139" s="2" t="s">
+        <v>675</v>
       </c>
       <c r="G139" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="2" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="I139" s="2" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="J139" s="2" t="s">
         <v>141</v>
@@ -7907,28 +8078,28 @@
         <v>139</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G140" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="I140" s="2" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="J140" s="2" t="s">
         <v>16</v>
@@ -7939,28 +8110,28 @@
         <v>140</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="G141" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="I141" s="2" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="J141" s="2" t="s">
         <v>141</v>
@@ -7971,28 +8142,28 @@
         <v>141</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G142" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="I142" s="2" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="J142" s="2" t="s">
         <v>16</v>
@@ -8003,10 +8174,10 @@
         <v>142</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D143" s="2" t="s">
         <v>328</v>
@@ -8015,16 +8186,16 @@
         <v>12</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G143" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="2" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="I143" s="2" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="J143" s="2" t="s">
         <v>16</v>
@@ -8035,28 +8206,28 @@
         <v>143</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G144" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="I144" s="2" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="J144" s="2" t="s">
         <v>16</v>
@@ -8067,30 +8238,28 @@
         <v>144</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F145" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fix landed in commit 3c33554 on develop ("Fix secret-scan false positive on hyphenated placeholders (Bugs S.No 143)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/3c33554 (the commit message says S.No 143; the sheet row is 144 — the sheet is correct). Walk it: runner/companion/guardrails.py (the placeholder allow-list). Prove it: pytest backend/tests/test_guardrails.py -k placeholder  (scoped on purpose — running the whole file also picks up test_run_build_clean_change_reports_ok, which fails for an unrelated, pre-existing reason: it needs real git workspace access. That failure is not this fix.)</t>
-        </is>
+      <c r="F145" s="2" t="s">
+        <v>706</v>
       </c>
       <c r="G145" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H145" s="2" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="I145" s="2" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="J145" s="2" t="s">
         <v>16</v>
@@ -8106,30 +8275,28 @@
         <v>146</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fix landed in commit 6f9671f on develop ("Make AI-engine / usage-limit build failures human-readable (Bugs S.No 146)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/6f9671f. NOTE the old reference said daemon.py:271, which has ROTTED (that line is now a bare `except`); the real code is: backend/drivers/claude_driver.py (captures the engine's stderr tail) and backend/orchestration/build_activities.py → classify_build_failure() (turns a raw usage/rate-limit error into a plain-language reason). Prove it: pytest backend/tests/test_build_activities.py -k classify. This row is still marked Open — the code fix has landed but is awaiting the team's live test.</t>
-        </is>
+      <c r="F147" s="2" t="s">
+        <v>712</v>
       </c>
       <c r="G147" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H147" s="2" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="I147" s="2" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="J147" s="2" t="s">
         <v>141</v>
@@ -8140,7 +8307,7 @@
         <v>147</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="D148" s="2" t="s">
         <v>571</v>
@@ -8148,28 +8315,20 @@
       <c r="E148" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence — reproduce on any build with blocking findings: the remediation child work items on the Work Items board show a bare title and an EMPTY description. Root of the evidence trail, verifiable by reading the code: backend/orchestration/review_provider.py → parse_findings() read only rem/severity/title/file/line and silently dropped the agent's `problem`/`fix`/`category`, and build_activities.py → run_code_review_core() created the WorkItem with no description at all — so the reviewer's words could not reach the board. The agent's own contract already emits those fields: see the verdict JSON example in agents/08_code_review/agent.md.</t>
-        </is>
+      <c r="F148" s="2" t="s">
+        <v>716</v>
       </c>
       <c r="G148" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H148" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BOTH sides, and the PLATFORM was the hard blocker. (1) Platform: the remediation child WorkItem was created with title=finding.title and NO description at all (build_activities). Worse, the Finding dataclass had no description field and parse_findings (review_provider) SILENTLY DROPPED the agent's problem/fix/category — so even a perfectly humanized review could never reach the board; the reviewer's words were discarded before they got there. Agent 07's remediation manifest had the same hole: it was asked to fix each finding from its one-line title. (2) Agent: 08_code_review/agent.md asked for 'a concise title' with no readability directive, and its JSON example — which is what the agent actually imitates — showed terse fragments ('unbounded result set').</t>
-        </is>
-      </c>
-      <c r="I148" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mirrors the proven S.No 118 pattern. PLATFORM: Finding now carries description/problem/fix/category and parse_findings maps them through; the WorkItem gets a real humanized brief composed by _remediation_description — a plain-language severity lead, 'What's wrong', 'What to do', and a 'Where' line keeping the technical nuance (file:line, review dimension, severity, REM id). A title-only finding says so honestly instead of implying a fuller brief. _render_remediation_section now folds the same detail into agent 07's manifest. AGENT: added a 'Writing standard' to 08_code_review/agent.md mirroring 06's proven one and scoped to the verdict findings fields (title = a board item's title, problem = what is wrong AND why it matters, fix = what to actually do, self-contained, no 'see above'); made the contract explicit that title/problem/fix are read by people on the Work Items board and are required on every blocking finding; REWROTE the JSON example into properly humanized findings. Audience is a developer, so the bar is 06's: plain language that keeps the technical nuance. Tests: parse_findings carries the fields + tolerates a detail-less finding; the composed description; the child WI end-to-end; the 07 brief. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/orchestration/review_provider.py → parse_findings() (now carries problem/fix/category); backend/orchestration/build_activities.py → Finding, _remediation_description() (builds the brief), _render_remediation_section() (gives agent 07 the same detail); agents/08_code_review/agent.md → 'Writing standard' + the rewritten verdict JSON example. Prove it: pytest backend/tests/test_build_activities.py -k remediation and pytest backend/tests/test_build_agents_migration.py -k parse_findings</t>
-        </is>
-      </c>
-      <c r="J148" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H148" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="I148" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="J148" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="259.5">
@@ -8177,10 +8336,10 @@
         <v>148</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>22</v>
@@ -8197,13 +8356,13 @@
         <v>149</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="G150" s="2" t="s">
         <v>23</v>
@@ -8217,7 +8376,7 @@
         <v>150</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="D151" s="2" t="s">
         <v>130</v>
@@ -8231,20 +8390,14 @@
       <c r="G151" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H151" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PhasesAndRuns rendered a plain native &lt;Select&gt; listing every work item in the project (~54), so finding one meant scrolling and eyeballing the list. The UI kit had only Input and Select — no Combobox/Autocomplete existed, so a searchable picker had to be built, not just wired up.</t>
-        </is>
-      </c>
-      <c r="I151" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Built a small reusable Combobox in the UI kit (team's choice over a filter box or a native &lt;datalist&gt;): type to filter the list in the dropdown itself, arrow keys move, Enter picks, Esc closes/reverts, click-outside closes, and it uses the standard combobox ARIA roles so screen readers announce it. Reuses the .input frame + .select chevron so it looks identical to the other controls, and says 'No work items match' rather than showing an empty box. Swapped into the Phases &amp; Runs work-item picker; available for any other long list. Tests (Combobox.test.tsx): filters as you type + click to pick, keyboard operable, empty-state, and shows the current selection when closed. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: frontend/src/components/ui/index.tsx → Combobox (new reusable component); frontend/src/features/lifecycle/PhasesAndRuns.tsx (the picker now uses it); frontend/src/styles/components.css (.combobox*). Prove it: cd frontend &amp;&amp; npx vitest run src/components/ui/Combobox.test.tsx</t>
-        </is>
-      </c>
-      <c r="J151" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H151" s="2" t="s">
+        <v>725</v>
+      </c>
+      <c r="I151" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="J151" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="162">
@@ -8252,7 +8405,7 @@
         <v>151</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="D152" s="2" t="s">
         <v>93</v>
@@ -8266,20 +8419,14 @@
       <c r="G152" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H152" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">work_item_key is a BRANCH SLUG, not a display name (build_types: 'branch name + run prompt'). trigger.py builds it as caller-supplied -&gt; the Jira id (TASK-001) -&gt; a fallback of 'WI-&lt;first 8 chars of the uuid&gt;'. Three places used it as a title: the Code Review artifact, the Code artifact, and the GitHub PR title (so it leaked to the system of record too). Rows that looked fine were agent-authored: open_build_pr / run_code_review are register-don't-recreate and never overwrite the agent's title — so bad names were always the platform's own fallback. The frontend was NOT at fault (artifactLabel already prefers the title).</t>
-        </is>
-      </c>
-      <c r="I152" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Added work_item_title to BuildInput, populated in trigger.py from work_item.title, and a display_name() helper that prefers the title and falls back to the key only when there is no title. The Code artifact, the Code Review artifact and the PR title now read the task title; work_item_key still names the branch, and the PR body carries it for traceability. Passed on the input rather than read from the DB inside the activity, so activities stay deterministic for Temporal replay. Tests: display_name prefers the title / falls back on blank+whitespace; artifacts + PR title carry the task title while the key stays in the body. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/orchestration/build_types.py → BuildInput.work_item_title + display_name(); backend/orchestration/trigger.py (populates it from work_item.title); backend/orchestration/build_activities.py → open_build_pr_core() (PR title + Code artifact) and run_code_review_core() (Code Review artifact). Prove it: pytest backend/tests/test_build_activities.py -k "display_name or task_title"</t>
-        </is>
-      </c>
-      <c r="J152" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H152" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="I152" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="J152" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="162">
@@ -8287,7 +8434,7 @@
         <v>152</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="D153" s="2" t="s">
         <v>93</v>
@@ -8301,20 +8448,14 @@
       <c r="G153" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The BUILD path had no publish step at all. The planning path has publish_artifacts_core, which publishes EVERY artifact of the run; the build path published exactly one — merge_build_pr_core grabbed only the single type='code' row. Grepping Status.PUBLISHED across orchestration returned only those two hits, so nothing else COULD publish them: the Assumptions and Code Review artifacts stayed Draft forever even though their gate was approved. Not intentional — 'internal' is those artifacts' SoR, not a lifecycle status, and the planning path deliberately publishes internal-SoR artifacts. A gap, not a decision.</t>
-        </is>
-      </c>
-      <c r="I153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Added publish_build_artifacts_core mirroring the planning path's publish_artifacts_core and called it from BuildWorkflow after merge_build_pr: it publishes every artifact of the run, skips already-published ones, and takes an immutable S3 audit snapshot of any body-bearing artifact. It changes ONLY `status` — each artifact already carries its correct SoR from registration (code -&gt; git, review -&gt; internal), so this is structurally incapable of clobbering the code pointer's sor=git. Run.status=COMPLETED and the artifacts.published event moved out of merge into publish, so a run can no longer report 'completed' while its artifacts are still draft; merge now performs only the gated SoR write. Idempotent for Temporal retries/replays. Tests: publishes all three artifact types (not just code), sor=git + the PR pointer survive, snapshot written, idempotent, and the merge/publish split; the phase-2 acceptance replay test was extended through the new step. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/orchestration/build_activities.py → publish_build_artifacts_core() (new; mirrors the planning path's publish_artifacts_core in backend/orchestration/activities.py — compare them side-by-side) and merge_build_pr_core() (now does only the gated write); backend/orchestration/build_workflow.py (calls publish_build_artifacts after the merge). Prove it: pytest backend/tests/test_build_activities.py -k publish_build</t>
-        </is>
-      </c>
-      <c r="J153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H153" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="I153" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="J153" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="129">
@@ -8322,7 +8463,7 @@
         <v>153</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>723</v>
+        <v>733</v>
       </c>
       <c r="D154" s="2" t="s">
         <v>93</v>
@@ -8345,13 +8486,13 @@
         <v>154</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="G155" s="2" t="s">
         <v>23</v>
@@ -8365,7 +8506,7 @@
         <v>155</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>725</v>
+        <v>735</v>
       </c>
       <c r="D156" s="2" t="s">
         <v>147</v>
@@ -8385,7 +8526,7 @@
         <v>156</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="D157" s="2" t="s">
         <v>147</v>
@@ -8393,28 +8534,20 @@
       <c r="E157" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F157" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence (1) rotation deadlock — Integrations → any configured capability → the secret field renders a disabled 'configured' box with no way to type a new value; the input was gated on secrets[field] being non-empty while the only control that could set it was that same input (frontend/src/features/setup/ConnectCapability.tsx). Evidence (2) DATA LOSS, reproduced by a test written BEFORE the fix — PATCH /api/integrations/{id}/ with {"binding": {...}, "secrets": {}} (exactly what the drawer sends when you edit a configured connection without retyping the token) returned 200 with configured=False and the stored token destroyed. Verbatim failure: `assert resp.data["configured"] is True` -&gt; `assert False is True`. Re-run it yourself: pytest backend/tests/test_integrations_admin.py -k empty_secrets_object. Evidence (3) not-a-live-probe — the old docstring on backend/apps/integrations/services.py → test_integration_connection() stated it proves the pair is 'constructible and a secret has been stored, not that the upstream API is currently reachable'.</t>
-        </is>
+      <c r="F157" s="2" t="s">
+        <v>737</v>
       </c>
       <c r="G157" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H157" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TWO independent causes, plus a latent data-loss bug found while investigating. (1) ROTATION — a UI deadlock; the backend was always fine (update_integration happily re-encrypts a new secret). ConnectCapability rendered the editable secret input ONLY when secrets[field] was already non-empty — and the only control that could set it was that very input, so it could never appear. The help text 'Enter a new value only to rotate it' described something unreachable. (2) TEST-BEFORE-SAVE — test_integration_connection was NOT a live probe (its own docstring said it proves the capability+vendor pair is constructible and a secret is stored, not that the API is reachable), AND the endpoint was detail=True + get_object(), so it structurally REQUIRED a saved row: that is why saving first was forced. (3) DATA LOSS (latent, proven by a failing test before fixing): the drawer sends secrets:{} whenever an admin edits a configured connection without retyping the token (e.g. changing only the project key). {} is not None, so update_integration re-encrypted an empty dict and SILENTLY WIPED the stored credential — the test showed `configured` flipping to False.</t>
-        </is>
-      </c>
-      <c r="I157" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(1) Rotation: an explicit `rotating` state + a Replace button next to the Configured badge (and Cancel to keep the stored value), which breaks the deadlock; secretsComplete now requires a value only once a rotation is actually opened, so Save is never blocked by a cancelled one. (2) Data loss fixed on BOTH ends: the frontend omits the `secrets` key entirely when nothing was typed, and the server treats an empty object as 'no change' rather than 'erase' (there is deliberately no way to blank a secret via PATCH — disconnect to remove). Regression test added. (3) Test-before-save: extracted a pure probe_connection() that writes nothing to the DB, and added POST /api/integrations/test-credentials/ (detail=False) which probes a throwaway in-memory connection that is NEVER saved; test-connection still probes a saved row and records health. The frontend dropped its !savedId guard and tests as-typed credentials. (4) REAL live probes via a capability-seam ping() on Jira (/rest/api/3/myself), GitHub (/user), Confluence (/rest/api/user/current) and Figma (/v1/me) — cheap, read-only 'who am I' calls that touch no project data; vendor errors are translated into actionable messages (401/403 -&gt; credentials rejected, 404 -&gt; check the site URL, 429 -&gt; rate-limited, 5xx -&gt; vendor down). Xray keeps the wiring-only check and SAYS SO ('no live check for this vendor') rather than implying reachability. NOTE — BEHAVIOR CHANGE: Test connection now makes a real authenticated call, so credentials that used to pass the constructible-only check will now fail if they are wrong; that is the point of the fix. Two pre-existing #39 tests saved dummy creds and asserted ok=True; their intent was 'the catalog slug resolves to a registered, constructible connector', never reachability, so they now assert the failure is not a registry-miss/build error. — REVIEW THE FIX: landed in commit 2a8bc23 on develop ("Fix artifact naming, build publish, remediation briefs, WI search, integrations (S.No 151/152/147/150/156)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/2a8bc23. Walk it: backend/apps/integrations/services.py → probe_connection() (new pure core, no DB writes), test_credentials() (unsaved in-memory probe), update_integration() (empty secrets = no change); backend/api/views.py → IntegrationViewSet.test_credentials_action (POST /api/integrations/test-credentials/); the ping() methods on integrations/atlassian/tasktracker.py, atlassian/docstore.py, github/codehost.py, figma/designsource.py; frontend/src/features/setup/ConnectCapability.tsx (rotating state + Replace). Prove it: pytest backend/tests/test_integrations_admin.py</t>
-        </is>
-      </c>
-      <c r="J157" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H157" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="I157" s="2" t="s">
+        <v>739</v>
+      </c>
+      <c r="J157" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="226.5">
@@ -8422,222 +8555,132 @@
         <v>157</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>727</v>
+        <v>740</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>728</v>
+        <v>741</v>
       </c>
       <c r="E158" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence — reproduce: trigger a build, make the merge fail for a non-conflict reason (e.g. a branch-protection rule on the base), and the run goes terminally FAILED; the only way forward is re-triggering, which re-runs the WHOLE build from step 1. Why it was unavoidable, verifiable in code: backend/orchestration/build_workflow.py called mark_build_failed and RETURNED, which closes the Temporal workflow — and a closed workflow can never be signalled, so there was nothing left to resume. Check the Temporal history of any failed build: it ends at that activity. Note run.inputs (backend/apps/runs/models.py) is never written — there was no checkpoint anywhere.</t>
-        </is>
+      <c r="F158" s="2" t="s">
+        <v>742</v>
       </c>
       <c r="G158" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H158" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On any error both workflows called mark_build_failed/fail_run and RETURNED — which CLOSES the Temporal history for good. A closed workflow can never be signalled, so there was nothing left to resume: the only way forward was trigger_build/trigger_phase creating a brand-new Run + workflow from step 1, re-doing the expensive build. No checkpoint existed anywhere (run.inputs is never written). Note Temporal ALREADY retries transient activity errors (3 attempts) — that was never the gap; the gap was the terminally-closed workflow.</t>
-        </is>
-      </c>
-      <c r="I158" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The workflow now PARKS instead of dying — the same pattern already proven three times here (ENH-2's merge-gate loop S.No 141, the S.No 89 non-terminal STALLED park, and the abandon_run signal). New idempotent activities park_build/park_run (STALLED + a classified reason + the step to resume from) and resume_build/resume_run_state (back to RUNNING, markers cleared), plus a _park() helper in both workflows that waits (human-paced, no timeout) for `resume_run` or `abandon_run`. Wired to: BuildWorkflow's PR/review/gate-setup errors and NON-conflict merge errors, and AgentRunWorkflow's verify_writes. dispatch_build sits OUTSIDE the retry loop, so the build itself is NEVER redone; every retried step is idempotent (open_build_pr register-don't-recreate, open_merge_gate get_or_create). A merge error resumes under the SAME approval — clicking Resume IS the human action. ENH-2's conflict loop is preserved untouched, and abandon reuses today's exact terminal path, so the worst case is today's behavior. EmptyBuild stays terminal (is_empty_build): the agent produced no changes, so resuming would fail identically forever. New POST /api/runs/{id}/resume/ + resume_stalled_run (modelled on take-over/; fires only for a run parked at a resumable error, never an S.No 89 companion-offline park). RunConsole shows the reason + 'Resume from where it stopped' / 'Take over instead'. No workflow.patched needed: the changes are on exception paths, and a workflow that had taken one would already have completed. Tests: park/resume idempotency + marker clearing, is_empty_build, resume refusing a companion-offline park, and three live-Temporal saga tests (merge-error -&gt; park -&gt; resume -&gt; merge with no rebuild; abandon -&gt; terminal; empty-build -&gt; never parked). — REVIEW THE FIX: landed in commit d12d9c7 on develop ("Resume an interrupted phase instead of restarting it (Bugs S.No 157)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/d12d9c7. Walk it: backend/orchestration/build_workflow.py → BuildWorkflow._park() + the resume_run/abandon_run signals; backend/orchestration/build_activities.py → park_build_core()/resume_build_core(); backend/orchestration/workflows.py → AgentRunWorkflow._park(); backend/orchestration/activities.py → park_run_core()/resume_run_state_core(); backend/orchestration/takeover.py → resume_stalled_run(); backend/api/views.py → RunViewSet.resume (POST /api/runs/{id}/resume/); build_types.py → is_empty_build(); frontend/src/features/lifecycle/RunConsole.tsx (Resume button). Prove it: pytest backend/tests/test_build_activities.py -k "park or resume or empty_build" and pytest backend/tests/test_phase_dispatch.py -k "park or resume". Live saga tests (need Temporal on localhost:7233, run ONE at a time — the file OOMs if run whole): pytest backend/tests/test_build_workflow.py::test_build_workflow_merge_error_parks_then_resumes_without_rebuilding</t>
-        </is>
-      </c>
-      <c r="J158" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H158" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="I158" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="J158" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="159" spans="1:10">
       <c r="A159" s="2">
         <v>158</v>
       </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A phase run can fail with no reason shown at all — the run console says it failed but the failure line is empty</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Found while investigating S.No 157. When the write-completeness check (verify_writes) rejects a phase, the run shows as failed but the console shows NO reason — the user is told only that something went wrong, with nothing to act on. Every other failure path records a readable reason; this one recorded nothing.</t>
-        </is>
-      </c>
-      <c r="D159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phases &amp; Runs</t>
-        </is>
-      </c>
-      <c r="E159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence — reproduce: run a phase whose expected artifact is not registered, so the write-completeness check rejects it. The run console shows the run FAILED with an empty failure line — no reason at all. Verifiable in code: backend/orchestration/workflows.py ran verify_writes with RetryPolicy(maximum_attempts=1) and nothing caught its error, so the workflow crashed before fail_run — and fail_run is the only thing that writes run.outputs.error, which is exactly the field frontend/src/features/lifecycle/RunConsole.tsx reads for that line. Not a display bug: the reason was never recorded. Found while investigating S.No 157.</t>
-        </is>
-      </c>
-      <c r="G159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verify_writes runs with RetryPolicy(maximum_attempts=1) and NOTHING caught its error, so the exception propagated and CRASHED AgentRunWorkflow before fail_run could run. fail_run is the only thing that writes run.outputs.error — and RunConsole reads exactly that field for its failure line — so the run was left FAILED with an empty reason. Not a display bug: the reason was never recorded anywhere.</t>
-        </is>
-      </c>
-      <c r="I159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed by the same change as S.No 157: verify_writes is now wrapped, and its failure PARKS the run via park_run, which always records the classified reason on run.outputs.error. So the console now shows the real reason, and the user can Resume to re-check once the missing artifact is registered instead of re-running the whole phase. Test: park_run_core records the reason and stays non-terminal. — REVIEW THE FIX: landed in commit d12d9c7 on develop ("Resume an interrupted phase instead of restarting it (Bugs S.No 157)") · github.com/RAGUWING369/AI-First-SDLC-App/commit/d12d9c7 (same change as S.No 157). Walk it: backend/orchestration/workflows.py (verify_writes is now wrapped in try/except and parks instead of crashing) → backend/orchestration/activities.py → park_run_core() (always records the classified reason on run.outputs.error). Prove it: pytest backend/tests/test_phase_dispatch.py -k park_run_core</t>
-        </is>
-      </c>
-      <c r="J159" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" spans="1:10">
+      <c r="B159" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>746</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H159" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="I159" s="2" t="s">
+        <v>749</v>
+      </c>
+      <c r="J159" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="52.5" customHeight="1">
       <c r="A160" s="2">
         <v>159</v>
       </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Test connection reports OK without checking the repo address it was given - a mistyped repo still shows a green tick, and nothing validates it until the build phase fails</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Found live on 2026-07-17 while setting up tenant SpendLog-2 (Edvensoft-2) for the fresh single-repo end-to-end retest. The Code Host repo was saved as 'RAGUWING369/ SpendLog-2-single-repo-refresh-test' - a stray SPACE after the slash. Test connection reported success and health was written 'healthy', because the probe only asks GitHub 'who am I' (GET /user) and, by its own docstring, 'touches no repository'. The repo address - the one field the whole build depends on - is never resolved. The typo is harmless through ideation / requirements / PRD / architecture / UX / task breakdown (none of them touch the repo), and would only surface at the build phase, AFTER a full planning run, when GitHubCodeHost._repo() passes the string straight into the request path (GET /repos/RAGUWING369/ SpendLog-2-single-repo-refresh-test/branches/main) with no strip/normalisation - a 404 on a malformed URL. Same class of defect as S.No 156, one level up: 156 upgraded the probe from 'is the connector constructible' to 'is the token real' precisely because the old check 'reported OK for a mistyped token, which is exactly what a connection test exists to catch'. A mistyped REPO now reports OK for the same reason. Not GitHub-specific: the same gap applies to any connector with a configured target (Jira project key, Confluence space, Figma file, Xray).</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Integrations / Code Host / Connection test</t>
-        </is>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence - reproduce: in Integrations &gt; Code Host, save a repo with a typo (e.g. a space after the slash: 'OWNER/ repo-name'), then click Test connection.
-Observed: Test connection PASSES ('Signed in to GitHub as RAGUWING369.') and IntegrationConnection.health is written 'healthy', while scopes['repo'] still holds the invalid address. No warning anywhere. Live record on tenant 7828e953-987e-43b2-8d5f-c8a45bfa8c6a at 11:17-11:59 held scopes={'repo': 'RAGUWING369/ SpendLog-2-single-repo-refresh-test'} with health reported OK.
-Proof the probe cannot catch it - GitHubCodeHost.ping() in backend/integrations/github/codehost.py issues only GET /user and its docstring states it 'touches no repository'. probe_connection() in backend/apps/integrations/services.py calls exactly that ping() and returns {ok: True} on success.
-Proof the address is never normalised - GitHubCodeHost._repo() returns the configured string unchanged (no .strip()); callers such as get_branch() / open_pull_request() interpolate it directly into '/repos/{repo}/...'.
-Proof a real check is cheap and would have caught it - with the space removed, the same connector resolves the repo for real:
-  ch.ping()             -&gt; 'Signed in to GitHub as RAGUWING369.'
-  ch.get_branch(name='main') -&gt; BranchRef(sha=e252eaedb3, url=https://github.com/RAGUWING369/SpendLog-2-single-repo-refresh-test/tree/main)
-The identical call against the space version raises a 404. One extra read-only call is the whole difference.</t>
-        </is>
-      </c>
-      <c r="G160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="H160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">probe_connection() validates CREDENTIALS only; it has no notion of the connection's configured TARGET. ping() is deliberately scoped to a cheap 'who am I' that touches no repository, and nothing else in the setup path resolves scopes['repo']. The first code that touches the repo address is the build phase, so a setup typo stays invisible until then. Compounding it, GitHubCodeHost._repo() does not strip or validate the string, so whitespace survives into the URL.</t>
-        </is>
-      </c>
-      <c r="I160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN - not fixed, logged for completeness at the team's request (2026-07-17); typo corrected by hand on SpendLog-2 so the retest could proceed. Proposed: extend probe_connection() so that where a connection carries a configured target, the probe resolves THAT too, not just /user - for codehost, a read-only get_branch(default_base) or GET /repos/{repo}; the connector already exposes everything needed. Report it as its own line ('Signed in as X; repo Y found') so the admin sees both facts. Keep it capability-generic (Jira project key, Confluence space, Figma file), not a GitHub special case, and reuse _probe_failure_detail() - its existing 404 wording ('Authenticated, but that address isn't right - check for typos') is already almost exactly the message this needs. Cheap hardening worth doing at the same time: strip the repo string on save in create_integration()/update_integration() and in GitHubCodeHost._repo(), and reject an address that is not OWNER/NAME shaped. Related: S.No 156 (same principle, one level down).</t>
-        </is>
-      </c>
-      <c r="J160" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
+      <c r="B160" s="2" t="s">
+        <v>750</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>752</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F160" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="G160" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H160" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="I160" s="2" t="s">
+        <v>755</v>
+      </c>
+      <c r="J160" s="2" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="161" spans="1:10">
       <c r="A161" s="2">
         <v>160</v>
       </c>
-      <c r="B161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The platform silently DISCARDS the agent's entire phase document and reports its cost as zero: every artifact the platform files itself is 0 bytes, and the gate opens on a blank page</t>
-        </is>
-      </c>
-      <c r="C161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Found live on 2026-07-17 on tenant SpendLog-2 (Edvensoft-2), run 2894a1e0 - the first ideation of the fresh single-repo retest. The companion ran the 01_ideation agent for ~6 minutes and reported a 34,474-character document costing $0.397562. The platform stored a 0-BYTE draft, content_hash = sha256 of the empty string, and run.cost_usd = 0.0. verify_writes then PASSED (it only checks that an artifact of the expected TYPE exists, never that it has content) and the gate opened on a blank document, asking a human to approve nothing. Temporal shows a clean history with no failure anywhere: the run looks perfect from every angle the platform reports on.
-SCOPE - this bites ONLY the platform's own fallback registration, which is why it hid for so long. When the agent registers its artifacts itself (register_artifact + stage_artifact_body over MCP), that path stages the body and the artifact is fine. Across the three live tenants: SpendLog-1 56 artifacts / 1 empty; Edvensoft 170 / 2 empty; SpendLog-2 1 / 1 empty. The empties are exactly the phase-typed artifacts the platform created itself - e.g. Edvensoft 'testing/testing' empty at 08:26 on 2026-07-17 while its sibling test_case / test_report artifacts, which the agent registered, have real bodies. On run 2894a1e0 the agent registered NOTHING, so the broken fallback carried the whole phase and the loss was total.
-AGGRAVATING - the phase.empty_result event blames the ENGINE for the platform's own bug: 'companion reported ok but the engine returned no final text', when the engine had in fact returned 34,474 characters. That message sent this investigation down the wrong path for a considerable time.</t>
-        </is>
-      </c>
-      <c r="D161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Orchestration / Phase result registration / Artifacts</t>
-        </is>
-      </c>
-      <c r="E161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence - reproduce: run any planning phase on the companion in which the agent does not register the phase artifact itself. The staged draft is 0 bytes and the run's cost is 0.0, while the companion's report holds the real body and cost.
-Observed live (run 2894a1e0, tenant 7828e953-987e-43b2-8d5f-c8a45bfa8c6a):
-  run.outputs['report'] = {'status':'ok', 'body': &lt;34474 chars&gt;, 'cost_usd': 0.397562, 'message': ''}
-  run.outputs['cost_usd'] = 0.0                    &lt;- should be 0.397562
-  run.cost_usd            = 0.0000                 &lt;- should be 0.3976
-  artifact e619681e: content_hash = sha256:e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855
-                     (that is the sha256 of the EMPTY string), title = '', status = draft
-  S3 drafts/&lt;tenant&gt;/&lt;project&gt;/2894a1e0-.../ideation.md -&gt; get() returns b'', length 0
-The COST is the decisive proof: 0.397562 arrived and 0.0 was stored. Only a defaulted read explains both fields going wrong at once, from one line.
-Ledger events for the run, in order: run.triggered 12:09:24 / phase.dispatched 12:09:28 / phase.reported 12:15:32 {'status':'ok'} / run.executed 12:15:36 / phase.empty_result 12:15:36 'companion reported ok but the engine returned no final text; the staged phase draft is empty' (FALSE - see Description) / gate.opened 12:15:38.
-Temporal history (agent-run-2894a1e0-6b6f-4772-9b0a-cc7ad8d4376f on 13.203.56.29:7233): #5 compose_manifest, #11 dispatch_phase, #18 SIGNAL phase_reported, #23 register_phase_result, #29 verify_writes, #35 open_gate. No failures.
-Code location - register_phase_result_core() in backend/orchestration/activities.py read the report with getattr(report,'body',''), getattr(report,'cost_usd',0.0) and getattr(report,'message',''), while register_phase_result_activity(inp: AgentRunInput, report) left `report` UNANNOTATED. It was the ONLY unannotated activity parameter in backend/orchestration (whole package scanned).
-Why the tests never caught it - every existing test in backend/tests/test_phase_dispatch.py passes a real PhaseReport dataclass straight into the core, a shape production never sends; the dict only appears once the argument crosses Temporal. Proof the new regression test reproduces it: on the pre-fix code it fails with  assert b'' == b'# PRD\nreal body'.</t>
-        </is>
-      </c>
-      <c r="G161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Temporal's data converter converts an activity argument to the type its parameter is ANNOTATED with, and hands an UNANNOTATED parameter back as the raw decoded JSON - a plain dict. register_phase_result_activity annotated `inp: AgentRunInput` (which is exactly why inp always worked) but left `report` bare, so the PhaseReport arrived as a dict. register_phase_result_core then read it with getattr, which looks up an ATTRIBUTE - a dict has none - so getattr returned its DEFAULT for every field: body '' and cost_usd 0.0. Nothing raised. The defaults are indistinguishable from an engine that genuinely produced nothing, which is precisely what the phase.empty_result message then asserted.
-verify_writes could not save it either: verify_write_completeness_core asserts only that an artifact of the expected TYPE exists, never that its body is non-empty - so the platform's own 0-byte row satisfied the last check before the gate.</t>
-        </is>
-      </c>
-      <c r="I161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IN PROGRESS (2026-07-17) - fixed locally, NOT committed, pending team test. Three parts, all in backend/orchestration/activities.py:
-1. ROOT FIX - annotate the activity: register_phase_result_activity(inp: AgentRunInput, report: PhaseReport). Temporal now converts the payload to a PhaseReport, matching the `inp` parameter that always worked. A test asserts the annotation stays put, so it cannot be silently dropped again.
-2. DEFENCE - new _as_phase_report() coerces dict / PhaseReport / duck-typed object to a PhaseReport, and the core reads report.body / report.cost_usd / report.message directly - no getattr on a possible dict anywhere in the path. The cores are also called directly by tests and by the takeover path, so both shapes must keep working.
-3. HONESTY - the phase.empty_result message no longer reads the report via getattr, so it can no longer blame the engine for the platform's own defaulted read.
-Tests (backend/tests/test_phase_dispatch.py): test_register_phase_result_core_reads_a_dict_report sends the exact wire shape Temporal delivers and asserts the body is staged, the hash is not the empty-file hash, and the cost survives (run.cost_usd is a 4dp Decimal column, so the stored value is the rounded 0.3976). test_register_phase_result_activity_annotates_its_report_param guards the root fix. Both fail on the pre-fix code and pass after.
-Verified: test_phase_dispatch 26 passed / 3 skipped; test_orchestration_activities + test_acceptance_phase45 + test_acceptance_phase47 = 14 passed / 1 failed, that 1 being the PRE-EXISTING test_offline_companion_parks_for_takeover, which fails identically without this change (logged as S.No 161).
-NOT fixed here, deliberately: verify_writes still passes an empty artifact (it checks type presence, not content). Logged separately so the last line of defence is fixed on its own merits rather than as a side effect. Related: S.No 59 (the other half of this seam - pointer-only artifacts never staged), S.No 158 (verify_writes crash).</t>
-        </is>
-      </c>
-      <c r="J161" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In Progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="162" spans="1:1">
+      <c r="B161" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>757</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F161" s="2" t="s">
+        <v>759</v>
+      </c>
+      <c r="G161" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H161" s="2" t="s">
+        <v>760</v>
+      </c>
+      <c r="I161" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="J161" s="2" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10">
       <c r="A162" s="2">
         <v>161</v>
       </c>
     </row>
-    <row r="163" spans="1:1">
+    <row r="163" spans="1:10">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -8646,153 +8689,135 @@
       <c r="A164" s="2">
         <v>163</v>
       </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clarification gate surfaced only Tier-1 (must-ask) questions - Tier-2 suggestions and Tier-3 inferences never reached the user</t>
-        </is>
-      </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The SDLC app promises a human is always in the loop and the platform never silently assumes. But agents classified each context gap into three tiers and only surfaced Tier 1 through the clarifications gate. Tier 2 (the agent's own suggestions) was written inline inside the deliverable, and Tier 3 (industry-standard inferences) was logged silently as assumptions the user never saw. So the user could not confirm or override the agent's Tier-2/3 choices, and the 'no silent assumptions' assurance was only partly true.</t>
-        </is>
-      </c>
-      <c r="D164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clarifications / Context Gap Scan</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Observed live across Ideation, Requirements and PRD runs on tenant Edvensoft-2: every phase logged Tier-3 items as assumptions and opened 0 clarifications, so the user never saw the agent's inferences. Verified in code: ask_human was the only human-question touchpoint and the shared rules told agents to front-load only Tier 1 and Tier 2. Retested after the fix on a live UX-design run - a single gate now shows Tier 1/2/3 sections.</t>
-        </is>
-      </c>
-      <c r="G164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The behaviour lived in the shared agent rules (backend/manifest/rules/prompt_rules.py): agents were told to 'front-load ALL Tier-1 and Tier-2 questions' and to record every Tier-3 inference silently as an assumption. Only Tier 1 was required/blocking; nothing surfaced Tier 2 or Tier 3 through the clarifications gate. The tier definitions were also thin (one line each), so classification was inconsistent.</t>
-        </is>
-      </c>
-      <c r="I164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reworked the shared rules so the agent front-loads ALL three tiers into ONE clarifications gate before starting work, each question tagged with its tier. Tier 1 stays required; Tier 2/3 are optional and carry the agent's proposed answer as a pre-filled 'suggestion' the user can accept, edit or override, with an 'Accept all' one-click. Any untouched Tier-2/3 item falls back to the suggestion, and the confirmed Tier-3 values are still recorded as assumptions for provenance. Also strengthened the tier definitions (a four-question test plus concrete examples per tier). The web gate groups questions under Tier 1/2/3 headers. No DB migration (questions are stored as JSON). Landed on develop in commit 0c19292; backend + frontend tests, type-checks and lint all pass; user-tested on a live UX-design run.</t>
-        </is>
-      </c>
-      <c r="J164" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="B164" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F164" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H164" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="I164" s="2" t="s">
+        <v>768</v>
+      </c>
+      <c r="J164" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="165" spans="1:10">
       <c r="A165" s="2">
         <v>164</v>
       </c>
-      <c r="B165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Platform does not verify the agent's tier classification - a mislabelled Tier-1 gap can still slip through as a Tier-3 guess</t>
-        </is>
-      </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Even with all three tiers now surfaced in the gate, the platform trusts the agent's own Tier 1/2/3 labelling. If the agent wrongly files a business-critical gap (for example pricing, compliance or a third-party integration) as a Tier-3 inference, it is shown pre-filled and quietly accepted rather than hard-asked. So the 'never assume' assurance still depends on the agent classifying correctly and the human reviewer noticing at the gate.</t>
-        </is>
-      </c>
-      <c r="D165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clarifications / Context Gap Scan</t>
-        </is>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enhancement</t>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Design gap, not a live failure. ask_human and create_clarification carry no tier logic (runner/companion/state_mcp.py, backend/apps/clarifications/services.py); the tier reasoning lives only in the agent prompt (backend/manifest/rules/prompt_rules.py). No validator checks a question or assumption against the hard-coded Tier-1 'never infer' category list.</t>
-        </is>
-      </c>
-      <c r="G165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="H165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">By design, tier classification is the agent's own reasoning; there is no control-plane check. The platform records and delivers whatever tiers the agent labels, and only a human reviewer reading the gate or the Assumptions Log can catch a misclassification.</t>
-        </is>
-      </c>
-      <c r="I165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proposed (future): a platform-side validator that scans each phase's questions and assumptions for the Tier-1 'never infer' categories and auto-promotes any match to a required Tier-1 question before the gate can close - turning tier classification from 'trust the agent' into 'the platform double-checks the high-risk categories'. Not yet implemented.</t>
-        </is>
-      </c>
-      <c r="J165" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="166" spans="1:1">
+      <c r="B165" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F165" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="G165" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H165" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="I165" s="2" t="s">
+        <v>773</v>
+      </c>
+      <c r="J165" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" ht="409.6">
       <c r="A166" s="2">
         <v>165</v>
       </c>
-    </row>
-    <row r="167" spans="1:1">
+      <c r="B166" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F166" s="2" t="e" vm="17">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J166" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10">
       <c r="A167" s="2">
         <v>166</v>
       </c>
     </row>
-    <row r="168" spans="1:1">
+    <row r="168" spans="1:10">
       <c r="A168" s="2">
         <v>167</v>
       </c>
     </row>
-    <row r="169" spans="1:1">
+    <row r="169" spans="1:10">
       <c r="A169" s="2">
         <v>168</v>
       </c>
     </row>
-    <row r="170" spans="1:1">
+    <row r="170" spans="1:10">
       <c r="A170" s="2">
         <v>169</v>
       </c>
     </row>
-    <row r="171" spans="1:1">
+    <row r="171" spans="1:10">
       <c r="A171" s="2">
         <v>170</v>
       </c>
     </row>
-    <row r="172" spans="1:1">
+    <row r="172" spans="1:10">
       <c r="A172" s="2">
         <v>171</v>
       </c>
     </row>
-    <row r="173" spans="1:1">
+    <row r="173" spans="1:10">
       <c r="A173" s="2">
         <v>172</v>
       </c>
     </row>
-    <row r="174" spans="1:1">
+    <row r="174" spans="1:10">
       <c r="A174" s="2">
         <v>173</v>
       </c>
     </row>
-    <row r="175" spans="1:1">
+    <row r="175" spans="1:10">
       <c r="A175" s="2">
         <v>174</v>
       </c>
     </row>
-    <row r="176" spans="1:1">
+    <row r="176" spans="1:10">
       <c r="A176" s="2">
         <v>175</v>
       </c>

</xml_diff>

<commit_message>
Bugs sheet: log the takeover-timeout terminal-failure race as S.No 169 (Open)
A companion run finalized to 'failed' by the takeover timeout is not reconciled when
the companion later returns and reports the phase succeeded with artifacts. Not fixed
yet — logged Open with root cause and proposed fix.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -8918,6 +8918,51 @@
       <c r="A170" s="2" t="n">
         <v>169</v>
       </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Takeover timeout marks a companion run terminally 'failed' even when the companion later comes back and reports the phase succeeded with artifacts registered — the late success does not reconcile the run, and the UI shows a false 'engine exited, no artifact' message.</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Found 2026-07-13 on the SpendLog Architecture run. When a companion (local Claude Code) goes offline after a phase is dispatched, the orchestrator's takeover reconciler fires phase.takeover (reason 'companion offline / no report before timeout') and sets the run to a terminal 'failed' state. If the companion later comes back, completes the work, registers artifacts, and posts phase.reported status=ok, that late success does NOT reconcile the run out of 'failed'. Result: the run shows failed with the canned UI message 'The engine exited before reporting. No artifact was registered.' — which is factually wrong (artifacts were registered, report status was ok). Event sequence proving the race: dispatched 19:49:55Z -&gt; ~7.5h gap (laptop asleep) -&gt; phase.reclaimed 03:25:12Z -&gt; phase.takeover 03:27:37Z (run set failed) -&gt; 11 artifacts registered 03:55:04-03:55:40Z -&gt; phase.reported ok 03:56:57Z.</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>Orchestration / Takeover + phase-report reconciliation</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>Found 2026-07-13, SpendLog Architecture run 8738d4ba-72ee-460f-b41f-86556fca5658 (tenant 212395b8-f118-4eef-93eb-ba2c45468226). Code: takeover path in the orchestrator + phase-report handler (backend/api/runner_views.py phases/&lt;id&gt;/report/).</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>'failed' is a terminal state and swallows a later successful report. Takeover finalizes the run to failed while the companion is merely offline (e.g. laptop asleep), and nothing re-opens it when the companion returns and reports ok with artifacts — takeover wins a race it is about to lose.</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — not yet fixed. Proposed: a successful late phase.reported (status=ok with registered artifacts) should reconcile the run to succeeded (the artifacts are the proof), OR takeover should not finalize while the companion is still making progress / a reclaim should re-open the run. Related operational trigger: companion-offline from laptop sleep stalls dispatched phases.</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">

</xml_diff>

<commit_message>
Updatded the Bugs sheet with Phases & Runs, Run console, Clarifications pages bugs and more from S.No - 170 - 175
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30318"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="175" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77C94B95-75A2-4B7D-95F4-DEC09B2B7B6F}"/>
+  <xr:revisionPtr revIDLastSave="207" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A04FBDF-F9BB-4AA7-B306-D4BE47860DD0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="17">
+  <futureMetadata name="XLRICHVALUE" count="21">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -158,8 +158,36 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="17"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="18"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="19"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="20"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="17">
+  <valueMetadata count="21">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -211,12 +239,24 @@
     <bk>
       <rc t="1" v="16"/>
     </bk>
+    <bk>
+      <rc t="1" v="17"/>
+    </bk>
+    <bk>
+      <rc t="1" v="18"/>
+    </bk>
+    <bk>
+      <rc t="1" v="19"/>
+    </bk>
+    <bk>
+      <rc t="1" v="20"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1314" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1393" uniqueCount="821">
   <si>
     <t>S.No</t>
   </si>
@@ -2326,10 +2366,10 @@
     <t>Companion / Dependency management</t>
   </si>
   <si>
-    <t>The companion depends on claude-agent-sdk, which in turn requires a newer anyio (the anyio.open_process 'user' keyword arrives in anyio 4.5.0; claude-agent-sdk 0.1.72 needs it). The repo's pins were stale (an old claude-agent-sdk pin and no floor on anyio), so a fresh environment installed anyio 4.4.0 and the agent crashed with "anyio.open_process() got an unexpected keyword argument 'user'". This session it was worked around by manually upgrading anyio on the host (pip install -U 'anyio&gt;=4.5' -&gt; 4.14.2), but that fix lives only on this machine - the repo still pins the broken combination, so the next developer or a rebuilt container will hit the same crash.</t>
-  </si>
-  <si>
-    <t>OPEN - not fixed this session (env-patched only). Recommended fix: pin the correct, mutually compatible versions in the repo lockfile/requirements - bump claude-agent-sdk to the version actually in use and add an explicit anyio&gt;=4.5 floor - then rebuild the companion/worker images from the lockfile so a clean install reproduces the working environment. Acceptance: a from-scratch install (no manual pip upgrades) runs a build without the open_process 'user' error.</t>
+    <t>Two compounding causes. (1) The companion ran in the GLOBAL Python with no venv, while the client app it builds (medslot / SDLC-expenselog) pins anyio==4.4.0 + httpx==0.27.0 in its own backend/requirements.txt. Any medslot build/preview `pip install -r requirements.txt` ran in that shared global env and downgraded anyio to 4.4.0, breaking claude-agent-sdk's engine launch (anyio.open_process(..., user=...) needs anyio&gt;=4.5) mid-build. (2) The repo's engine pins were also stale, so a clean install reproduced the broken combination. The earlier note treated this as pins-only; in practice the operative cause was the global-env pollution from the app being built.</t>
+  </si>
+  <si>
+    <t>Fixed 2026-07-20/21. (a) Pinned the engine dep set in the repo (commit 28531e1): claude-agent-sdk==0.1.72, mcp==1.27.0, anyio==4.14.2. (b) Dedicated companion venv OUTSIDE all projects: C:\Users\Msi\sdlc-companion-venv; launch by the venv's absolute python path WITHOUT activating, so build-subprocess pip installs still hit the global env and can never reach the companion's anyio. (c) Startup guard (commit 8c34c24): serve/run call _assert_engine_env() and exit(2) with an actionable message if anyio can't launch the engine. Validated live: WI-38/39/60/41/42/44/45 retriggers all cleared the engine-launch step with no anyio error.</t>
   </si>
   <si>
     <t>Build branches are merged without first being updated against their base, causing merge conflicts at the gate</t>
@@ -2672,6 +2712,42 @@
     <t>In Progress</t>
   </si>
   <si>
+    <t>When a build's remediation loop hit its cycle cap it hard-failed the WorkItem with no diagnostics and no way forward — the user could not complete the WorkItem.</t>
+  </si>
+  <si>
+    <t>The 07&lt;-&gt;08 remediation loop was capped at max_remediation_cycles. On exhaustion the workflow raised a hard failure and stopped. The run console showed only blocking-finding COUNTS across cycles (e.g. 2 -&gt; 1 -&gt; 3 -&gt; 3) with no visibility into what the findings actually were, and there was no automated retry — a human had to step in, defeating the automation promise. If remediation kept exhausting, the WorkItem was simply stuck.</t>
+  </si>
+  <si>
+    <t>Orchestration / Build saga / Remediation</t>
+  </si>
+  <si>
+    <t>commit 29e934b; backend/orchestration/build_workflow.py, build_activities.py (handle_remediation_exhausted), trigger.py, build_types.py</t>
+  </si>
+  <si>
+    <t>On remediation exhaustion the workflow had a single terminal branch (hard fail). It neither captured the real blocking-finding text nor attempted a fresh build attempt, so an exhausted WorkItem had nowhere to go.</t>
+  </si>
+  <si>
+    <t>commit 29e934b. run_code_review now persists the actual blocking-finding detail (rem/severity/title/file/line) into run.outputs['review_cycles'], not just counts. New handle_remediation_exhausted activity: if attempt &lt; max_auto_attempts (default 2) it marks the current run failed with a clear 'auto-retrying' message, logs build.remediation_exhausted_retry, and re-triggers the build with attempt+1 and a seeded prior_attempt_context digest of what blocked the prior attempt — fully automated, no human. Only after all auto-attempts are exhausted does it park for a human. Tests in backend/tests/test_build_activities.py. Validated live 2026-07-21: WI-60 fired build.remediation_exhausted_retry {attempt:1,next_attempt:2} and auto-started attempt 2.</t>
+  </si>
+  <si>
+    <t>A build's remediation could start from an empty tree or push a non-fast-forward when a different companion continued a WorkItem than the one that started it — remediation work was lost or the push was rejected.</t>
+  </si>
+  <si>
+    <t>Each companion provisioned its worktree from its own LOCAL branch state. When companion B continued a WorkItem that companion A had started and pushed, B based the worktree on a stale or absent local ref, producing either an empty build or a non-fast-forward push that failed during the remediation cycle. Subsumes the older stale-local-branch empty-build issue (#145).</t>
+  </si>
+  <si>
+    <t>Companion / Worktree provisioning</t>
+  </si>
+  <si>
+    <t>commits 9863c16, d008643; runner/companion/worktree.py (provision_worktree)</t>
+  </si>
+  <si>
+    <t>provision_worktree based the worktree on a possibly-stale local remote-tracking ref. git fetch does not prune, so a stale origin/&lt;branch&gt; ref (left after the remote branch was deleted) could resurrect a dead branch at an old commit; and a genuinely continued branch was never re-fetched from the true remote tip.</t>
+  </si>
+  <si>
+    <t>commits 9863c16 + d008643. provision_worktree now authoritatively checks `git ls-remote --heads &lt;remote&gt; &lt;branch&gt;`. If the branch exists on the remote it fetches and bases the worktree on &lt;remote&gt;/&lt;branch&gt; (git worktree add -B branch &lt;remote-tip&gt;), so ANY companion continues from the true shared work-in-progress; it falls back to `base` only for a genuinely new/offline branch. Tests in backend/tests/test_companion_runner.py (validated on the host with real git; the container has no git binary). Validated live: WI-39's remediation cycle pushed successfully after previously failing.</t>
+  </si>
+  <si>
     <t>Clarification gate surfaced only Tier-1 (must-ask) questions - Tier-2 suggestions and Tier-3 inferences never reached the user</t>
   </si>
   <si>
@@ -2708,6 +2784,117 @@
     <t>The team has observed that in the Architecture phase of System Architecure artifact: The container and component diagrams are not rendered properly and also NFR-to-Architecture Traceability Matrix Table is over entended not fitted in the designated window. 
 Note: The above issue is observed for tenant - test2@edvensoft.com but the same issues are not present for the tenant - test@edvensoft.com. You must go through both the tenant Architecture Phase - System architecture artifact to confirm and come up with the best fix.
 Important Note: The same issues might be come up in later phases or will be observed (definitive chance) - so we need a surgical fix not temporary.</t>
+  </si>
+  <si>
+    <t>Not a content bug - the artifact's diagrams and matrix were valid markdown. In the shared Markdown renderer (frontend/src/components/ui/Markdown.tsx) the rendered Mermaid diagram was placed in a div carrying the class 'diagram-frame', whose CSS rule '.diagram-frame svg { width:40px; height:40px }' - intended only for the empty-state placeholder icon - shrank every real diagram to a 40x40 px smudge. Confirmed by fetching both tenants' System Architecture artifacts from S3: test@edvensoft.com had 0 Mermaid diagrams (so it never hit the bug and looked fine), while test2@edvensoft.com had 3 valid 'graph TD' diagrams that got shrunk. Separately, GFM tables (the NFR-to-Architecture Traceability Matrix) rendered as a plain width:100% table with no scroll container, so a wide matrix over-extended its pane instead of scrolling. Both are shared-renderer defects, so they affect any artifact with diagrams or wide tables in any phase - which is why the same issue was expected to recur in later phases.</t>
+  </si>
+  <si>
+    <t>Surgical fix in the shared Markdown renderer (frontend only - no backend, no DB, no agent change). (1) Diagrams: the rendered container no longer reuses the 'diagram-frame' placeholder class - it uses its own '.md-body__mermaid' class that owns its sizing (svg max-width:100%, height:auto), so diagrams render full size instead of 40x40. (2) Tables: every table is wrapped in a '.md-body__table-wrap' scroll container (overflow-x:auto, max-width:100%), so wide tables scroll inside their pane instead of spilling. Because the fix lives in the shared renderer it covers every phase/artifact and will not recur. Verified live in the running app: the demo diagram rendered at 582x299 px (not 40x40) with no 'diagram-frame' leak, and at mobile width a wide table scrolled inside its wrapper with the page NOT overflowing horizontally. Unit tests (Markdown.test.tsx), typecheck and lint all pass. Files: Markdown.tsx, components.css. To see it: restart the frontend container and hard-refresh the browser - no agent re-run needed, the stored artifact body is unchanged.</t>
+  </si>
+  <si>
+    <t>Work-item search dropdown (Combobox) is clipped for a small list - some items are unreachable because the list only scrolls when it is very long</t>
+  </si>
+  <si>
+    <t>On the Phases &amp; Runs page, the 'Search work items' dropdown shows only the first few items and the rest are cut off with no way to scroll to them when there is a small/limited number of work items. A scrollbar only appears when the list is very long. Observed with 6 work items: WI-6/WI-5/WI-4 show and the remaining ones are clipped and unreachable.</t>
+  </si>
+  <si>
+    <t>Phases &amp; Runs / Combobox</t>
+  </si>
+  <si>
+    <t>Repro: Phases &amp; Runs &gt; 'Search work items' with ~6 work items - the dropdown is cut off at the panel edge and cannot be scrolled to reach the hidden items. With many work items an internal scrollbar appears and all items are reachable.</t>
+  </si>
+  <si>
+    <t>The shared Combobox dropdown (.combobox__list, frontend/src/components/ui) is absolutely positioned with max-height:260px and overflow-y:auto, and it sits inside a Panel whose CSS '.panel { overflow: hidden }' (used for rounded corners) clips the dropdown at the panel edge. When the list is shorter than 260px it gets NO internal scrollbar, so items past the panel edge are clipped and unreachable; only when the list exceeds 260px does the internal scrollbar appear - which is why 'scroll works' only with many items.</t>
+  </si>
+  <si>
+    <t>Two options - team to decide, then fix. Option A (surgical, low-risk, recommended for this screen): stop the Trigger-a-phase Panel from clipping the floating dropdown - add a modifier class (e.g. .panel--menu { overflow: visible }) applied to that one panel; touches PhasesAndRuns.tsx + components.css; fixes this screen only. Option B (general): render the Combobox dropdown in a portal to document.body so it can never be clipped by any container - fixes every Combobox everywhere but is a larger change to the shared component (position calc, reposition on scroll/resize, test updates). Recommend A now; upgrade to B if the same clipping shows up on other screens.</t>
+  </si>
+  <si>
+    <t>Work-item (Epic / User Story / Task) descriptions from Task Breakdown are shown as raw markdown - the content is good but not rendered (bold, code, tables and lists appear as literal ** ` | characters)</t>
+  </si>
+  <si>
+    <t>In the work-item detail pages, the Description that the Task Breakdown agent writes is good but is displayed as plain text: markdown like **bold**, `code`, pipe tables and bullet lists appear as literal characters instead of being rendered, so it is not user-friendly. Observed on TASK-006, TASK-015 and US-009 (Story). General rule the team wants: wherever the app shows content that is meant to be markdown, it must render in a user-friendly way.</t>
+  </si>
+  <si>
+    <t>Work Items / Content rendering</t>
+  </si>
+  <si>
+    <t>Evidence (screenshots shared with the team): TASK-006 and TASK-015 Description panels and the US-009 'Description &amp; context' panel show literal '**Type:**', '**What to build:**', backtick-quoted code and pipe-tables as plain text instead of rendered markdown.</t>
+  </si>
+  <si>
+    <t>The work-item detail views render the description as PLAIN TEXT in a &lt;p&gt; tag instead of through the shared Markdown renderer: WorkItemTask.tsx (line 134), WorkItemEpic.tsx (line 97) and WorkItemDefect.tsx all do '&lt;p className="t-body"&gt;{workItem.data.description}&lt;/p&gt;'. The Markdown component (frontend/src/components/ui/Markdown.tsx - GFM via react-markdown + remark-gfm, already used for artifact previews and hardened in S.No 165) is never applied to work-item descriptions, so the agent's markdown shows raw.</t>
+  </si>
+  <si>
+    <t>FIXED. Routed work-item descriptions through the shared Markdown renderer (frontend/src/components/ui/Markdown.tsx) instead of a plain &lt;p&gt;. Added an optional className prop to Markdown (default 'doc-preview prose md-body') so it renders inside an existing Panel without a nested card; WorkItemTask.tsx and WorkItemEpic.tsx now render the description with &lt;Markdown className='prose md-body'&gt;, keeping the 'No description yet.' fallback. Bold, inline code, lists and tables now render correctly. Reuses the same hardened renderer as artifact previews (S.No 165), so it is consistent and not a temporary patch. Scope: Task and User Story/Epic detail (the reported surfaces); WorkItemDefect shows its description inside status Banners (different UX, not Task-Breakdown output) and Board cards show short snippets, both left as-is. Verified live: markdown renders in-panel with no nested card, no raw ** or backticks, no console errors; typecheck, lint and 20 frontend tests pass. User-verified on real work items.</t>
+  </si>
+  <si>
+    <t>A WorkItem could show state=done while its run was still awaiting_gate / in review, with no workitem.transitioned event — the build agent marked its own item done, bypassing the merge gate.</t>
+  </si>
+  <si>
+    <t>Seen repeatedly (WI-40, WI-44, WI-41, WI-60). The WorkItem showed done while its run was still in the review/remediation loop or awaiting the merge gate, with no workitem.transitioned event (the only legitimate done path always logs one) and no merge. It resolved 'correctly' later when the gate was approved, but the premature/orphaned done was misleading and — more seriously — meant work was marked complete without an approved gate (a control-plane gate bypass, non-negotiables #2/#5).</t>
+  </si>
+  <si>
+    <t>Orchestration / Gates / Companion agent capability + GitHub webhook reconciliation</t>
+  </si>
+  <si>
+    <t>commits 83a2036 (primary) + 05058d0 (secondary); agents/07_implementation/agent.md, backend/api/runner_views.py, backend/integrations/webhooks.py</t>
+  </si>
+  <si>
+    <t>Two paths let a WorkItem reach done without an approved gate or a transition event. PRIMARY: the 07 implementation agent was instructed (agent.md step R2/7) to transition the item 'toward done' with the transition_work_item MCP tool once it judged acceptance met, and the companion allow-listed that tool. So the engine marked its own task done when it finished coding — before code review and the merge gate — and the agent-facing tool path (tools.transition_work_item) logs no workitem.transitioned event. SECONDARY: the merged-PR webhook (_reconcile_pull_request) set the item done on any merged-PR event, even while a merge_gate was still PENDING, and logged only webhook.pr_merged, never workitem.transitioned.</t>
+  </si>
+  <si>
+    <t>PRIMARY (commit 83a2036): (1) agents/07_implementation/agent.md no longer tells the agent to transition the item to done — it only logs completion; the platform closes each remediation item when the review re-run no longer sees the finding, and marks the item done only after the merge gate. (2) The agent/companion state endpoint (RunnerStateView, the single HTTP entry for every platform-state call) now rejects a transition_work_item call whose to_state is 'done' with 403; the orchestrator calls the tool in-process, not through this view, so its legitimate post-approval transition is unaffected. SECONDARY (commit 05058d0): the merged-PR webhook now defers to the saga while a merge_gate is PENDING (records webhook.pr_merged + publishes the code pointer but does not transition), and when it does legitimately transition a genuine out-of-band merge it emits the canonical workitem.transitioned event. Tests in backend/tests/test_runner_state_api.py and test_webhook_reconcile.py. Non-build phases and the agent's own -&gt; in_progress transition are unaffected.</t>
+  </si>
+  <si>
+    <t>Takeover timeout marks a companion run terminally 'failed' even when the companion later comes back and reports the phase succeeded with artifacts registered — the late success does not reconcile the run, and the UI shows a false 'engine exited, no artifact' message.</t>
+  </si>
+  <si>
+    <t>Found 2026-07-13 on the SpendLog Architecture run. When a companion (local Claude Code) goes offline after a phase is dispatched, the orchestrator's takeover reconciler fires phase.takeover (reason 'companion offline / no report before timeout') and sets the run to a terminal 'failed' state. If the companion later comes back, completes the work, registers artifacts, and posts phase.reported status=ok, that late success does NOT reconcile the run out of 'failed'. Result: the run shows failed with the canned UI message 'The engine exited before reporting. No artifact was registered.' — which is factually wrong (artifacts were registered, report status was ok). Event sequence proving the race: dispatched 19:49:55Z -&gt; ~7.5h gap (laptop asleep) -&gt; phase.reclaimed 03:25:12Z -&gt; phase.takeover 03:27:37Z (run set failed) -&gt; 11 artifacts registered 03:55:04-03:55:40Z -&gt; phase.reported ok 03:56:57Z.</t>
+  </si>
+  <si>
+    <t>Orchestration / Takeover + phase-report reconciliation</t>
+  </si>
+  <si>
+    <t>Found 2026-07-13, SpendLog Architecture run 8738d4ba-72ee-460f-b41f-86556fca5658 (tenant 212395b8-f118-4eef-93eb-ba2c45468226). Code: takeover path in the orchestrator + phase-report handler (backend/api/runner_views.py phases/&lt;id&gt;/report/).</t>
+  </si>
+  <si>
+    <t>'failed' is a terminal state and swallows a later successful report. Takeover finalizes the run to failed while the companion is merely offline (e.g. laptop asleep), and nothing re-opens it when the companion returns and reports ok with artifacts — takeover wins a race it is about to lose.</t>
+  </si>
+  <si>
+    <t>OPEN — not yet fixed. Proposed: a successful late phase.reported (status=ok with registered artifacts) should reconcile the run to succeeded (the artifacts are the proof), OR takeover should not finalize while the companion is still making progress / a reclaim should re-open the run. Related operational trigger: companion-offline from laptop sleep stalls dispatched phases.</t>
+  </si>
+  <si>
+    <t>In Repository page - The optional Preview URL box is not alliged with the rest of the boxes (UX design) and the message comment below the box which says – “A running app for 09b to explore while writing tests” where the user wouldn’t know what is 09b and the message is not understandable for the user.</t>
+  </si>
+  <si>
+    <t>Repositories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workspace Dashboard &amp; Phases and Runs pages: 
+In Workspace Dashboard a separate box is present for the companion and it says “Connected --” and in Phases &amp; Runs page it display a light green box which shows “Companion ready --” The team believes the top navigation bar already shows the companion status and do not need a separate companion status messages in the workspace dashboard and phases &amp; runs page.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workspace Dashboard - Phases &amp; Runs </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run Concole page:
+When a user triggers a phase and navigates to the run console page to see the live progress - The page is displaying - Phases &amp; Runs: Id, Workflow Agent-run-Id and Engine: Claude. Now the team wants to understand what those IDs represent and is there a better way to humasize them because for a user they do not make any sense and he would not understand them.  
+Let say, the user created a “Work item 10” and he went to the phases and runs page and invoked the work item 10. Now he went to the run console page but, there he cannot know which work item is running. How does the user confirm that the right work item is running? This is a subtle part of the above issue – also needs fixing while fixing the above issue. 
+Team developer note: Sometimes ids are required for debugging. We have to understand what Ids are currently showing. Make them Human readable if required. </t>
+  </si>
+  <si>
+    <t>Run Console</t>
+  </si>
+  <si>
+    <t>Phases &amp; Runs Page:
+When the companion is offline – in the Trigger a Phase card – only Ideation, Requirements and PRD phases are shown as placeholders but should have shown all the phases. When the companion is online the page shows all the phases and they are clikable which is right response. 
+When the companion is offline: In the Runs card below the trigger a phase card: To the right-hand side, the most recent task is displayed which is not necessary and should be removed (no need any display) 
+When the companion is online: In the Runs card below, the trigger a phase card: To the right-hand side, the most recent task/phase is displayed which is the right response because the companion is online and ready to work.  
+Note: First, tell the team what the message is displayed dynamically there and will decide on removing or keeping it.</t>
+  </si>
+  <si>
+    <t>Clarifications Page:
+In the clarifications page: The default page states, "nothing is billed while it waits” message below the clarification header and “(billing $0) “text in the box below when no clarifications to present. The team decided to remove those two texts, and the rest of the message should be clealy aligned.</t>
   </si>
 </sst>
 </file>
@@ -3551,7 +3738,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="17">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="21">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -3620,6 +3807,22 @@
     <v>16</v>
     <v>5</v>
   </rv>
+  <rv s="0">
+    <v>17</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>18</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>19</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>20</v>
+    <v>5</v>
+  </rv>
 </rvData>
 </file>
 
@@ -3651,6 +3854,10 @@
   <rel r:id="rId15"/>
   <rel r:id="rId16"/>
   <rel r:id="rId17"/>
+  <rel r:id="rId18"/>
+  <rel r:id="rId19"/>
+  <rel r:id="rId20"/>
+  <rel r:id="rId21"/>
 </richValueRels>
 </file>
 
@@ -3955,7 +4162,7 @@
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33" style="2" customWidth="1"/>
     <col min="3" max="3" width="40" style="2" customWidth="1"/>
     <col min="4" max="4" width="16.140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="14" style="2" bestFit="1" customWidth="1"/>
@@ -7967,20 +8174,14 @@
       <c r="G136" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two compounding causes. (1) The companion ran in the GLOBAL Python with no venv, while the client app it builds (medslot / SDLC-expenselog) pins anyio==4.4.0 + httpx==0.27.0 in its own backend/requirements.txt. Any medslot build/preview `pip install -r requirements.txt` ran in that shared global env and downgraded anyio to 4.4.0, breaking claude-agent-sdk's engine launch (anyio.open_process(..., user=...) needs anyio&gt;=4.5) mid-build. (2) The repo's engine pins were also stale, so a clean install reproduced the broken combination. The earlier note treated this as pins-only; in practice the operative cause was the global-env pollution from the app being built.</t>
-        </is>
-      </c>
-      <c r="I136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed 2026-07-20/21. (a) Pinned the engine dep set in the repo (commit 28531e1): claude-agent-sdk==0.1.72, mcp==1.27.0, anyio==4.14.2. (b) Dedicated companion venv OUTSIDE all projects: C:\Users\Msi\sdlc-companion-venv; launch by the venv's absolute python path WITHOUT activating, so build-subprocess pip installs still hit the global env and can never reach the companion's anyio. (c) Startup guard (commit 8c34c24): serve/run call _assert_engine_env() and exit(2) with an actionable message if anyio can't launch the engine. Validated live: WI-38/39/60/41/42/44/45 retriggers all cleared the engine-launch step with no anyio error.</t>
-        </is>
-      </c>
-      <c r="J136" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
+      <c r="H136" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="I136" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="J136" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="409.6" customHeight="1">
@@ -8585,7 +8786,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="159" spans="1:10">
+    <row r="159" spans="1:10" ht="409.6">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -8649,7 +8850,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="161" spans="1:10">
+    <row r="161" spans="1:10" ht="409.6">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -8681,165 +8882,129 @@
         <v>762</v>
       </c>
     </row>
-    <row r="162" spans="1:10">
+    <row r="162" spans="1:10" ht="409.6">
       <c r="A162" s="2">
         <v>161</v>
       </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">When a build's remediation loop hit its cycle cap it hard-failed the WorkItem with no diagnostics and no way forward — the user could not complete the WorkItem.</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The 07&lt;-&gt;08 remediation loop was capped at max_remediation_cycles. On exhaustion the workflow raised a hard failure and stopped. The run console showed only blocking-finding COUNTS across cycles (e.g. 2 -&gt; 1 -&gt; 3 -&gt; 3) with no visibility into what the findings actually were, and there was no automated retry — a human had to step in, defeating the automation promise. If remediation kept exhausting, the WorkItem was simply stuck.</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Orchestration / Build saga / Remediation</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commit 29e934b; backend/orchestration/build_workflow.py, build_activities.py (handle_remediation_exhausted), trigger.py, build_types.py</t>
-        </is>
-      </c>
-      <c r="G162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On remediation exhaustion the workflow had a single terminal branch (hard fail). It neither captured the real blocking-finding text nor attempted a fresh build attempt, so an exhausted WorkItem had nowhere to go.</t>
-        </is>
-      </c>
-      <c r="I162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commit 29e934b. run_code_review now persists the actual blocking-finding detail (rem/severity/title/file/line) into run.outputs['review_cycles'], not just counts. New handle_remediation_exhausted activity: if attempt &lt; max_auto_attempts (default 2) it marks the current run failed with a clear 'auto-retrying' message, logs build.remediation_exhausted_retry, and re-triggers the build with attempt+1 and a seeded prior_attempt_context digest of what blocked the prior attempt — fully automated, no human. Only after all auto-attempts are exhausted does it park for a human. Tests in backend/tests/test_build_activities.py. Validated live 2026-07-21: WI-60 fired build.remediation_exhausted_retry {attempt:1,next_attempt:2} and auto-started attempt 2.</t>
-        </is>
-      </c>
-      <c r="J162" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="163" spans="1:10">
+      <c r="B162" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F162" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="G162" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H162" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="I162" s="2" t="s">
+        <v>768</v>
+      </c>
+      <c r="J162" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" ht="388.5">
       <c r="A163" s="2">
         <v>162</v>
       </c>
-      <c r="B163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A build's remediation could start from an empty tree or push a non-fast-forward when a different companion continued a WorkItem than the one that started it — remediation work was lost or the push was rejected.</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Each companion provisioned its worktree from its own LOCAL branch state. When companion B continued a WorkItem that companion A had started and pushed, B based the worktree on a stale or absent local ref, producing either an empty build or a non-fast-forward push that failed during the remediation cycle. Subsumes the older stale-local-branch empty-build issue (#145).</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Companion / Worktree provisioning</t>
-        </is>
-      </c>
-      <c r="E163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commits 9863c16, d008643; runner/companion/worktree.py (provision_worktree)</t>
-        </is>
-      </c>
-      <c r="G163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">provision_worktree based the worktree on a possibly-stale local remote-tracking ref. git fetch does not prune, so a stale origin/&lt;branch&gt; ref (left after the remote branch was deleted) could resurrect a dead branch at an old commit; and a genuinely continued branch was never re-fetched from the true remote tip.</t>
-        </is>
-      </c>
-      <c r="I163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commits 9863c16 + d008643. provision_worktree now authoritatively checks `git ls-remote --heads &lt;remote&gt; &lt;branch&gt;`. If the branch exists on the remote it fetches and bases the worktree on &lt;remote&gt;/&lt;branch&gt; (git worktree add -B branch &lt;remote-tip&gt;), so ANY companion continues from the true shared work-in-progress; it falls back to `base` only for a genuinely new/offline branch. Tests in backend/tests/test_companion_runner.py (validated on the host with real git; the container has no git binary). Validated live: WI-39's remediation cycle pushed successfully after previously failing.</t>
-        </is>
-      </c>
-      <c r="J163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="164" spans="1:10">
+      <c r="B163" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="G163" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H163" s="2" t="s">
+        <v>773</v>
+      </c>
+      <c r="I163" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="J163" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" ht="409.6">
       <c r="A164" s="2">
         <v>163</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>763</v>
+        <v>775</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>764</v>
+        <v>776</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>765</v>
+        <v>777</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>766</v>
+        <v>778</v>
       </c>
       <c r="G164" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H164" s="2" t="s">
-        <v>767</v>
+        <v>779</v>
       </c>
       <c r="I164" s="2" t="s">
-        <v>768</v>
+        <v>780</v>
       </c>
       <c r="J164" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="165" spans="1:10">
+    <row r="165" spans="1:10" ht="226.5">
       <c r="A165" s="2">
         <v>164</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>769</v>
+        <v>781</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>770</v>
+        <v>782</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>765</v>
+        <v>777</v>
       </c>
       <c r="E165" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>771</v>
+        <v>783</v>
       </c>
       <c r="G165" s="2" t="s">
         <v>23</v>
       </c>
       <c r="H165" s="2" t="s">
-        <v>772</v>
+        <v>784</v>
       </c>
       <c r="I165" s="2" t="s">
-        <v>773</v>
+        <v>785</v>
       </c>
       <c r="J165" s="2" t="s">
         <v>141</v>
@@ -8850,7 +9015,7 @@
         <v>165</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>774</v>
+        <v>786</v>
       </c>
       <c r="D166" s="2" t="s">
         <v>93</v>
@@ -8864,245 +9029,248 @@
       <c r="G166" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H166" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not a content bug - the artifact's diagrams and matrix were valid markdown. In the shared Markdown renderer (frontend/src/components/ui/Markdown.tsx) the rendered Mermaid diagram was placed in a div carrying the class 'diagram-frame', whose CSS rule '.diagram-frame svg { width:40px; height:40px }' - intended only for the empty-state placeholder icon - shrank every real diagram to a 40x40 px smudge. Confirmed by fetching both tenants' System Architecture artifacts from S3: test@edvensoft.com had 0 Mermaid diagrams (so it never hit the bug and looked fine), while test2@edvensoft.com had 3 valid 'graph TD' diagrams that got shrunk. Separately, GFM tables (the NFR-to-Architecture Traceability Matrix) rendered as a plain width:100% table with no scroll container, so a wide matrix over-extended its pane instead of scrolling. Both are shared-renderer defects, so they affect any artifact with diagrams or wide tables in any phase - which is why the same issue was expected to recur in later phases.</t>
-        </is>
-      </c>
-      <c r="I166" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Surgical fix in the shared Markdown renderer (frontend only - no backend, no DB, no agent change). (1) Diagrams: the rendered container no longer reuses the 'diagram-frame' placeholder class - it uses its own '.md-body__mermaid' class that owns its sizing (svg max-width:100%, height:auto), so diagrams render full size instead of 40x40. (2) Tables: every table is wrapped in a '.md-body__table-wrap' scroll container (overflow-x:auto, max-width:100%), so wide tables scroll inside their pane instead of spilling. Because the fix lives in the shared renderer it covers every phase/artifact and will not recur. Verified live in the running app: the demo diagram rendered at 582x299 px (not 40x40) with no 'diagram-frame' leak, and at mobile width a wide table scrolled inside its wrapper with the page NOT overflowing horizontally. Unit tests (Markdown.test.tsx), typecheck and lint all pass. Files: Markdown.tsx, components.css. To see it: restart the frontend container and hard-refresh the browser - no agent re-run needed, the stored artifact body is unchanged.</t>
-        </is>
-      </c>
-      <c r="J166" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="167" spans="1:10">
+      <c r="H166" s="2" t="s">
+        <v>787</v>
+      </c>
+      <c r="I166" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="J166" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" ht="409.6">
       <c r="A167" s="2">
         <v>166</v>
       </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Work-item search dropdown (Combobox) is clipped for a small list - some items are unreachable because the list only scrolls when it is very long</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On the Phases &amp; Runs page, the 'Search work items' dropdown shows only the first few items and the rest are cut off with no way to scroll to them when there is a small/limited number of work items. A scrollbar only appears when the list is very long. Observed with 6 work items: WI-6/WI-5/WI-4 show and the remaining ones are clipped and unreachable.</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phases &amp; Runs / Combobox</t>
-        </is>
-      </c>
-      <c r="E167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Repro: Phases &amp; Runs &gt; 'Search work items' with ~6 work items - the dropdown is cut off at the panel edge and cannot be scrolled to reach the hidden items. With many work items an internal scrollbar appears and all items are reachable.</t>
-        </is>
-      </c>
-      <c r="G167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P3</t>
-        </is>
-      </c>
-      <c r="H167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The shared Combobox dropdown (.combobox__list, frontend/src/components/ui) is absolutely positioned with max-height:260px and overflow-y:auto, and it sits inside a Panel whose CSS '.panel { overflow: hidden }' (used for rounded corners) clips the dropdown at the panel edge. When the list is shorter than 260px it gets NO internal scrollbar, so items past the panel edge are clipped and unreachable; only when the list exceeds 260px does the internal scrollbar appear - which is why 'scroll works' only with many items.</t>
-        </is>
-      </c>
-      <c r="I167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two options - team to decide, then fix. Option A (surgical, low-risk, recommended for this screen): stop the Trigger-a-phase Panel from clipping the floating dropdown - add a modifier class (e.g. .panel--menu { overflow: visible }) applied to that one panel; touches PhasesAndRuns.tsx + components.css; fixes this screen only. Option B (general): render the Combobox dropdown in a portal to document.body so it can never be clipped by any container - fixes every Combobox everywhere but is a larger change to the shared component (position calc, reposition on scroll/resize, test updates). Recommend A now; upgrade to B if the same clipping shows up on other screens.</t>
-        </is>
-      </c>
-      <c r="J167" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="168" spans="1:10">
+      <c r="B167" s="2" t="s">
+        <v>789</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>790</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>791</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F167" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H167" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="I167" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="J167" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" ht="409.6">
       <c r="A168" s="2">
         <v>167</v>
       </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Work-item (Epic / User Story / Task) descriptions from Task Breakdown are shown as raw markdown - the content is good but not rendered (bold, code, tables and lists appear as literal ** ` | characters)</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In the work-item detail pages, the Description that the Task Breakdown agent writes is good but is displayed as plain text: markdown like **bold**, `code`, pipe tables and bullet lists appear as literal characters instead of being rendered, so it is not user-friendly. Observed on TASK-006, TASK-015 and US-009 (Story). General rule the team wants: wherever the app shows content that is meant to be markdown, it must render in a user-friendly way.</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Work Items / Content rendering</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evidence (screenshots shared with the team): TASK-006 and TASK-015 Description panels and the US-009 'Description &amp; context' panel show literal '**Type:**', '**What to build:**', backtick-quoted code and pipe-tables as plain text instead of rendered markdown.</t>
-        </is>
-      </c>
-      <c r="G168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The work-item detail views render the description as PLAIN TEXT in a &lt;p&gt; tag instead of through the shared Markdown renderer: WorkItemTask.tsx (line 134), WorkItemEpic.tsx (line 97) and WorkItemDefect.tsx all do '&lt;p className="t-body"&gt;{workItem.data.description}&lt;/p&gt;'. The Markdown component (frontend/src/components/ui/Markdown.tsx - GFM via react-markdown + remark-gfm, already used for artifact previews and hardened in S.No 165) is never applied to work-item descriptions, so the agent's markdown shows raw.</t>
-        </is>
-      </c>
-      <c r="I168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FIXED. Routed work-item descriptions through the shared Markdown renderer (frontend/src/components/ui/Markdown.tsx) instead of a plain &lt;p&gt;. Added an optional className prop to Markdown (default 'doc-preview prose md-body') so it renders inside an existing Panel without a nested card; WorkItemTask.tsx and WorkItemEpic.tsx now render the description with &lt;Markdown className='prose md-body'&gt;, keeping the 'No description yet.' fallback. Bold, inline code, lists and tables now render correctly. Reuses the same hardened renderer as artifact previews (S.No 165), so it is consistent and not a temporary patch. Scope: Task and User Story/Epic detail (the reported surfaces); WorkItemDefect shows its description inside status Banners (different UX, not Task-Breakdown output) and Board cards show short snippets, both left as-is. Verified live: markdown renders in-panel with no nested card, no raw ** or backticks, no console errors; typecheck, lint and 20 frontend tests pass. User-verified on real work items.</t>
-        </is>
-      </c>
-      <c r="J168" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="169" spans="1:10">
+      <c r="B168" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>797</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F168" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="G168" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H168" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="I168" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="J168" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" ht="409.6">
       <c r="A169" s="2">
         <v>168</v>
       </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A WorkItem could show state=done while its run was still awaiting_gate / in review, with no workitem.transitioned event — the build agent marked its own item done, bypassing the merge gate.</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seen repeatedly (WI-40, WI-44, WI-41, WI-60). The WorkItem showed done while its run was still in the review/remediation loop or awaiting the merge gate, with no workitem.transitioned event (the only legitimate done path always logs one) and no merge. It resolved 'correctly' later when the gate was approved, but the premature/orphaned done was misleading and — more seriously — meant work was marked complete without an approved gate (a control-plane gate bypass, non-negotiables #2/#5).</t>
-        </is>
-      </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Orchestration / Gates / Companion agent capability + GitHub webhook reconciliation</t>
-        </is>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">commits 83a2036 (primary) + 05058d0 (secondary); agents/07_implementation/agent.md, backend/api/runner_views.py, backend/integrations/webhooks.py</t>
-        </is>
-      </c>
-      <c r="G169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="H169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two paths let a WorkItem reach done without an approved gate or a transition event. PRIMARY: the 07 implementation agent was instructed (agent.md step R2/7) to transition the item 'toward done' with the transition_work_item MCP tool once it judged acceptance met, and the companion allow-listed that tool. So the engine marked its own task done when it finished coding — before code review and the merge gate — and the agent-facing tool path (tools.transition_work_item) logs no workitem.transitioned event. SECONDARY: the merged-PR webhook (_reconcile_pull_request) set the item done on any merged-PR event, even while a merge_gate was still PENDING, and logged only webhook.pr_merged, never workitem.transitioned.</t>
-        </is>
-      </c>
-      <c r="I169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PRIMARY (commit 83a2036): (1) agents/07_implementation/agent.md no longer tells the agent to transition the item to done — it only logs completion; the platform closes each remediation item when the review re-run no longer sees the finding, and marks the item done only after the merge gate. (2) The agent/companion state endpoint (RunnerStateView, the single HTTP entry for every platform-state call) now rejects a transition_work_item call whose to_state is 'done' with 403; the orchestrator calls the tool in-process, not through this view, so its legitimate post-approval transition is unaffected. SECONDARY (commit 05058d0): the merged-PR webhook now defers to the saga while a merge_gate is PENDING (records webhook.pr_merged + publishes the code pointer but does not transition), and when it does legitimately transition a genuine out-of-band merge it emits the canonical workitem.transitioned event. Tests in backend/tests/test_runner_state_api.py and test_webhook_reconcile.py. Non-build phases and the agent's own -&gt; in_progress transition are unaffected.</t>
-        </is>
-      </c>
-      <c r="J169" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="170" spans="1:10">
+      <c r="B169" s="2" t="s">
+        <v>801</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>802</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F169" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="G169" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H169" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="I169" s="2" t="s">
+        <v>806</v>
+      </c>
+      <c r="J169" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" ht="388.5">
       <c r="A170" s="2">
         <v>169</v>
       </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takeover timeout marks a companion run terminally 'failed' even when the companion later comes back and reports the phase succeeded with artifacts registered — the late success does not reconcile the run, and the UI shows a false 'engine exited, no artifact' message.</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Found 2026-07-13 on the SpendLog Architecture run. When a companion (local Claude Code) goes offline after a phase is dispatched, the orchestrator's takeover reconciler fires phase.takeover (reason 'companion offline / no report before timeout') and sets the run to a terminal 'failed' state. If the companion later comes back, completes the work, registers artifacts, and posts phase.reported status=ok, that late success does NOT reconcile the run out of 'failed'. Result: the run shows failed with the canned UI message 'The engine exited before reporting. No artifact was registered.' — which is factually wrong (artifacts were registered, report status was ok). Event sequence proving the race: dispatched 19:49:55Z -&gt; ~7.5h gap (laptop asleep) -&gt; phase.reclaimed 03:25:12Z -&gt; phase.takeover 03:27:37Z (run set failed) -&gt; 11 artifacts registered 03:55:04-03:55:40Z -&gt; phase.reported ok 03:56:57Z.</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Orchestration / Takeover + phase-report reconciliation</t>
-        </is>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bug</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Found 2026-07-13, SpendLog Architecture run 8738d4ba-72ee-460f-b41f-86556fca5658 (tenant 212395b8-f118-4eef-93eb-ba2c45468226). Code: takeover path in the orchestrator + phase-report handler (backend/api/runner_views.py phases/&lt;id&gt;/report/).</t>
-        </is>
-      </c>
-      <c r="G170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="H170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">'failed' is a terminal state and swallows a later successful report. Takeover finalizes the run to failed while the companion is merely offline (e.g. laptop asleep), and nothing re-opens it when the companion returns and reports ok with artifacts — takeover wins a race it is about to lose.</t>
-        </is>
-      </c>
-      <c r="I170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN — not yet fixed. Proposed: a successful late phase.reported (status=ok with registered artifacts) should reconcile the run to succeeded (the artifacts are the proof), OR takeover should not finalize while the companion is still making progress / a reclaim should re-open the run. Related operational trigger: companion-offline from laptop sleep stalls dispatched phases.</t>
-        </is>
-      </c>
-      <c r="J170" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="171" spans="1:10">
+      <c r="B170" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F170" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="G170" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H170" s="2" t="s">
+        <v>811</v>
+      </c>
+      <c r="I170" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="J170" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" ht="210.75">
       <c r="A171" s="2">
         <v>170</v>
       </c>
-    </row>
-    <row r="172" spans="1:10">
+      <c r="B171" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="E171" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F171" s="2" t="e" vm="18">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G171" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J171" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" ht="243">
       <c r="A172" s="2">
         <v>171</v>
       </c>
-    </row>
-    <row r="173" spans="1:10">
+      <c r="B172" s="2" t="s">
+        <v>815</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>816</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F172" s="2" t="e" vm="19">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G172" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J172" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" ht="409.6">
       <c r="A173" s="2">
         <v>172</v>
       </c>
-    </row>
-    <row r="174" spans="1:10">
+      <c r="B173" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>818</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F173" s="2" t="e" vm="20">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G173" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J173" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" ht="409.6">
       <c r="A174" s="2">
         <v>173</v>
       </c>
-    </row>
-    <row r="175" spans="1:10">
+      <c r="B174" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F174" s="2" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G174" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J174" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" ht="194.25">
       <c r="A175" s="2">
         <v>174</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>820</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="176" spans="1:10">

</xml_diff>

<commit_message>
Re-updated the Bugs sheet
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="207" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A04FBDF-F9BB-4AA7-B306-D4BE47860DD0}"/>
+  <xr:revisionPtr revIDLastSave="217" documentId="11_14FDEAE3397E350B81F2A24CBED9C52169691D91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B39CCE5D-1D7C-4DAE-8871-EA9F0B2E43B3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="21">
+  <futureMetadata name="XLRICHVALUE" count="23">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -186,8 +186,22 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="21"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="22"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="21">
+  <valueMetadata count="23">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -251,12 +265,18 @@
     <bk>
       <rc t="1" v="20"/>
     </bk>
+    <bk>
+      <rc t="1" v="21"/>
+    </bk>
+    <bk>
+      <rc t="1" v="22"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1393" uniqueCount="821">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="822">
   <si>
     <t>S.No</t>
   </si>
@@ -2895,6 +2915,11 @@
   <si>
     <t>Clarifications Page:
 In the clarifications page: The default page states, "nothing is billed while it waits” message below the clarification header and “(billing $0) “text in the box below when no clarifications to present. The team decided to remove those two texts, and the rest of the message should be clealy aligned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phases &amp; Runs page: 
+After the user has connected the companion and selects the work item and triggers a phase – A Runs card shows in the page where the card shows info about the tiggered run and a link to navigate the run console page. Now here the team has decided to revome the “COST(EST)” column which is not needed anymore and the message below the card is also to be revomed (not needed any more). Those details were added for the testing purposes and do not need any more. 
+Note: Also check whether the same behaviour happens in the UI, like for example: while a clarification gate has opend and does a recon over the complete SDLC app and tell the team whether the same scenario of issues appears anywhere? </t>
   </si>
 </sst>
 </file>
@@ -3738,7 +3763,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="21">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="23">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -3823,6 +3848,14 @@
     <v>20</v>
     <v>5</v>
   </rv>
+  <rv s="0">
+    <v>21</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>22</v>
+    <v>5</v>
+  </rv>
 </rvData>
 </file>
 
@@ -3858,6 +3891,8 @@
   <rel r:id="rId19"/>
   <rel r:id="rId20"/>
   <rel r:id="rId21"/>
+  <rel r:id="rId22"/>
+  <rel r:id="rId23"/>
 </richValueRels>
 </file>
 
@@ -9272,10 +9307,37 @@
       <c r="E175" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="176" spans="1:10">
+      <c r="F175" s="2" t="e" vm="22">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G175" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J175" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" ht="409.6">
       <c r="A176" s="2">
         <v>175</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E176" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F176" s="2" t="e" vm="23">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G176" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J176" s="2" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="177" spans="1:1">

</xml_diff>

<commit_message>
Bugs sheet: log 4 mid-run recovery + UI gaps (S.No 181-184, Open)
From today's recon of how a failed phase can continue rather than restart:
- 181 (P2) Build: an initial-build companion failure is terminal-only, no resume.
- 182 (P1) Planning/Scan: a mid-run engine/session-limit failure fails terminally
  with no resume - only a fresh re-run from scratch (yesterday's security case).
- 183 (P2) Planning/Scan: no finding/artifact-level idempotency, so a re-run
  duplicates what the failed run already produced.
- 184 (P3) Clarifications UI: the native select's long options overflow the card.

Each row carries a code-grounded root cause and a planned surgical fix. Fixes to
follow. Sheet edited image-safe (in-cell screenshots preserved).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -9625,24 +9625,184 @@
         </is>
       </c>
     </row>
-    <row r="182" spans="1:1">
+    <row r="182" spans="1:10">
       <c r="A182" s="2">
         <v>181</v>
       </c>
-    </row>
-    <row r="183" spans="1:1">
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build phase: a companion-reported failure of the INITIAL build (before or at the first report) is terminal - the user cannot resume, only re-run from scratch. When the build agent's first report is status!=ok (e.g. the Claude session/usage limit is hit during the build itself, or the engine errors before reporting), the build workflow runs mark_build_failed and ends. The Run console then offers only 'Retry run' (a brand-new run), never 'Resume from where it stopped'. Every OTHER build error (open PR, merge, remediation) parks and is resumable - only this first-report failure is a dead end. S.No 162 branch-continuity helps only if a branch was already pushed; if the limit hits before any push, the whole build restarts. Blocks a user mid-build with no way to carry on.</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build phase / Implementation</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recon 2026-07-22. Verified: backend/orchestration/build_workflow.py:130-135 (report.status!=ok -&gt; mark_build_failed -&gt; return build_failed, terminal); the resumable _park branches are all inside the PR/review/merge block (:205,:264,:311), AFTER the first ok report; dispatch_build (:111-114) sits outside it; frontend RunConsole.tsx:236-249 shows 'Retry run' for status=failed and 'Resume' only for status=stalled.</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The initial-build report failure is routed to mark_build_failed (terminal) instead of the S.No 157 park path. dispatch_build is outside the resumable while-loop, so an engine/usage failure during it has no park branch; the Temporal workflow closes and a closed workflow can never be signalled to resume - so the only recovery is a fresh trigger.</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED (team to fix 2026-07-22): classify the initial-build report failure (reuse classify_build_failure) - when it is a usage/session/rate-limit or a transient engine failure, PARK the build as resumable (park_build, resume_from='dispatch_build') instead of mark_build_failed, so the workflow stays alive and 'Resume from where it stopped' re-dispatches; keep genuinely terminal failures on mark_build_failed. Combine with S.No 162 branch continuity so a resume continues the already-pushed branch.</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" spans="1:10">
       <c r="A183" s="2">
         <v>182</v>
       </c>
-    </row>
-    <row r="184" spans="1:1">
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planning &amp; Scan phases (ideation..deployment, and the Security scan): a mid-run engine failure fails the whole run terminally with NO resume - the user must re-run from scratch. When the companion reports the phase status!=ok (e.g. the Claude session/usage limit is hit mid-run, or the agent/engine errors), AgentRunWorkflow runs fail_run and ends. The Run console offers only 'Retry run', which starts a brand-new run from zero - there is no 'Resume from where it stopped'. Partial work already produced (e.g. security findings already registered) is not continued. This is exactly what hit the Security run on 2026-07-21 (failed on the session limit; a rerun must redo the entire scan). Remediation-exhaust does NOT apply here (planning/scan have no remediation loop). The only resumable park on this path is the narrow verify_writes case (a run that reported OK but is missing its artifact) - not a mid-run failure.</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planning &amp; Scan phases / Runs</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recon 2026-07-22. Verified: backend/orchestration/workflows.py:122-127 (report.status!=ok -&gt; fail_run -&gt; return phase_failed, terminal); the only _park on this workflow is the verify_writes check at :147-159 (post-report, artifact-missing); no remediation loop exists on this workflow; frontend RunConsole.tsx:236-249 gives 'Retry run' (fresh) for status=failed.</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A companion-reported phase failure is routed to fail_run (terminal) rather than the S.No 157 park path, which is wired ONLY around the verify_writes write-completeness check. So a mid-run engine/usage failure has no resumable branch - the workflow closes and cannot be signalled, forcing a fresh trigger. Planning/scan also produce no branch, so there is no S.No 162-style continuity to fall back on.</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED (team to fix 2026-07-22, TWO-part surgical fix - both parts required to be bulletproof; part 2 is logged separately as S.No 183): (1) On a companion-reported failure, classify it (reuse classify_phase_failure): if it is a usage/session/rate-limit or a transient engine failure, PARK the run resumable (park_run, resume_from='dispatch_phase') instead of fail_run, keeping the Temporal workflow alive so 'Resume from where it stopped' re-dispatches the remaining work; keep genuinely terminal failures on fail_run. (2) Depends on finding/artifact-level idempotency (S.No 183) so the resume/rerun continues rather than duplicating.</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" spans="1:10">
       <c r="A184" s="2">
         <v>183</v>
       </c>
-    </row>
-    <row r="185" spans="1:1">
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planning &amp; Scan phases: no artifact/finding-level idempotency, so a re-run (or a future resume) DUPLICATES what a failed run already produced. Idempotency today is keyed by run_id only (execute_agent_core skips duplicates only within the SAME run); a fresh Retry gets a NEW run_id, so nothing dedups against the failed run's already-registered artifacts. Concretely, the Security scan that failed on 2026-07-21 had already registered findings SEC-001..004; a fresh rerun re-scans and can register the same findings again as new artifacts (and, once the defect loopback of S.No 177 is wired, could open duplicate defect work items). This makes any 'continue after a failure' unsafe and must be fixed for the S.No 182 resume to be bulletproof.</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planning &amp; Scan phases / Artifacts</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recon 2026-07-22. Verified: backend/orchestration/activities.py execute_agent_core is idempotent by run_id only; a re-trigger creates a new Run/run_id (frontend RunConsole.tsx:141-148 handleRetry -&gt; trigger by agent_key); security findings carry a stable external_ref finding_id (SEC-00x) but nothing dedups artifacts across runs of the same work_item+phase.</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artifact registration has no natural key beyond run_id, so across a failed run and its fresh retry there is no dedup on (work_item, phase, expected type / finding_id); partial output from the failed run is neither reused nor suppressed - it is duplicated.</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED (team to fix 2026-07-22): add finding/artifact-level idempotency keyed on a stable natural key - for findings the external_ref finding_id (SEC-00x); for phase artifacts (work_item, phase, type). On register, upsert by that key within the work_item+phase scope instead of always inserting, so a resumed or re-triggered run continues (updates/skips existing) rather than duplicating. Pairs with S.No 182.</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" spans="1:10">
       <c r="A185" s="2">
         <v>184</v>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clarifications page: the answer dropdown's option list overflows OUTSIDE the clarification card and looks broken. The Tier-1 'choice' answer control is a native select; when the agent's options are long sentences (seen live in a build-phase clarification - TASK-033, run dd5080df - e.g. 'Create a new backlog task for expenses CRUD router (GET/POST/PATCH/DELETE /api/v1/expenses) and merge TASK-033 as-is...'), the browser-drawn option popup extends past the card's left/right edges and the long option text does not wrap, so option text spills outside the window. Cosmetic but unpolished and can push text off-screen.</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clarifications / UI</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI issue</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recon 2026-07-22. Verified: frontend/src/features/lifecycle/Clarifications.tsx:190-203 renders a native &lt;Select&gt; (design-system wrapper over &lt;select&gt;) with one &lt;option&gt; per agent-provided q.options; native &lt;select&gt; option popups are browser/OS-drawn (not in the DOM flow) so they are not clipped to the card, and native &lt;option&gt; text cannot be made to wrap - long option strings render on one line and overflow horizontally.</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The choice answer uses a native HTML select. A native select's option dropdown is rendered by the browser outside the page layout, so it is not constrained/clipped to the clarification card, and native &lt;option&gt; elements cannot be styled to wrap - long option labels render single-line and spill past the card bounds.</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED (team to fix 2026-07-22): replace the native select for clarification choices with a custom, card-constrained dropdown/listbox (popup width bounded to the field, long options wrap or truncate-with-tooltip), OR render long-option questions as a radio-button list (each option on its own wrapping line) instead of a dropdown. Preserve the isOtherOption free-text reveal behaviour (Clarifications.tsx:77).</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="186" spans="1:1">

</xml_diff>

<commit_message>
Stop the CICD agent hardcoding secrets in the local docker-compose file
The CICD agent was told to generate a docker-compose.yml with database and
cache services but given no rule about secret values, so it wrote a real
generated dev password straight into the file. The companion's pre-push secret
scan correctly flagged it and blocked the push, so the build finished all its
work but never opened a PR.

Added an explicit rule in Step 3 to reference every credential as an
environment variable and ship a .env.example placeholder instead of a literal,
and reinforced the same point in the quality gate. Verified live end to end: a
fresh CICD run then went through code, PR, code-review remediation, and merge
with no secret-scan block.

Also updates the bug log (Bugs.xlsx): S.No 193 for this fix (now validated),
plus the earlier email-delivery enhancement and context-provisioning entries.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -10120,14 +10120,94 @@
         </is>
       </c>
     </row>
-    <row r="193" spans="1:1">
+    <row r="193" spans="1:10">
       <c r="A193" s="2">
         <v>192</v>
       </c>
-    </row>
-    <row r="194" spans="1:1">
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invitation &amp; password-reset emails are NOT actually delivered to users - the invitee only sees the accept/reset link in the dev console (server terminal log), never in an inbox. EMAIL_BACKEND defaults to Django's console backend and there is no SendGrid (or any SMTP/API) delivery wired for production. Today an admin must copy the invitation link out of the server log and share it manually (Slack/chat). Enhancement: turn on real transactional email delivery so invited users receive their invitation (and password resets) by email.</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auth / Tenant invitations + password reset (email delivery)</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verified 2026-07-23. The email SEND code is already complete and wired: backend/apps/tenancy/emails.py (send_invitation_email / send_password_reset_email over Django send_mail), called on invitation create (backend/api/views.py:702) and on password reset. Links are built from FRONTEND_BASE_URL. The only stub is the delivery backend: backend/config/settings.py:169 EMAIL_BACKEND defaults to django.core.mail.backends.console.EmailBackend (prints to log instead of sending).</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intentional dev stub, not a defect. EMAIL_BACKEND is a deliberate pluggable seam set to the console backend for local dev (links print to the log). No production mail backend/credentials were configured and no SendGrid integration exists yet, so nothing is transmitted over the wire.</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED - config only, no code change needed. Recommended: use Django's built-in SMTP backend against SendGrid's SMTP relay. Set EMAIL_BACKEND=django.core.mail.backends.smtp.EmailBackend, EMAIL_HOST=smtp.sendgrid.net, EMAIL_PORT=587, EMAIL_USE_TLS=True, EMAIL_HOST_USER=apikey (literal), EMAIL_HOST_PASSWORD=&lt;SENDGRID_API_KEY&gt;, DEFAULT_FROM_EMAIL=&lt;verified sender e.g. no-reply@edvensoft.com&gt;, and a correct FRONTEND_BASE_URL. Team side (in SendGrid, not our code): (1) verify a sender or domain via DNS auth, (2) generate an API key. Effort: a few hours, mostly the SendGrid sender verification; no new Python package required. Optional polish: add an EMAIL_* block to .env.example + a short docs note so it is a drop-in when creds arrive. The same seam also switches on password-reset emails.</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" spans="1:10">
       <c r="A194" s="2">
         <v>193</v>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Triggering the CI/CD phase (11_cicd) runs the agent to completion and registers its artifacts, but the build then FAILS at the very last step: the companion's pre-push secret scan blocks the branch push, so no PR is ever opened. Live: SpendLog WI-146 run cab0535c failed with '[high_entropy_secret] docker-compose.yml:64 - dev-***rs (55 chars)'. The CICD agent's Step 3 tells it to generate a local docker-compose.yml with database + cache services but gives NO secret-handling guidance, so the agent hardcodes a real generated dev password/token literal into the compose file. The pre-push guardrail correctly flags it and blocks the push (a TRUE positive), killing the build after all agent work is done.</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CI/CD phase (11_cicd) - generated docker-compose.yml</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verified 2026-07-23. Confirmed AGENT-SIDE: docker-compose.yml exists nowhere on the SpendLog repo default branch (TARUN51/medslot-single-repo main has only backend/Dockerfile + backend/.env.example + frontend/.env.example), and the run's branch feature/WI-79a3804c never reached GitHub (push was blocked) - so the file was freshly generated by 11_cicd this run. Scanner working as intended: runner/companion/guardrails.py:59-75 flags a secret/password/token key assigned a &gt;=20-char, high-entropy (Shannon&gt;=3.5), non-placeholder value; ${VAR}/placeholder values are skipped. agents/11_cicd/agent.md Step 3 (compose) had no no-hardcode rule, unlike Step 2 (Dockerfile: 'no secrets in the Dockerfile'). Platform passes the finding through unchanged (backend/orchestration/build_activities.py:427); run is terminal so the console shows 'Retry run'. Note S.No 130 (commit 52533c4) only made the finding readable - it did not cause or change the block.</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The 11_cicd agent body's Step 3 instructs generating a local docker-compose.yml with database + cache services (which need credentials) but - unlike the Dockerfile and Jenkinsfile steps - never says how to handle those secret values. The agent therefore hardcodes a concrete dev credential literal, which the companion's pre-push secret scan (PG14) correctly blocks. NOT a scanner defect - the scanner did its job; the agent violated the 'never hardcode secrets' principle its own quality gate already states.</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-07-23 (agent-body fix; team to re-test). agents/11_cicd/agent.md Step 3 now explicitly forbids hardcoding any secret in the compose file (even a dev DB/cache password) and requires env-var references (e.g. POSTGRES_PASSWORD: ${POSTGRES_PASSWORD} or env_file) plus a committed .env.example with placeholders only; the git-ignored real .env holds values. The Quality Gate line was also extended to cover local compose credentials, noting a hardcoded high-entropy value trips the pre-push scan. Scanner intentionally NOT weakened (that would let real secrets through). Immediate unblock: replace the literal on docker-compose.yml:64 with an env reference and re-trigger; a fresh run with the fixed agent body should no longer hardcode. VALIDATED LIVE 2026-07-23: a fresh end-to-end CICD run on SpendLog succeeded - agent wrote code, opened the PR, ran the code-review remediation loop, and merged with NO secret-scan block. Fix confirmed working.</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
       </c>
     </row>
     <row r="195" spans="1:1">

</xml_diff>

<commit_message>
Add the executive demo deck and log recent bug entries
Adds the interactive SDLC executive-preview deck (docs/demo) used for the COO
demo — opening pitch, the intelligence story, and a per-agent behind-the-scenes
explorer for narrating runs.

Updates the bug log with the entries raised over the last few sessions: the
email-delivery enhancement, the CICD secret-hardcode fix, the deployment
honesty + readiness-gate fixes, the platform-executed-deployment enhancement,
and the greenfield knowledge-index enhancement.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -10345,9 +10345,49 @@
         </is>
       </c>
     </row>
-    <row r="198" spans="1:1">
+    <row r="198" spans="1:10">
       <c r="A198" s="2">
         <v>197</v>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Greenfield flow does NOT populate the Knowledge Index, so its retrieval is dead for greenfield projects. The Knowledge Index (apps/knowledge) chunks artifact bodies into KnowledgeChunk rows and retrieve() ranks them with a hybrid of BM25 keyword + optional vector cosine (fused via Reciprocal Rank Fusion). But index_artifact is only called during brownfield onboarding - never on greenfield artifact registration/publish. So for a greenfield project retrieve() returns nothing, get_context's _retrieve_knowledge yields [], and agents rely solely on the required+situational artifact tiers. Separately, semantic search is globally OFF (EMBEDDING_PROVIDER=null) so even where chunks exist, only the keyword baseline runs and the pgvector column is empty.</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Knowledge Index / greenfield context retrieval</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verified 2026-07-23. index_artifact is called ONLY from backend/integrations/onboarding.py:400 (brownfield); no call on greenfield register/publish. Live backend env: EMBEDDING_PROVIDER=null (BM25-only; pgvector column unused). retrieve() (backend/apps/knowledge/index.py:106) already fuses BM25 + vector cosine via RRF and falls back to keyword if embeddings fail/are off. Providers built + ready: Voyage voyage-code-3 (dim 1024), Gemini gemini-embedding-001 (dim 1536); current column dim = 1536.</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">index_artifact was wired only into brownfield onboarding; greenfield artifact registration/publish never indexes. The embedding provider defaults to null (zero-cost baseline), so vectors are off platform-wide. Neither is a defect in the retrieval engine (which already does hybrid search) - it is unwired population + a disabled provider.</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED (enhancement + team decision on hybrid). (1) Populate greenfield: call index_artifact on artifact PUBLISH (gated), same path brownfield uses - publish-only (not every draft) to bound embedding cost. (2) Enable semantic search via a provider: Gemini gemini-embedding-001 (dim 1536) matches the current column so NO re-migration; Voyage voyage-code-3 (dim 1024, code-optimized) would need a column re-migration + re-embed. (3) KEEP the hybrid (team idea, already implemented): retrieve() fuses BM25 + vector via RRF so keyword covers exact identifiers, vectors cover meaning/synonyms, and it degrades gracefully to keyword-only if embeddings are off/fail. Pros of vector: semantic match, better on mature projects, fits agents' NL queries. Cons: per-chunk API cost+latency, external dependency/keys, dimension lock-in at migration, weaker on exact tokens, extra privacy egress. Net: enable greenfield population + turn on Gemini, keep both methods fused.</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="199" spans="1:1">

</xml_diff>

<commit_message>
Bugs sheet: log the connect-machine fake-token issue (S.No 198, P2, Open)
A QA member with a brand-new workspace and no project yet tried to connect the
companion and got a token that would not authenticate. The token was actually a
hardcoded placeholder the screen shows on failure, not a real one — so a failed
generation looked like a valid token. Logged with the root cause (no project to
enroll against + the frontend masking the real error) and the planned fix.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -10446,9 +10446,49 @@
         </is>
       </c>
     </row>
-    <row r="199" spans="1:1">
+    <row r="199" spans="1:10">
       <c r="A199" s="2">
         <v>198</v>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connect-machine token generation fails silently when the workspace has no project, and the UI shows a fake placeholder token instead of the real error. A new member (e.g. a QA tester) creates a workspace but has not created a project yet, opens "Connect your machine" and clicks "Generate enrollment token". The screen appears to produce a token and shows the companion serve command, but the token displayed is a hardcoded placeholder "rnr_3f9a…b2" (note the literal ellipsis) — not a real token — so the companion cannot authenticate. Reported by a QA member who ran: python -m runner.companion serve --api-url http://localhost:8000 --tenant ce135c3e-... --token rnr_3f9a…b2. A genuine token is a ~43-character secrets.token_urlsafe(32) string with no rnr_ prefix and no ellipsis, so what he copied was never a real (or partial) token — generation had actually failed and the failure was masked as a valid-looking token.</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connect Machine / companion enrollment (S-06)</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reported 2026-07-24 by a QA member on a newly-created workspace that had no project yet. Verified in code (no screenshot): the string "rnr_3f9a…b2" is a hardcoded mock placeholder, not a truncated real token.</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two layers. (1) The enroll endpoint requires a valid project: RunnerEnrollmentView.post (backend/api/runner_views.py:165-170) returns HTTP 400 ("project_id required" / "not found in tenant") when project_id is missing/invalid. (2) The Connect-machine screen picks the project from currentUser.memberships[0].project_id (frontend/src/features/identity/ConnectMachine.tsx:64); a brand-new workspace with no project has no membership, so project_id is empty and the POST 400s. The onGenerate catch block (ConnectMachine.tsx:68-70) swallows that error and calls setToken("rnr_3f9a…b2") — the same hardcoded placeholder used as the null fallback at line 61 — so a failed generation is rendered as a real-looking, copyable token instead of the backend's actual message. Net: there was no project to enroll the companion against, but the UI hid that behind a mock token. Same "fake mock data hides a real failure" pattern already fixed once on the invite-accept page (commit b77bdff).</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLANNED (not yet fixed). Immediate workaround: the member must create a project (and be a member of it) before generating the token — then the button returns a real ~43-char token and the serve command authenticates. Proper fix (frontend, ConnectMachine.tsx): on token-generate failure, surface the backend's real error message and do NOT fall back to a hardcoded token; guard the flow when the user has no project yet (show a clear "create a project first" prompt) instead of posting an empty project_id; and ensure the placeholder mock value can never be presented as a copyable token.</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="200" spans="1:1">

</xml_diff>

<commit_message>
Bugs sheet: record the Task Breakdown humanization completion (S.No 118)
The 2026-07-15 fix set the writing rule but left the technical examples, so
Tasks still read too technically. This records the follow-up that completed it
at the example level (worked Story/Task exemplars that lead with plain-language
intent, plus the manifest budget bump so long tasks reach the build agent).
The team re-ran Task Breakdown and confirmed the improvement, so S.No 118 stays
Fixed with the fuller detail. Siblings S.No 121-126 remain separately open.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -7719,8 +7719,11 @@
       <c r="G119" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I119" s="2" t="s">
-        <v>573</v>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED (2026-07-15). agents/06_task_breakdown/agent.md: added a 'Writing standard' requiring every Epic/Story/Task Description + Acceptance Criterion to be plain-language-with-technical-nuance, detailed and self-contained enough that a developer can implement by reading it ALONE (behaviour, inputs/outputs, states, edge cases), with concrete hand-verifiable acceptance criteria and no bare placeholders; modelled the standard in all three template placeholders. Improvement flows to the Work Items board + artifact previews automatically. Test: test_agents_migration.test_task_breakdown_descriptions_and_ac_are_humanized. Per team decision the blast radius today was 06 only; the SAME defect in 02/09/00c/04/03/10 is logged as S.No 121-126 (register-condition per audience: technical-humanized for testing/security, plain+nuance for the rest) and NOT fixed this session.
+FOLLOW-UP COMPLETION (2026-07-24, verified live by the team). The 2026-07-15 fix set the INSTRUCTION but left the technical exemplars in place, and the model imitates exemplars more than rules — so Epics read well (they already had good plain-language examples) but Tasks still came out too technical. Completed the fix at the EXAMPLE level: agents/06_task_breakdown/agent.md now carries worked Story AND Task exemplars that OPEN with a one-sentence plain-language statement of intent (what it delivers and why) BEFORE the technical detail, with concrete given/when/then acceptance criteria; added an explicit 'lead with plain-language intent' requirement for both Stories and Tasks; and rewrote the terse counter-examples (the endpoint-string title, the venv/env-file acceptance criteria) so nothing pulls the output back to terse. Platform side: backend/manifest/composer.py raised the Current Work Item token budget 300-&gt;650 so long task descriptions reach the implementation agent untruncated (avg 1,263 / max 1,835 chars already exceeded the old ~1,200-char cap). Strengthened the test to assert the intent-lead + the worked exemplars. Committed f27455d (pushed to develop). Team re-ran Task Breakdown on tenant 7828e953 and confirmed a great improvement vs the old artifacts. Scope decision this session was Tasks + Stories; siblings S.No 121-126 (agents 02/09/00c/04/03/10) remain separately Open.</t>
+        </is>
       </c>
       <c r="J119" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Bugs sheet: log the 09b test automation fixes from this session (S.No 199-205)
Logs the NUL/binary park bug, the remediation preview-target bug, the
generated-artifacts gitignore, the Test cases button, the headed browser
option, and two open items (phase gating, gitignore not untracking existing
files).
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -10494,39 +10494,319 @@
         </is>
       </c>
     </row>
-    <row r="200" spans="1:1">
+    <row r="200" spans="1:10">
       <c r="A200" s="2">
         <v>199</v>
       </c>
-    </row>
-    <row r="201" spans="1:1">
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09b test-automation run parks with a Postgres DataError ("unsupported Unicode escape sequence ... \u0000 cannot be converted to text") after the PR and artifacts have already been created, even when the generated test itself passed. Reproduced twice on the same test case (WI-95 / TC-001): runs 1299c7de and e583a454 both parked identically with the same corrupted bytes, though neither companion report itself contained a NUL.</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09b Test Automation / code review manifest</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reproduced 2026-07-22, tenant 212395b8-f118-4eef-93eb-ba2c45468226, WI-95 (TC-001), repo TARUN51/medslot-single-repo, PR #31. Confirmed via list_pr_files + get_file that tests/automated/playwright-report/data/*.webm and *.png contained NUL bytes.</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AgentReviewProvider._render_pr_section (backend/orchestration/review_provider.py:225-245) inlines the content of every PR-changed file into the review manifest, which dispatch_review_task then stores in the JSON run.inputs column. A 09b build commits Playwright report artifacts (screenshots/videos) into the PR; those binaries contain NUL, which Postgres text/jsonb cannot store, so the save fails with DataError and the workflow parks the run as "pr/gate setup failed" - after the PR/test_report/code artifacts already registered successfully. See S.No 201 for the fix that stops new binaries from being committed in the first place.</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. _render_pr_section now skips any file whose content contains a NUL byte (a binary marker) and inlines a "(binary file - omitted from review)" placeholder instead (review_provider.py:246-252). dispatch_review_task also scrubs NUL from the whole payload before saving, as defense-in-depth, via a shared build_types.scrub_nul helper; companion build reports are scrubbed the same way in build_report.py. Tests: test_render_pr_section_omits_binary_files, test_dispatch_review_task_scrubs_nul (test_review_dispatch.py), test_report_scrubs_nul_bytes_before_persisting (test_build_report_api.py).</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" spans="1:10">
       <c r="A201" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row r="202" spans="1:1">
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A 09b remediation build (auto-fixing a code-review finding) fails immediately with "no preview target for this repo - set the repo's Preview URL...", even though the repo's Preview URL was already set and the initial build had just run successfully against it.</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09b Test Automation / remediation loop</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reproduced 2026-07-22 on WI-95/TC-001 after the 08 review opened REM-W2/REM-W3; the run went straight to status=failed right after the build.remediation_dispatched event.</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dispatch_build_core (backend/orchestration/build_activities.py:62-81) ships payload['preview_url']/['preview_start'] for the test_automation phase, but dispatch_remediation_core (build_activities.py:781-826), which re-dispatches 09b to fix review findings, built its payload without that block - so the companion's remediation build had no preview target and its fail-loud guard tripped instantly. See S.No 199 for the review-manifest bug found on the same run.</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. dispatch_remediation_core now ships the same preview_url/preview_start (resolved via apps.projects.preview_config), phase-gated identically to the initial dispatch (build_activities.py:816-822). Test: test_dispatch_remediation_ships_preview_for_test_automation (test_review_dispatch.py).</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" spans="1:10">
       <c r="A202" s="2">
         <v>201</v>
       </c>
-    </row>
-    <row r="203" spans="1:1">
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The 09b test-automation agent commits its own generated run output (Playwright HTML report, test-results, MCP exploration snapshots) into the PR alongside the authored test script. These directories are bulky (one PR carried a 533KB report index.html plus screenshots and a video) and can contain binary files - the root cause of the review-manifest NUL crash at S.No 199. The 08 code review itself independently flagged this as a finding (REM-W1: "Generated Playwright artifacts... committed").</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09b Test Automation / generated worktree output</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed 2026-07-22, PR #31 (medslot-single-repo): tests/automated/playwright-report/, tests/automated/test-results/, and .playwright-mcp/ were all committed by the build.</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The 09b agent body had no instruction to ignore generated run/report output, so every file the dry run (Step 6) or Playwright MCP (Step 4) wrote into the worktree was committed by the platform, which commits everything present in the worktree.</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. Added a required ".gitignore" step to agents/09b_test_automation/agent.md Step 3 (Scaffolding Detection, line 123 on): the agent creates/extends a worktree-root .gitignore excluding .playwright-mcp/, playwright-report/, test-results/, blob-report/, and framework build/cache directories, while still committing the authored test scripts, page objects, and config. Note: does not retroactively untrack files a prior run already committed on the same branch - see S.No 205.</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" spans="1:10">
       <c r="A203" s="2">
         <v>202</v>
       </c>
-    </row>
-    <row r="204" spans="1:1">
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The "Test cases" coverage screen (per-story test-case list with automation status + Generate script) has no link anywhere in the UI - it is only reachable by typing its URL (/work-items/:id/test-cases) directly.</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test cases (P3-09b coverage screen)</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed 2026-07-22 while trying to generate a script for TC-001 on WI-70: the epic/story detail page had no way to navigate to its test cases.</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The coverage screen (frontend/src/features/lifecycle/TestCases.tsx) and its route were built, but the intended entry point (a tabbed story/epic detail) was deferred as a later enhancement, and no interim link was added in the meantime.</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. Added a "Test cases" button to the work-item detail header (frontend/src/features/lifecycle/WorkItemEpic.tsx:88-92), linking to /work-items/:id/test-cases. The tabbed story/epic detail remains a separately deferred enhancement.</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" spans="1:10">
       <c r="A204" s="2">
         <v>203</v>
       </c>
-    </row>
-    <row r="205" spans="1:1">
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The companion always runs the 09b Playwright MCP (and the generated test suite) headless, so a developer watching a run locally has no way to see the agent explore the app or the test execute, even while attended at the keyboard.</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Companion runner / 09b Live Application Exploration</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requested 2026-07-22, to observe a local 09b run end-to-end (locator discovery + test execution) for QA/demo purposes.</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">build_mcp_servers always passed --headless to the Playwright MCP (runner/companion/runner.py), and the agent's generated Playwright config had no signal telling it to run visibly instead.</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. Added SDLC_COMPANION_HEADED, read by _headed_enabled() (runner/companion/runner.py:112-117): drops --headless from the Playwright MCP, and manifest_with_preview injects an instruction so the agent generates "headless: !process.env.SDLC_COMPANION_HEADED" in playwright.config.ts, so the same config still runs headless in CI. Added "serve --headed" as a first-class flag (runner/companion/__main__.py:110-115) that sets the env var in-process, so no separate shell export is needed. Default remains headless.</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" spans="1:10">
       <c r="A205" s="2">
         <v>204</v>
       </c>
-    </row>
-    <row r="206" spans="1:1">
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Phases &amp; Runs, every catalog phase (Ideation .. Deployment) is shown as triggerable for ANY work-item type, including a test_case WI - a user can trigger "Ideation" or "Task Breakdown" on a test case, which is meaningless for that type and only 09b_test_automation should apply.</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phases &amp; Runs / phase catalog</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed 2026-07-22 while triggering 09b Test Automation on a test_case work item (WI-95): all ~16 phases appeared as trigger options, not just Test Automation.</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">There is no per-WI-type phase gating in the trigger UI or backend catalog - the phase picker (frontend/src/features/lifecycle/PhasesAndRuns.tsx) renders every catalog entry regardless of the selected work item's type.</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed - deferred. Would need the phase catalog (or the picker) to filter by work_item.type, e.g. only 09b_test_automation (and perhaps re-running 09_testing) for type=test_case.</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" spans="1:10">
       <c r="A206" s="2">
         <v>205</v>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A .gitignore added by the 09b agent (S.No 201) only stops NEW files from being committed going forward - it does not untrack files a prior run on the SAME branch already committed (e.g. Playwright report binaries from an earlier attempt). Resuming or remediating on an existing branch/PR can therefore keep re-triggering the code review's binary-artifact finding (REM-W1, S.No 199) even after the .gitignore fix ships.</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09b Test Automation / worktree branch reuse</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed 2026-07-22: re-running 09b on the same branch/PR (#31) after adding the .gitignore rule still showed the previously-committed playwright-report binaries until the branch was closed and recreated from scratch.</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Git's .gitignore only governs untracked files from that point forward; files already added to the index/history stay tracked. The platform reuses the existing branch/worktree for a resumed or re-triggered build (register-don't-recreate), so old committed binaries persist across runs.</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed - workaround documented: close the PR, delete the remote branch, and let 09b start a fresh branch so the new .gitignore takes effect from the first commit. A platform-side fix (e.g. "git rm --cached" the newly-ignored paths on resume) is not implemented.</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="207" spans="1:1">

</xml_diff>

<commit_message>
Bugs sheet: log this session's fixes and open enhancements (S.No 206-210)
Null-enrollment unclaimable run, empty-build-on-retry, and the S.No 161
auto-retry UI-visibility gap are all fixed. Companion silent-death
alerting and the cross-WI method-signature collision are left open as
enhancements.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -10809,29 +10809,229 @@
         </is>
       </c>
     </row>
-    <row r="207" spans="1:1">
+    <row r="207" spans="1:10">
       <c r="A207" s="2">
         <v>206</v>
       </c>
-    </row>
-    <row r="208" spans="1:1">
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A build (or phase) Run dispatched with inputs.dispatch.enrollment_id=null matched no companion in the claim query, so it sat running+pending forever, invisible in the UI, and blocked new triggers on the same WorkItem.</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Runner dispatch / claim (RunnerWorkClaimView)</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surfaced 2026-07-21, tenant 212395b8-f118-4eef-93eb-ba2c45468226. Two paths hit it: the S.No 161 remediation auto-retry called trigger_build without triggered_by, and a user triggering before their companion enrolled. Validated live: run 812577a3 self-healed after the fix.</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RunnerWorkClaimView's claim query only matched Run.inputs.dispatch.enrollment_id == runner.id - a dispatch created with enrollment_id=null (no companion known yet) matched nothing, so no companion could ever claim it.</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. backend/api/runner_views.py: the claim query now also broadcast-matches any pending/claimed dispatch with enrollment_id null/empty for the same tenant+project, and binds enrollment_id to the claiming companion. backend/orchestration/build_activities.py: handle_remediation_exhausted_core now forwards triggered_by into the retry's trigger_build call so retries route to the original companion instead of null. Tests added in test_phase_dispatch.py, test_build_activities.py.</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" spans="1:10">
       <c r="A208" s="2">
         <v>207</v>
       </c>
-    </row>
-    <row r="209" spans="1:1">
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clicking Retry run on a build whose feature branch a prior attempt had already pushed failed with "Empty build: the agent produced no changes to commit", even though real work already existed on the branch.</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Companion build retry / worktree (runner/companion)</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surfaced 2026-07-21 on WI-45's retry after a companion redeploy. Validated live on WI-f717ea04 (merged) after the fix; also validated with a standalone host git script reproducing the exact retry scenario.</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S.No 162's branch-continuity provisions the retry worktree from the branch's remote tip, not local/base. If the agent makes no new local commit on retry (the real work is already on the pushed branch), run_build left head_sha empty, and the empty-build guard failed the run even though the branch has real commits ahead of base.</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. runner/companion/worktree.py adds commits_ahead_of_base(). runner/companion/runner.py's run_build now reports the existing branch tip as head_sha when there's no new local commit but the branch is already ahead of base, so the saga opens/continues the PR against the existing work instead of false-failing. Tests added in test_companion_runner.py.</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" spans="1:10">
       <c r="A209" s="2">
         <v>208</v>
       </c>
-    </row>
-    <row r="210" spans="1:1">
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-up to S.No 161: when remediation exhausts an attempt and the platform auto-starts a fresh run, the user got no proactive signal - the failed run's console showed 'auto-retrying' text but no link to the new run, so a WorkItem appeared to show a failed run AND a separate pending gate with nothing connecting them.</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run console / lifecycle (RunConsole.tsx)</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed this confused a user reviewing WI-43's gate. Backend already stored retry_run_id on the failed run's outputs (build_activities.py); zero frontend references to it before this fix.</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The notification bell only counts pending gates + clarifications (AppShell.tsx bellCount), and the failed-run view never rendered the stored outputs.retry_run_id, so the two runs for the same WorkItem appeared unrelated.</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed. frontend/src/features/lifecycle/RunConsole.tsx: the failed view now reads outputs.retry_run_id, shows an info banner ("The platform started a fresh attempt...") with a live status link to the retry run, and swaps the primary action to "Go to the retry run -&gt;" when one exists. Shipped as PR #7, merged to develop (aafd1f9).</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" spans="1:10">
       <c r="A210" s="2">
         <v>209</v>
       </c>
-    </row>
-    <row r="211" spans="1:1">
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When a companion dies/hangs mid-build (e.g. crashes during a remediation cycle), the claimed run just sits running with no user-facing signal until the orchestrator's takeover reconciler eventually fires and fails it - the user has no way to know earlier that their companion needs restarting.</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Runner heartbeat / takeover reconciler</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed 2026-07-22 on WI-59 (run 925e7fde): companion 4a34ecf2's last heartbeat was 06:50:55 UTC; the run sat claimed/running with zero new events until "Build takeover - runner offline / no report before timeout" finally fired and failed it, well over an hour later. Retriggering after restarting the companion completed the build successfully.</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The takeover timeout is the only mechanism that reconciles a dead companion's claim; there is no earlier heartbeat-staleness check that surfaces a warning to the user while the run is still nominally in-flight.</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed. Suggested: surface a "companion appears offline" warning on the run console (and/or the companion status pill) once RunnerEnrollment.last_seen exceeds the ONLINE_THRESHOLD for a run that is still claimed/running, instead of waiting for the full takeover window.</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" spans="1:10">
       <c r="A211" s="2">
         <v>210</v>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two independently-dispatched work items (TASK-021 ExpenseRepository CRUD and TASK-033 DashboardService) each implemented get_monthly_total/get_category_breakdown/get_recent on the same repository class, with different return contracts (plain tuples vs a CategoryTotal dataclass) - since neither WI's planning had visibility into the other's in-flight interface, it only surfaced as an add/add merge conflict when both branches reached main.</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work-item decomposition / planning - parallel WI interface overlap</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enhancement</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surfaced 2026-07-22 resolving WI-59's merge gate conflict against main (already carrying WI-35's merged CRUD repository). Resolved by keeping main's superset repository and adapting DashboardService/tests to the CategoryTotal contract; validated with the full backend suite (412 passed).</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planning dispatches WIs against the same file/class independently when their scopes overlap (both needed the same three read methods), with no shared interface contract or ownership check between them before they diverge in the codebase - the S.No 137 recon closed a similar-looking report as a false alarm, but this is a real, reproduced instance of the same class of problem.</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed generally (this instance resolved manually). Suggested: when planning dispatches multiple WIs that touch the same file/module, either serialize them or require an explicit shared interface note so the return contract is agreed before either branch is built.</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
       </c>
     </row>
     <row r="212" spans="1:1">

</xml_diff>

<commit_message>
Log the remediation loop bug as S.No 241
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -4968,7 +4968,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J241"/>
+  <dimension ref="A1:J242"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -12184,6 +12184,56 @@
         </is>
       </c>
     </row>
+    <row r="242" spans="1:10" ht="232.5" x14ac:dyDescent="0.35">
+      <c r="A242" s="2">
+        <v>241</v>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code review remediation loop can never finish - the build agent is briefed with a finding the reviewer is no longer raising</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TASK-029 (Apply Leave form) ran for 26 hours across two runs, 20 review cycles and 15 remediation rebuilds without ever clearing review. The QA member resumed it four times; each resume granted a fresh cycle budget and hit the same wall. The reviewer was blocking on one thing (the duration-preview endpoint accepts reversed date ranges) while the implementation agent was repeatedly asked to fix a different thing it had already fixed 15 cycles earlier (a COMPOFF_EXPIRED message in a frontend file). The loop could not converge by construction, not by chance.</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build pipeline / code review remediation loop (run_code_review_core, dispatch_remediation_core, review manifest)</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tenant 9dd11483 (QA, PeopleDesk) WI-87 TASK-029, runs 4e62a433 (failed, 4 cycles) and b80802ac (stalled, 16 cycles), 2026-08-26 to 2026-08-27. Same signature on every other remediation-exhausted run in the tenant: WI-55, 57, 65, 67, 72, 86 - 8 of 8, against 0 of the 24 runs that converged normally in 2-3 cycles.</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A rem id (REM-W1, REM-C1) is a POSITION in one review's output, not an identity: the reviewer numbers its findings from 1 on every re-review, and the review manifest never carried the previous cycle's ids, so the agent had nothing to reuse even though agents/08_code_review/agent.md line 274 instructs it to. Three defects then compound. (1) REM-W1 silently comes to mean a different problem the moment the finding set changes shape. (2) run_code_review_core only ever wrote a remediation child WorkItem at creation - the reopen branch flipped state and nothing else, so title, description, file and line stayed frozen at cycle 1 forever, and dispatch_remediation_core briefs agent 07 from exactly those fields. (3) The children hang off the WorkItem, not the run, so the auto-retry run inherited the failed attempt's board and was mis-briefed on its very first cycle. Evidence on WI-87: the board was written 9 times, all inside the first 20 minutes; 14 of the 15 remediation builds ran after it stopped changing; and the file the reviewer was blocking on was last touched by the INITIAL build and by none of the 15 remediation builds. The one-line fix the reviewer wanted (previewWorkingDays never calls the validateDateRange that already sits directly above it) was never attempted.</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed 2026-08-27 on develop (commit e7e791e). (1) run_code_review_core now rewrites the child's title, description, severity, file and line from the CURRENT finding every cycle instead of only flipping state, and logs remediation.retargeted when the meaning under an id really changes, so the collision is visible instead of hidden behind a count. (2) The review manifest gained a 'Findings Already Open From Your Previous Review' section listing live rem ids with file:line, so the reviewer can honour the reuse-or-omit contract its own body states; absent on cycle 1 and degrades to nothing on any error, since a missing section must never fail a review. (3) handle_remediation_exhausted_core closes the open remediation board before starting a retry attempt - closed, never deleted, and prior_attempt_context already carries the substance forward to the new agent. 5 new tests in test_build_activities.py and test_review_dispatch.py, 4 of them verified failing against the unfixed source. No data repair needed: TASK-029 self-corrects on its next review cycle after the QA member pulls, restarts the worker and clicks Resume.</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J239" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">

</xml_diff>

<commit_message>
Log the worker hand-over gap as S.No 242
A worker that is being replaced waits until it has nothing in hand before
it leaves. It judges that by whether a step is running right now, but a
build spends nearly all its time waiting on the developer's companion
with nothing running at all, so the outgoing worker calls itself finished
after five minutes and shuts down while the build is still live. The
build is tied to that worker, so it then waits for a worker that is no
longer there and shows as queued with nothing visibly wrong.

Not seen in the wild yet, and it needs a second worker on different code
to start mid-build. Logged as Open with the stopgap noted: the wait is
already configurable, so setting it longer than a build avoids it without
any code change.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -4968,7 +4968,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J242"/>
+  <dimension ref="A1:J243"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -12234,6 +12234,56 @@
         </is>
       </c>
     </row>
+    <row r="243" spans="1:10" ht="232.5" x14ac:dyDescent="0.35">
+      <c r="A243" s="2">
+        <v>242</v>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A worker handing over to a newer build can quit while a build is still running, stranding it with no error</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The worker hand-over is meant to let an outgoing worker finish what it holds before it leaves. It decides whether it is still holding something by asking whether a step is executing right now - but for nearly all of a build the worker is doing nothing, waiting for the developer's companion to write the code and report back. After five minutes of that wait it concludes it is finished and shuts down. The build is stamped with that worker's build id, so when the companion finally reports there is no worker that matches and the run stops dead showing 'Queued' with a healthy companion and a healthy worker. Same symptom as the unversioned-worker fence found the same day, different cause - which is exactly what makes it expensive to diagnose the second time.</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporal worker hand-over (orchestration/worker_election.drain_when_superseded)</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-08-28 by reading the code while fixing the queued-build incident on tenant 9dd11483 (QA, PeopleDesk) TASK-030. NOT yet observed in the wild. Confirmed against the live server that the premise holds: workflow build-run-9da5a94d carries worker stamp build_id=20260828T073458Z-83c57f55a83d with use_versioning=True, so a versioned worker does tie the execution to its own build, while TASK-029 (served unversioned) carries no such tie. The hand-over code reached develop the same day in eda970d + 9347e13.</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drain_when_superseded declares itself drained when TrackingExecutor reports in_flight == 0 and idle &gt;= WORKER_DRAIN_IDLE_SECONDS (default 300s). TrackingExecutor is the ACTIVITY executor, so it counts only activities that are executing. A build spends nearly all of its life inside workflow.wait_condition waiting for the companion's build report, with no activity in flight for 20-90 minutes, so a worker minding a perfectly live build reports itself idle within five minutes of that wait starting. Idleness is therefore the wrong signal: it measures 'am I busy this second', not 'is any build still tied to me'. Once the worker exits, the workflow task scheduled by the companion's report has no matching poller and the run stalls with no error anywhere - the same dead end as a fenced-out worker.</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed. Stopgap with NO code change: set WORKER_DRAIN_IDLE_SECONDS longer than a build (e.g. 7200), so a superseded worker lingers long enough to see its builds through; WORKER_DRAIN_MAX_SECONDS (default 86400) still caps it. Proper fix: drain on whether any workflow is still assigned to this build rather than on activity idleness. Note get_worker_task_reachability cannot be used for that signal - it reports a non-default build as still NEW_WORKFLOWS reachable. Scope: only bites when a second worker running DIFFERENT code starts mid-build on a shared queue; a task queue per stack (as the brownfield stack already does with sdlc-brown) removes the race entirely, so this row is moot if the team splits the queues.</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J239" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">

</xml_diff>

<commit_message>
Log the missed CORS requirement as S.No 243
TASK-006 asked the build agent for four things in one sentence. It delivered
three and dropped "Configure CORS to allow the FRONTEND_URL env var origin with
credentials". The review agent passed it, the gate was approved, and the task is
marked done. Nobody noticed for 18 days because no test in the pipeline opens a
browser, and CORS is only enforced by a browser.

The product fix goes back through the platform as TASK-050 in the QA tenant. The
platform finding stays open: the review agent is never shown the work item's
acceptance criteria, so it cannot notice one that was never delivered.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -4968,7 +4968,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J243"/>
+  <dimension ref="A1:J244"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -12284,6 +12284,56 @@
         </is>
       </c>
     </row>
+    <row r="244" spans="1:10" ht="232.5" x14ac:dyDescent="0.35">
+      <c r="A244" s="2">
+        <v>243</v>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An explicit acceptance criterion was dropped by the build agent and passed by the review agent - the API has no CORS, so no browser can reach it</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TASK-006's description told the implementation agent, in one sentence carrying four requirements, to "Configure CORS to allow the FRONTEND_URL env var origin with credentials". The ValidationPipe with all three flags, Swagger at /api/docs and the health endpoint - the other three requirements in that same sentence - were all delivered. CORS was not. The review agent passed the PR, the merge gate was approved, and TASK-006 is marked done and merged as PR #11 on 2026-08-13. The miss stayed invisible for 18 days and 29 further tasks because nothing in the pipeline ever opens a browser. It surfaced only when a QA member tried to open the product for the first time: the SPA is on :5173, the API on :3000, and every request including the login POST dies at the browser preflight.</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agent quality / implementation + code review acceptance-criteria coverage (PeopleDesk TASK-006)</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tenant 9dd11483 (QA, PeopleDesk) TASK-006 = WI-64, PR edvensoft/PeopleDesk#11 merged 2026-08-13. The same requirement is also stated in FOUND-003 = WI-56 (PR #3) and was missed there too. Verified 2026-09-01 by reading packages/backend/src/main.ts at origin/main via the platform's codehost capability: no enableCors call present. Surfaced as finding B1 of the QA readiness review dated 2026-08-31.</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two gaps in sequence. (1) The build agent completed three of four requirements in a single run-on sentence and silently dropped the fourth; nothing checks a delivered PR back against the individual clauses of its acceptance criteria, so a partial delivery reads as a complete one. (2) The review agent inspects the diff for defects in what was written, not for what the work item asked for and is absent - a call that was never made has no line to flag. Neither the agent's tests nor CI could catch it: CORS is enforced by the browser, and every test in the pipeline calls the API in-process via supertest, where no preflight ever occurs. The requirement was stated twice (FOUND-003 and TASK-006) and missed both times, so this is a systematic gap, not a one-off slip.</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed. The PRODUCT fix is routed through the platform itself as TASK-050 (WI-212) under WI-56/FOUND-003 in tenant 9dd11483 - one enableCors({ origin: FRONTEND_URL, credentials: true }) call in packages/backend/src/main.ts plus preflight e2e tests - deliberately built, reviewed and merged by the normal build loop rather than hand-patched, so the fix is itself a test of the pipeline. The PLATFORM finding is the open item: the code review agent is never given the work item's acceptance criteria to verify delivery against. Candidate fix - include the work item's acceptance criteria verbatim in the 08_code_review manifest and require an explicit per-criterion verdict before a review may report zero blocking findings.</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J239" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">

</xml_diff>

<commit_message>
Log the stranded-build bug as S.No 244
TASK-036 sat on "dispatched for review" for 31 hours with nothing reporting an
error. The worker was healthy and polling the whole time. The job had been
stamped with the worker's code version when it started, the worker later
restarted on newer code, and Temporal treats the two versions as unrelated - so
there was no longer any worker allowed to pick that job up.

The version stamping was added in August to stop a worker running old code from
stealing jobs. It works, but because our version changes on every code change
and a build runs for hours, any pull during a build now strands that build.
Nothing raises an error when this happens, which is why it has cost us three
investigations.

Recovery for TASK-036 is done. The underlying fix is not - the options are
written into the row.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -4968,7 +4968,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J244"/>
+  <dimension ref="A1:J245"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -12334,6 +12334,56 @@
         </is>
       </c>
     </row>
+    <row r="245" spans="1:10" ht="232.5" x14ac:dyDescent="0.35">
+      <c r="A245" s="2">
+        <v>244</v>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A worker restart on changed code silently orphans every build still running - the job stays addressed to a code version that no longer exists</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TASK-036 showed 'dispatched for review' for 31 hours with no error anywhere. The workflow reported Running, the worker reported healthy and was polling the same queue seconds before it was checked, the queue reported healthy, and the UI showed a normal state. Nothing was wrong with the agent, the review or the shared server: the review agent had in fact reported back four separate times. The job was simply addressed to a worker build that no longer existed, and no part of the platform notices that. Recovering it required terminating the workflow by hand, because a restart cannot help - each restart mints yet another version, no closer to the one the job is waiting for.</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporal worker build-ID versioning (orchestration/worker_election.elect)</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tenant 9dd11483 (QA, PeopleDesk) TASK-036 = WI-93, run 7ebe493a, workflow build-run-7ebe493a-c054-4e99-adfb-fefd312176d6, PR edvensoft/PeopleDesk#43. Build started 2026-09-01 10:02 UTC on build 20260901T075033Z-a2228a4ad85e; worker restarted 2026-09-02 07:53 UTC as 20260902T075326Z-5ceff9d45ff3; workflow task pending and unstarted from 2026-09-02 02:00:18 UTC until terminated 2026-09-03 09:18 UTC. Queue sdlc-planning then carried 6 registered version sets and 8 running workflows, ALL 8 stranded on retired builds (7 were pre-existing orphans up to 42 days old, never noticed). Same family as S.No 242 and the 2026-08-28 TASK-030 fence, different mechanism.</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">worker_election.elect registers each worker's badge with BuildIdOpAddNewDefault, which makes every badge a NEW INCOMPATIBLE version set rather than a successor of the previous one. The badge is derived from the newest source file mtime plus a code fingerprint, so any git pull or edit produces a new badge and therefore a new incompatible generation. Temporal deliberately pins a running workflow to the build it started on for its whole life, so that it cannot have code change underneath it. Those two behaviours are individually correct and jointly fatal: our version changes on every code change while a build lasts hours, so any restart during a build leaves that build addressed to a generation nobody serves - permanently, and with no error, no failed state and no alert. The versioning was added on 2026-08-26 to fence out a stale worker running old code; the cure now strands the work it was protecting.</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not fixed. Recovery for this instance (2026-09-03): terminated the one workflow by exact id, closed run 7ebe493a via mark_build_failed_core so the work item was no longer blocked by an active run, and re-triggered TASK-036 - the branch feature/WI-35b48096 and PR #43 were untouched, and the new run continues from the remote tip, so only the last review cycle repeats. Candidate fixes, in preference order: (1) one task queue per stack, which sdlc-brown already does and which removes the contest entirely; (2) register each new badge as COMPATIBLE with the previous one (BuildIdOpAddNewCompatible) so a newer worker may serve older in-flight workflows, accepting that this reintroduces some stale-worker risk; (3) at minimum, detect and surface the condition - compare each running workflow's stamped build against the live pollers and raise it in the UI, because today the only symptom is silence. NOTE a separate open sub-question on the same run: the run_code_review activity never once completed its 30-minute wait across three attempts while the companion reported four times, so the worker was not staying alive through the wait; cause not determined from server-side data and needs the worker/companion log from the QA member's machine.</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J239" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">

</xml_diff>

<commit_message>
Log the two issues found while testing the board and a test case
S.No 268: a test case's detail page said "No description yet" for every
case the Testing phase created, because the steps live in the artifact
and nothing on the page followed the pointer.

S.No 269: the Work Items board's horizontal scrollbar sat below the
fold, because the columns grew without limit and the scrollbar belongs
to the bottom of the container.

Both were fixed in a68be43. The rows record what was seen, why it
happened and what changed.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -5159,7 +5159,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J268"/>
+  <dimension ref="A1:J270"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -14021,8 +14021,112 @@
         </is>
       </c>
     </row>
+    <row r="269" spans="1:10">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">268</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A test case's detail page says "No description yet" for every case the Testing phase created - the steps are never shown anywhere on the work item</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-09-20 on SpendLog WI-99 (TC-005 - User Login Happy Path), and true of all 42 auto-created cases on that project. The detail page renders `workItem.description`, which `materialize_test_cases` never writes: it copies the title and an `external_ref` pointer to the `test_case` artifact and nothing else. So the steps, preconditions and test data the user needs to read BEFORE triggering Test Automation are not on the screen at all. Cases added BY HAND look fine, because that form writes its steps straight into the description - so the same screen tells the truth for one kind of test case and not the other, which is what made it read as a rendering bug rather than missing data.</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work item detail - test cases (frontend WorkItemTask.tsx; backend apps/workitems/test_cases.materialize_test_cases writes the pointer only)</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WI-99 / WI-95 / WI-98 on project SpendLog (tenant 212395b8); frontend/src/features/lifecycle/WorkItemTask.tsx Description panel</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The test case's content lives in the `test_case` artifact, not on the work item, and nothing on the detail page ever followed the pointer. The page had one Description panel, bound to a field that is empty by design for this type.</t>
+        </is>
+      </c>
+      <c r="I269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed 2026-09-20 (a68be43). A `Test case` panel replaces the Description panel for `test_case` items that carry `external_ref.test_case_artifact_id`, reading the body through the existing artifact preview endpoint and linking to the artifact. Deliberately a POINTER, not a copy (#1/#3): the artifact stays the source of truth, the page cannot drift when Testing re-runs, and what the user reads is exactly what 09b reads when it writes the script - which is the reason to look at it. Test cases only; every other type keeps the ordinary Description panel, a hand-added case (which carries its own steps) keeps it too, and an artifact that cannot be read says so instead of rendering blank. Mockups were presented and the option chosen before any code was written (non-negotiable #11). Tests: 4 new in frontend testCasePanel.test.tsx; full FE suite 641 pass, tsc + eslint clean.</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" spans="1:10">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">269</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Work Items board's horizontal scrollbar sits below the fold - you must scroll to the bottom of the page to move sideways between phase columns</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-09-20 on SpendLog, whose Backlog column holds 122 cards. The board is the horizontal scroll container, but its columns grow without limit, so the element becomes thousands of pixels tall and its scrollbar sits at the very bottom of all that - far below the window. Reaching the later lifecycle columns meant scrolling the whole page down past every card first, and the column headings scrolled away on the journey. Related but distinct from S.No 166 (a dropdown clipped by its container's overflow, not a scrollbar out of reach).</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work Items board (frontend styles/components.css .board, WorkItemsBoard.tsx)</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">frontend/src/styles/components.css `.board { overflow-x: auto }` with `.board__list` having no height cap; SpendLog board, Backlog column 122 cards</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`.board` owned the horizontal overflow while `.board__list` had no maximum height, so the scroll container's own height was the height of its longest column. A scrollbar belongs to the bottom of its container, and the container had no reason to stay inside the window.</t>
+        </is>
+      </c>
+      <c r="I270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed 2026-09-20 (a68be43). The board view now fills what is left of the window below the topbar and scrolls INSIDE itself: each column caps at that height and scrolls its own cards, the column heading stays put while they do, and the horizontal scrollbar is always on screen. Scoped to the board with a `canvas-pad--board` modifier so the list and empty views scroll the page exactly as before; columns stay content-sized, so a short column is not a tall empty box. Mockups were presented and the option chosen first (non-negotiable #11). Verified in a browser against the real stylesheets with a 122-card column at 1280x800: page no longer scrolls vertically, board bottom inside the viewport, board scrolls horizontally, long column scrolls on its own, heading visible. Full FE suite 641 pass. NOTE still open as a usability matter, not a defect: 122 cards in one column is a lot to scroll even now - a per-column 'show more' cap was raised and deliberately left out of scope.</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J268" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:J270" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">
       <filters blank="1">
         <filter val="Open"/>

</xml_diff>

<commit_message>
Stop long work item titles flickering when you hover them in the picker
The box that shows a cut-off title in full sat on top of its row and caught the mouse,
so it closed and reopened on every movement. It now lets the mouse through to the row,
so it stays still and a click picks the row. This also fixes the run history filters.
Logged as Bugs S.No 282, with a QA row.
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -5159,7 +5159,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J282"/>
+  <dimension ref="A1:J283"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -14749,8 +14749,60 @@
         </is>
       </c>
     </row>
+    <row r="283" spans="1:10">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">282</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work item picker: hovering a long title makes it flicker instead of showing it</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On Phases &amp; Runs, hovering a work item whose title is cut off in the dropdown made the full-title box flash on and off with every mouse movement; a click could land on the box and pick nothing. The same happened on the closed field and on the two searchable pickers in the run history filters.</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phases &amp; Runs - work item picker; run history filters (frontend components/ui Combobox / TruncationPeek, styles/components.css)</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reported by the team 2026-09-21 (screenshot). Introduced by b40c557 (12 Sep, the full-title peek). Option A chosen.</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The full-title box is drawn over the row but took the mouse itself: the list saw the mouse leave and closed it, the row saw the mouse again and reopened it - a loop on every movement.</t>
+        </is>
+      </c>
+      <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed 2026-09-21 (Option A). The box lets the mouse pass through to the row (pointer-events: none), so it sits still and a click picks the row under it. Looks exactly as approved on 12 Sep. A test pins the rule. Awaiting QA live pass.</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J282" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:J283" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">
       <filters blank="1">
         <filter val="Open"/>

</xml_diff>

<commit_message>
Record the accessibility fixes in Bugs and QA, and drop the retitling migration
- Bugs.xlsx rows 371-389: every accessibility fix from the 10 Oct recon and live audit
- New QA suite TS-16 (TC-954 to TC-966) for the audit, review queue, statement, signing and export
- Removed the migration that retitled older defects: the demo always starts from a fresh
  workspace, so only new defects need the new titles
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -5159,7 +5159,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J371"/>
+  <dimension ref="A1:J390"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -19396,8 +19396,996 @@
         </is>
       </c>
     </row>
+    <row r="372" spans="1:10">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">371</t>
+        </is>
+      </c>
+      <c r="B372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An accessibility check whose agent stopped early waited forever instead of failing</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If the AI judge or keyboard-journey agent stopped part-way, the run was parked as 'waiting' and the audit never finished or failed.</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - audit and journeys</t>
+        </is>
+      </c>
+      <c r="E372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility runs were treated like ordinary phases, which are parked for a retry when the engine stops; nothing ever resumed them.</t>
+        </is>
+      </c>
+      <c r="I372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Accessibility runs now fail when the engine stops, which closes their unfinished journey or AI pass so the screen says what happened. Covered by automated tests; the live engine-stop test is part of the greenfield pass after the demo.</t>
+        </is>
+      </c>
+      <c r="J372" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="373" spans="1:10">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">372</t>
+        </is>
+      </c>
+      <c r="B373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The keyboard-journey address could be pre-filled from an audit that failed</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The suggested address came from the latest audit whatever its outcome, so a failed audit's wrong address was offered again.</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - keyboard journeys</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The suggestion did not filter on the audit's outcome.</t>
+        </is>
+      </c>
+      <c r="I373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Only a completed audit's address is suggested.</t>
+        </is>
+      </c>
+      <c r="J373" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" spans="1:10">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">373</t>
+        </is>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The activity log said nothing when an accessibility audit started or finished</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An audit could run, fail or be abandoned with no entry in the activity log.</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Pages &amp; audit</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Audit status changes were saved without writing an event.</t>
+        </is>
+      </c>
+      <c r="I374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). 'Audit started', 'finished', 'failed' and 'abandoned' entries are written, naming the pages. Seen live: 'audit started' listed all 5 pages.</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" spans="1:10">
+      <c r="A375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">374</t>
+        </is>
+      </c>
+      <c r="B375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The activity log said the baseline was 'published' while it was still a draft</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The log entry read 'baseline published' at audit time, but the document stays Draft until the statement is signed.</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Pages &amp; audit</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The event name predates the rule that signing publishes the evidence.</t>
+        </is>
+      </c>
+      <c r="I375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Renamed to 'baseline recorded'. Seen live.</t>
+        </is>
+      </c>
+      <c r="J375" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" spans="1:10">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">375</t>
+        </is>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility defect titles showed element ids and page paths</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Titles read like '... on /loans/current - #main' instead of naming the page and the part of it.</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work items - accessibility defects</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The title was built from the scanner's selector and route path.</t>
+        </is>
+      </c>
+      <c r="I376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Titles name the page and the part in words, e.g. 'Reflow (1.4.10) on the Opening hours page - main content', 'Use of Color (1.4.1) on the Current loans page - row 3 in the loans table'. An element with no wording of its own falls back to its name in quotes (approved). Applies to defects filed from now on; older defects keep their old titles (team decision 2026-10-10: the demo always uses a fresh workspace, so no retitling migration). Seen live on 10 new defects.</t>
+        </is>
+      </c>
+      <c r="J376" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" spans="1:10">
+      <c r="A377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">376</t>
+        </is>
+      </c>
+      <c r="B377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Audits were named by an id number</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The statement and documents said 'audit 48506881' - meaningless to a reader.</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The audit's label was its id.</t>
+        </is>
+      </c>
+      <c r="I377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Named by when it ran: 'the audit of 10 Oct 2026, 6:12 PM'; a second audit the same day says so. The id is kept on the signing record only. Seen live (judging document and statement).</t>
+        </is>
+      </c>
+      <c r="J377" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" spans="1:10">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">377</t>
+        </is>
+      </c>
+      <c r="B378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Undecided criteria gave no reason why a person had to decide</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows marked 'needs your decision' did not say why the checks could not settle them.</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The reason existed only in the code's logic, never on the row.</t>
+        </is>
+      </c>
+      <c r="I378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Each such row says why, e.g. 'Only a person can judge this criterion - no check can observe it. Choose a level.' Seen live.</t>
+        </is>
+      </c>
+      <c r="J378" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" spans="1:10">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">378</t>
+        </is>
+      </c>
+      <c r="B379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The conformance numbers looked final while an audit was still running, and it could be signed then</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mid-audit the tiles showed partial counts with nothing saying they were still coming in, and Sign stayed open.</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The statement screen did not know an audit was in progress.</t>
+        </is>
+      </c>
+      <c r="I379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). A banner says an audit is running, the first tile reads 'Checked so far', and Sign waits ('Sign opens when the audit finishes.'). The server refuses a signature during an audit too.</t>
+        </is>
+      </c>
+      <c r="J379" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="380" spans="1:10">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">379</t>
+        </is>
+      </c>
+      <c r="B380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A statement could be signed when nothing had been checked</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">With no audit at all, the statement could still be signed - a signature resting on no evidence.</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Signing only required the acknowledgement, not any evidence.</t>
+        </is>
+      </c>
+      <c r="I380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). With nothing checked the panel says 'Run an audit first' and the server refuses to sign.</t>
+        </is>
+      </c>
+      <c r="J380" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="381" spans="1:10">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">380</t>
+        </is>
+      </c>
+      <c r="B381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Signing the statement left the accessibility report and baseline as Draft</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After signing, both documents still read Draft in Artifacts (team: Draft is fine as the label before signing, but signing must publish them).</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nothing moved the evidence documents on when the statement was signed.</t>
+        </is>
+      </c>
+      <c r="I381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Signing publishes the report and baseline and records which audit it rests on and what it published. Seen live 10 Oct 18:51: both turned Published; the AI judging notes stay 'Run output'.</t>
+        </is>
+      </c>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="382" spans="1:10">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">381</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two different 'waiting' numbers looked like a contradiction</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Audit tab said 'Waiting on a person 0' while the Conformance tab said 'Waiting on you 5'. Both were right - elements versus criteria - but read as a clash.</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Audit and Conformance tabs</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two counts of different things shared nearly the same words.</t>
+        </is>
+      </c>
+      <c r="I382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Audit tab: 'Items to review' with a link 'in the Review queue'. Conformance tab: 'Criteria to decide', plus 'Not settled yet' for the unknowns. Seen live.</t>
+        </is>
+      </c>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="383" spans="1:10">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">382</t>
+        </is>
+      </c>
+      <c r="B383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The audit header showed the start time beside the word 'complete'</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Audit complete' was followed by when it started, while the statement showed when it finished - two unlabelled times for one audit.</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Pages &amp; audit</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The header used the audit's creation time.</t>
+        </is>
+      </c>
+      <c r="I383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). 'Audit complete - finished 10 Oct 2026, 6:26 PM' with 'started 6:12 PM' under it. Seen live.</t>
+        </is>
+      </c>
+      <c r="J383" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="384" spans="1:10">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">383</t>
+        </is>
+      </c>
+      <c r="B384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Audit screen wording: 'pages each', 'Would not open', 'route(s) registered'</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machine-like or unclear words on the Pages &amp; audit tab.</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Pages &amp; audit</t>
+        </is>
+      </c>
+      <c r="E384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wording carried over from the internals.</t>
+        </is>
+      </c>
+      <c r="I384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). 'up to 60 pages per pass', 'Pages that didn't load', '5 pages listed' / '1 excluded'. Seen live.</t>
+        </is>
+      </c>
+      <c r="J384" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="385" spans="1:10">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">384</t>
+        </is>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A defect's state on its own page read differently from the board</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The defect page showed a stored state word while the board showed 'Not started'.</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work items - defect page</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The two screens used different labels for the same state.</t>
+        </is>
+      </c>
+      <c r="I385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Both use the board's label.</t>
+        </is>
+      </c>
+      <c r="J385" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" spans="1:10">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">385</t>
+        </is>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Export on the conformance statement said 'Preparing...' and then did nothing</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After signing, pressing Export flashed 'Preparing...' and nothing followed; the statement stayed Approved.</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="H386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The button only asked the server whether export was allowed and ignored the answer. Following that answer would have opened the generic publish screen set to Xray (statements are filed under Testing), which would have turned the statement into test cases.</t>
+        </is>
+      </c>
+      <c r="I386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Export now publishes the signed statement inside the platform and downloads exactly the signed wording; it never goes to Xray. The box then says 'Exported 10 Oct 2026, 7:23 PM - the file is in your downloads' with 'Export again'. Team-approved mockup, option A. Seen live 10 Oct 19:23, file downloaded.</t>
+        </is>
+      </c>
+      <c r="J386" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" spans="1:10">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">386</t>
+        </is>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Open publish gate' link on the conformance statement</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The link suggested a gate had opened needing action, and took the user to the generic 'Publish to system of record' screen.</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The link pointed at the generic publish screen.</t>
+        </is>
+      </c>
+      <c r="I387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Renamed 'View statement'; it opens the statement's own page in Artifacts. Seen live.</t>
+        </is>
+      </c>
+      <c r="J387" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="388" spans="1:10">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">387</t>
+        </is>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Engine and prompt-version sentence shown under Export</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'The engine, prompt version and scanner version ... are deliberately not shown here.' - not needed by the user.</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An internal explanation was placed on a client screen.</t>
+        </is>
+      </c>
+      <c r="I388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). Removed. The versions are still recorded on the signing record. Seen live.</t>
+        </is>
+      </c>
+      <c r="J388" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" spans="1:10">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">388</t>
+        </is>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Sign panel said signing 'does not publish anything'</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untrue once signing publishes the report and baseline.</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The sentence predates the sign-publishes change.</t>
+        </is>
+      </c>
+      <c r="I389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). 'Signing records your name, your role and the exact wording, and publishes the accessibility report and baseline it rests on. The statement itself is published when you export it.'</t>
+        </is>
+      </c>
+      <c r="J389" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" spans="1:10">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">389</t>
+        </is>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dates printed three different ways on the Accessibility tabs</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Oct 10, 06:26 PM', 'October 10, 2026 at 06:26 PM' and '6:12 PM' for the same audit.</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Audit and Conformance tabs</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-10 in the brownfield accessibility recon and live audit on a fresh workspace (team request).</t>
+        </is>
+      </c>
+      <c r="G390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each screen asked the browser for a different date shape.</t>
+        </is>
+      </c>
+      <c r="I390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-10, branch SDLC_Enhancements_9-30-26, commit c8f0072 (NOT merged to develop - the team dev decides when). One format everywhere: '10 Oct 2026, 6:12 PM'. Seen live on the statement.</t>
+        </is>
+      </c>
+      <c r="J390" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J371" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:J390" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">
       <filters blank="1">
         <filter val="Open"/>

</xml_diff>

<commit_message>
Keep the statement on screen after signing, and say "result" instead of "level"
- Signing no longer hides the Statement and Export boxes until a reload: the reply to Sign now
  says who may sign, like the page load does
- While the first audit runs, the statement says so instead of warning that no audit exists
- The person's pick is a "conformance result" everywhere, so it can't be confused with WCAG's
  Level A / AA
- Bugs.xlsx rows 390-392 and QA cases TC-967 to TC-969
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -5159,7 +5159,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J390"/>
+  <dimension ref="A1:J393"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -20384,8 +20384,164 @@
         </is>
       </c>
     </row>
+    <row r="391" spans="1:10">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">390</t>
+        </is>
+      </c>
+      <c r="B391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After signing, the Statement and Export boxes disappeared until the page was reloaded</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pressing Sign hid both boxes under the criteria table; they came back only after going to another page and returning.</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-12 in the brownfield accessibility re-run on a freshly cleaned workspace (team observation).</t>
+        </is>
+      </c>
+      <c r="G391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="H391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The screen shows both boxes only when the server says this person may sign. The page load includes that answer; the reply to Sign did not, and the screen replaced its data with that reply, so it read the missing answer as 'no' (and could also show 'You are not the accessibility reviewer'). Present since the statement was built; first seen when the team watched the screen right after signing.</t>
+        </is>
+      </c>
+      <c r="I391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-12, branch SDLC_Enhancements_9-30-26 (NOT merged to develop - the team dev decides when). The reply to Sign now carries the same 'may sign' answer as the page load; no screen code changed. Covered by a new automated test; retest live by re-signing.</t>
+        </is>
+      </c>
+      <c r="J391" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" spans="1:10">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">391</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">While the first audit ran, the statement warned 'No completed audit is recorded'</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mid-audit the Statement box showed a yellow warning that nothing rests on a check, while numbers were already coming in.</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-12 in the brownfield accessibility re-run on a freshly cleaned workspace (team observation).</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The warning only asked whether an audit had FINISHED, not whether one was running.</t>
+        </is>
+      </c>
+      <c r="I392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-12, branch SDLC_Enhancements_9-30-26 (NOT merged to develop - the team dev decides when). Team mockup A1: a blue note 'The first audit is still running - This statement will be compiled from it once it finishes. Until then, the numbers above are only what has been checked so far.' The yellow warning stays for a project never audited.</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
+    <row r="393" spans="1:10">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">392</t>
+        </is>
+      </c>
+      <c r="B393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Choose a level' was confused with WCAG Level A / AA</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The third tile ('choose a level for these below'), every row reason ('Choose a level.') and the Sign box ('14 levels were suggested') used 'level' for the person's pick, on a page whose table has a WCAG Level column.</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-12 in the brownfield accessibility re-run on a freshly cleaned workspace (team observation).</t>
+        </is>
+      </c>
+      <c r="G393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One word used for two different things on the same page.</t>
+        </is>
+      </c>
+      <c r="I393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-12, branch SDLC_Enhancements_9-30-26 (NOT merged to develop - the team dev decides when). Team mockup B: tile 'Pick a conformance result for each one in the table below' (or 'Nothing left to decide' at 0); row reasons end 'Pick its result in the Conformance column.'; Sign box '14 results were suggested'. WCAG's own Level A / AA unchanged.</t>
+        </is>
+      </c>
+      <c r="J393" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - automated tests only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J390" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:J393" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">
       <filters blank="1">
         <filter val="Open"/>

</xml_diff>

<commit_message>
Show the time of the latest export, not the first one
- After an edit, re-sign and re-export, the Export box showed the earlier export's time; it now
  shows the latest export of the current signature (Artifacts keeps the first-published date)
- Bugs.xlsx: rows 390 and 392 verified live, new row 393; QA case TC-966 extended
</commit_message>
<xml_diff>
--- a/docs/Bugs.xlsx
+++ b/docs/Bugs.xlsx
@@ -5159,7 +5159,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J393"/>
+  <dimension ref="A1:J394"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.81640625" style="2" bestFit="1" customWidth="1"/>
@@ -20432,7 +20432,7 @@
       </c>
       <c r="J391" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed - automated tests only</t>
+          <t xml:space="preserve">Fixed - verified live 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -20536,12 +20536,64 @@
       </c>
       <c r="J393" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed - automated tests only</t>
+          <t xml:space="preserve">Fixed - verified live 2026-10-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="394" spans="1:10">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">393</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After a re-sign and re-export, the Export box showed the first export's time</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edit, re-sign and export again at 1:37 PM: the box still said 'Exported 12 Oct 2026, 1:00 PM'.</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibility - Conformance statement</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bug</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 2026-10-12 while verifying S.No 390 live (re-sign and re-export).</t>
+        </is>
+      </c>
+      <c r="G394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The box read the document's first-published date, which is deliberately never moved (reports rely on it). Introduced by the 10 Oct Export fix (S.No 385); only visible after a second export.</t>
+        </is>
+      </c>
+      <c r="I394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED 2026-10-12, branch SDLC_Enhancements_9-30-26 (NOT merged to develop - the team dev decides when). The box now shows the latest export of the current signature, read from the activity log; Artifacts keeps the first-published date. Server only, no screen change. Confirmed on the live workspace: it now reports 1:37 PM.</t>
+        </is>
+      </c>
+      <c r="J394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed - verified live 2026-10-12</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J393" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="A1:J394" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="9">
       <filters blank="1">
         <filter val="Open"/>

</xml_diff>